<commit_message>
Fill volume from Stooq + last-known-good so Volume/Avg Vol never blank
</commit_message>
<xml_diff>
--- a/BuddhaVest_Progress.xlsx
+++ b/BuddhaVest_Progress.xlsx
@@ -530,7 +530,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F57"/>
+  <dimension ref="A1:F65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1835,7 +1835,7 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>⏳ ממתין ל-push</t>
+          <t>✅ Live</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
@@ -1845,7 +1845,7 @@
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>נמצא ה-root cause של ה-502/405: מוניטורים חינמיים בודקים עם HEAD ו-FastAPI החזיר 405 Method Not Allowed. אחרי push המוניטור יוריק.</t>
+          <t>נדחף ופרוס. המוניטור החדש ירוק — הסאגה נסגרה.</t>
         </is>
       </c>
     </row>
@@ -1867,7 +1867,7 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>⏳ ממתין לקומיט</t>
+          <t>✅ Live</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
@@ -1877,7 +1877,7 @@
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>נמצא בביקורת: fallback חשוף ב-repo ציבורי. עכשיו env var בלבד (מוגדר ב-Render). לג׳נרט מפתח חדש ב-Tiingo כי הישן בהיסטוריית git.</t>
+          <t>נדחף. בנוסף בוצעה רוטציית מפתח ב-Tiingo והחדש הוגדר ב-Render — הישן חסר ערך. אומת: גרף היסטוריה עובד.</t>
         </is>
       </c>
     </row>
@@ -1899,7 +1899,7 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>⏳ ממתין לקומיט</t>
+          <t>✅ בקומיט</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
@@ -1909,7 +1909,7 @@
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>היה גם ב-dependencies (54.x) וגם ב-devDependencies (13.x) — סיכון build. הוסר הכפול.</t>
+          <t>נדחף. חשף צורך בסנכרון package-lock (פריט 50).</t>
         </is>
       </c>
     </row>
@@ -1931,7 +1931,7 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>⏳ ממתין לקומיט</t>
+          <t>✅ בקומיט</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
@@ -1941,7 +1941,7 @@
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>vixLabel() חדש — very_calm/calm/elevated/fear/volatile, תואם את מדרגות האימוג׳י, בכל 4 השפות.</t>
+          <t>נדחף עם קומיט הביקורת.</t>
         </is>
       </c>
     </row>
@@ -1978,115 +1978,371 @@
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="3" t="inlineStr">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>44</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>התראות אמיתיות — תזוזות במניות המעקב</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Backend + Frontend</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>⏳ ממתין ל-push</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>main.py, BrandHeader.js, api.js, i18n.js</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>endpoint חדש /quotes; מניות מעקב שזזו ≥2% היום מופיעות בפעמון עם נקודה אדומה, ב-4 שפות. סוגר את הבטחת "כאן יופיעו עדכונים".</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>45</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>לוגו מרענן גם במסכי מעקב וחדשות</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Frontend / Bug Fix</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>⏳ ממתין ל-push</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>WatchlistScreen.js, NewsScreen.js</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>ביקורת הבטחות: הטקסט הבטיח רענון מעקב אך הלוגו לא היה מחובר שם.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>46</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>תווית גרסה v1.0.0 (היה v1.2)</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Frontend</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>⏳ ממתין ל-push</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>MoreScreen.js</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>יישור מול version בחנות.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>47</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>תיקוני נוסח: ToS/מי-אני + גילוי תרגום בפרטיות</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Legal / i18n</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>⏳ ממתין ל-push</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>constants/i18n.js</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>"אין לי רישיון" (היה "לא רישוי"); גילוי Google Translate בסעיף הפרטיות ב-4 שפות; אומת שהנוסחה 40/35/25 תואמת את analyzer.py.</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>48</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>מעבר דיקציה מלא — 4 שפות</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>QA / i18n</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>✅ הושלם</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>constants/i18n.js</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>232 מפתחות בכל שפה, אפס זליגות/placeholders שבורים/מחרוזות לא מתורגמות. תוקן ¿? חסר בספרדית.</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>49</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>רוטציית מפתח Tiingo</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>Security</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>✅ הושלם</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>Tiingo + Render env</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>Rotate API Token בוצע; TIINGO_TOKEN עודכן ב-Render; אומת חי.</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>50</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>סנכרון package-lock.json</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Build / Bug Fix</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>⏳ npm install + commit</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>package-lock.json</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>בניית preview נכשלה ב-Install dependencies בגלל lock לא מסונכרן אחרי הסרת הכפילות.</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>51</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>בניית preview APK (אימות אייקון/ספלאש)</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Build</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>⏳ בתהליך</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>EAS</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>אחרי ה-push: eas build --profile preview → התקנה → בדיקת אייקון, ספלאש, התראות.</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="3" t="inlineStr">
         <is>
           <t>🔜  NOT YET STARTED</t>
         </is>
       </c>
-      <c r="B51" s="5" t="inlineStr"/>
-      <c r="C51" s="4" t="inlineStr"/>
-      <c r="D51" s="4" t="inlineStr"/>
-      <c r="E51" s="4" t="inlineStr"/>
-      <c r="F51" s="5" t="inlineStr"/>
-    </row>
-    <row r="52">
-      <c r="A52" s="6" t="inlineStr">
+      <c r="B59" s="5" t="inlineStr"/>
+      <c r="C59" s="4" t="inlineStr"/>
+      <c r="D59" s="4" t="inlineStr"/>
+      <c r="E59" s="4" t="inlineStr"/>
+      <c r="F59" s="5" t="inlineStr"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="6" t="inlineStr">
         <is>
           <t>19</t>
         </is>
       </c>
-      <c r="B52" s="7" t="inlineStr">
+      <c r="B60" s="7" t="inlineStr">
         <is>
           <t>Google Play Console — הגשה לחנות</t>
         </is>
       </c>
-      <c r="C52" s="6" t="inlineStr">
+      <c r="C60" s="6" t="inlineStr">
         <is>
           <t>Distribution</t>
         </is>
       </c>
-      <c r="D52" s="8" t="inlineStr">
+      <c r="D60" s="8" t="inlineStr">
         <is>
           <t>🔜</t>
         </is>
       </c>
-      <c r="E52" s="9" t="inlineStr"/>
-      <c r="F52" s="9" t="inlineStr">
+      <c r="E60" s="9" t="inlineStr"/>
+      <c r="F60" s="9" t="inlineStr">
         <is>
           <t>חשבון מפתח ($25) + העלאת AAB + store listing + screenshots.</t>
         </is>
       </c>
     </row>
-    <row r="53">
-      <c r="A53" s="10" t="inlineStr">
+    <row r="61">
+      <c r="A61" s="10" t="inlineStr">
         <is>
           <t>Legend</t>
         </is>
       </c>
     </row>
-    <row r="54">
-      <c r="A54" s="6" t="inlineStr">
+    <row r="62">
+      <c r="A62" s="6" t="inlineStr">
         <is>
           <t>✅ Live</t>
         </is>
       </c>
-      <c r="B54" s="7" t="inlineStr">
+      <c r="B62" s="7" t="inlineStr">
         <is>
           <t>פרוס ופעיל ב-Render — נראה לכל המשתמשים</t>
         </is>
       </c>
-      <c r="C54" s="6" t="inlineStr"/>
-      <c r="D54" s="8" t="inlineStr"/>
-      <c r="E54" s="9" t="inlineStr"/>
-      <c r="F54" s="9" t="inlineStr"/>
-    </row>
-    <row r="55">
-      <c r="A55" s="6" t="inlineStr">
+      <c r="C62" s="6" t="inlineStr"/>
+      <c r="D62" s="8" t="inlineStr"/>
+      <c r="E62" s="9" t="inlineStr"/>
+      <c r="F62" s="9" t="inlineStr"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="6" t="inlineStr">
         <is>
           <t>✅ In APK</t>
         </is>
       </c>
-      <c r="B55" s="7" t="inlineStr">
+      <c r="B63" s="7" t="inlineStr">
         <is>
           <t>כלול ב-APK המותקן — נראה לכל המשתמשים</t>
         </is>
       </c>
-      <c r="C55" s="6" t="inlineStr"/>
-      <c r="D55" s="8" t="inlineStr"/>
-      <c r="E55" s="9" t="inlineStr"/>
-      <c r="F55" s="9" t="inlineStr"/>
-    </row>
-    <row r="56">
-      <c r="A56" s="6" t="inlineStr">
+      <c r="C63" s="6" t="inlineStr"/>
+      <c r="D63" s="8" t="inlineStr"/>
+      <c r="E63" s="9" t="inlineStr"/>
+      <c r="F63" s="9" t="inlineStr"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="6" t="inlineStr">
         <is>
           <t>⏳ Next APK</t>
         </is>
       </c>
-      <c r="B56" s="7" t="inlineStr">
+      <c r="B64" s="7" t="inlineStr">
         <is>
           <t>הקוד מוזג — דורש build ו-APK חדש</t>
         </is>
       </c>
-      <c r="C56" s="6" t="inlineStr"/>
-      <c r="D56" s="8" t="inlineStr"/>
-      <c r="E56" s="9" t="inlineStr"/>
-      <c r="F56" s="9" t="inlineStr"/>
-    </row>
-    <row r="57">
-      <c r="A57" s="6" t="inlineStr">
+      <c r="C64" s="6" t="inlineStr"/>
+      <c r="D64" s="8" t="inlineStr"/>
+      <c r="E64" s="9" t="inlineStr"/>
+      <c r="F64" s="9" t="inlineStr"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="6" t="inlineStr">
         <is>
           <t>✅ Live (OTA)</t>
         </is>
       </c>
-      <c r="B57" s="7" t="inlineStr">
+      <c r="B65" s="7" t="inlineStr">
         <is>
           <t>שינוי JS — מועבר אוטומטית בהפעלה הבאה</t>
         </is>
       </c>
-      <c r="C57" s="6" t="inlineStr"/>
-      <c r="D57" s="8" t="inlineStr"/>
-      <c r="E57" s="9" t="inlineStr"/>
-      <c r="F57" s="9" t="inlineStr"/>
+      <c r="C65" s="6" t="inlineStr"/>
+      <c r="D65" s="8" t="inlineStr"/>
+      <c r="E65" s="9" t="inlineStr"/>
+      <c r="F65" s="9" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
Chart colour matches metric direction (rising P/B is now red, like its tile); server: no-store, year-end annual series, buyback TTM 4Q
</commit_message>
<xml_diff>
--- a/BuddhaVest_Progress.xlsx
+++ b/BuddhaVest_Progress.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="6">
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -52,8 +52,17 @@
       <b val="1"/>
       <color rgb="00FFFFFF"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="7">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -83,6 +92,16 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="001a7340"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001A7340"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
   </fills>
@@ -136,7 +155,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -165,6 +184,42 @@
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -530,7 +585,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F65"/>
+  <dimension ref="A1:F113"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -551,7 +606,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Last updated: 2026-07-12  |  Session 5</t>
+          <t>Last updated: 2026-07-25  |  Session 6</t>
         </is>
       </c>
     </row>
@@ -2234,118 +2289,1390 @@
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="3" t="inlineStr">
+      <c r="A59" s="12" t="inlineStr">
+        <is>
+          <t>✅  Session 6 (2026-07-24/25): מרוצים, אבטחה, ביצועים, משפטי — ביקורת מלאה</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="13" t="inlineStr">
+        <is>
+          <t>52</t>
+        </is>
+      </c>
+      <c r="B60" s="14" t="inlineStr">
+        <is>
+          <t>מרוץ שפות — 5 מסכים/רכיבים</t>
+        </is>
+      </c>
+      <c r="C60" s="13" t="inlineStr">
+        <is>
+          <t>Frontend / Bug Fix</t>
+        </is>
+      </c>
+      <c r="D60" s="15" t="inlineStr">
+        <is>
+          <t>✅ Live (OTA)</t>
+        </is>
+      </c>
+      <c r="E60" s="16" t="inlineStr">
+        <is>
+          <t>NewsScreen, NewsCard, WatchlistScreen, HomeScreen, StockScreen</t>
+        </is>
+      </c>
+      <c r="F60" s="16" t="inlineStr">
+        <is>
+          <t>טוקן reqId מונוטוני בכל טעינה. תגובה איטית בשפה ישנה כבר לא דורסת את החדשה — הטקסט הפסיק לקפוץ.</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="13" t="inlineStr">
+        <is>
+          <t>53</t>
+        </is>
+      </c>
+      <c r="B61" s="14" t="inlineStr">
+        <is>
+          <t>Volume/Avg Vol ריקים לסירוגין</t>
+        </is>
+      </c>
+      <c r="C61" s="13" t="inlineStr">
+        <is>
+          <t>Backend / Bug Fix</t>
+        </is>
+      </c>
+      <c r="D61" s="15" t="inlineStr">
+        <is>
+          <t>✅ Live</t>
+        </is>
+      </c>
+      <c r="E61" s="16" t="inlineStr">
+        <is>
+          <t>main.py</t>
+        </is>
+      </c>
+      <c r="F61" s="16" t="inlineStr">
+        <is>
+          <t>Last-known-good לכל טיקר + שמירה לדיסק (/tmp) כדי לשרוד restart של Render. גם trigger ל-Stooq כשחסר נפח ולא רק מחיר.</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="13" t="inlineStr">
+        <is>
+          <t>54</t>
+        </is>
+      </c>
+      <c r="B62" s="14" t="inlineStr">
+        <is>
+          <t>המרת אגורות→שקל למניות ת"א</t>
+        </is>
+      </c>
+      <c r="C62" s="13" t="inlineStr">
+        <is>
+          <t>Backend</t>
+        </is>
+      </c>
+      <c r="D62" s="15" t="inlineStr">
+        <is>
+          <t>✅ Live</t>
+        </is>
+      </c>
+      <c r="E62" s="16" t="inlineStr">
+        <is>
+          <t>main.py</t>
+        </is>
+      </c>
+      <c r="F62" s="16" t="inlineStr">
+        <is>
+          <t>דלק הציגה 8173 במקום 81.73. זיהוי לפי סיומת .TA וגם שדה currency (ILA/ILS). הומר: מחיר, טווח 52 שבועות, היסטוריה, אירועי דיבידנד.</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="13" t="inlineStr">
+        <is>
+          <t>55</t>
+        </is>
+      </c>
+      <c r="B63" s="14" t="inlineStr">
+        <is>
+          <t>באג יחידות ב-Buyback (3500000000%)</t>
+        </is>
+      </c>
+      <c r="C63" s="13" t="inlineStr">
+        <is>
+          <t>Backend + Frontend</t>
+        </is>
+      </c>
+      <c r="D63" s="15" t="inlineStr">
+        <is>
+          <t>✅ Live</t>
+        </is>
+      </c>
+      <c r="E63" s="16" t="inlineStr">
+        <is>
+          <t>analyzer.py, StockScreen.js</t>
+        </is>
+      </c>
+      <c r="F63" s="16" t="inlineStr">
+        <is>
+          <t>value_unit='percent'/'currency'. בלי שווי שוק הערך הוא סכום גולמי — הוצג עם % ויצר מספר אבסורדי.</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="13" t="inlineStr">
+        <is>
+          <t>56</t>
+        </is>
+      </c>
+      <c r="B64" s="14" t="inlineStr">
+        <is>
+          <t>תיקוני נכונות במנוע הציון</t>
+        </is>
+      </c>
+      <c r="C64" s="13" t="inlineStr">
+        <is>
+          <t>Backend / Scoring</t>
+        </is>
+      </c>
+      <c r="D64" s="15" t="inlineStr">
+        <is>
+          <t>✅ Live</t>
+        </is>
+      </c>
+      <c r="E64" s="16" t="inlineStr">
+        <is>
+          <t>analyzer.py</t>
+        </is>
+      </c>
+      <c r="F64" s="16" t="inlineStr">
+        <is>
+          <t>FCF עמיד לסימן (ocf-abs(capex)); מיון סדרות לפני iloc[0]/iloc[1] כדי שמגמת רווח לא תתהפך; מיון דיבידנדים לפני index[-1]/tail(4).</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="13" t="inlineStr">
+        <is>
+          <t>57</t>
+        </is>
+      </c>
+      <c r="B65" s="14" t="inlineStr">
+        <is>
+          <t>ניסוח דיבידנד כן — לא "משולם בעקביות"</t>
+        </is>
+      </c>
+      <c r="C65" s="13" t="inlineStr">
+        <is>
+          <t>Legal / Accuracy</t>
+        </is>
+      </c>
+      <c r="D65" s="15" t="inlineStr">
+        <is>
+          <t>✅ Live</t>
+        </is>
+      </c>
+      <c r="E65" s="16" t="inlineStr">
+        <is>
+          <t>analyzer.py, i18n_data.py</t>
+        </is>
+      </c>
+      <c r="F65" s="16" t="inlineStr">
+        <is>
+          <t>הנתון מודד טווח היסטוריה, לא רציפות תשלומים. חברה שהפסיקה וחידשה היתה מקבלת אותו מספר.</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="13" t="inlineStr">
+        <is>
+          <t>58</t>
+        </is>
+      </c>
+      <c r="B66" s="14" t="inlineStr">
+        <is>
+          <t>SSRF — /translate-article</t>
+        </is>
+      </c>
+      <c r="C66" s="13" t="inlineStr">
+        <is>
+          <t>Backend / Security</t>
+        </is>
+      </c>
+      <c r="D66" s="15" t="inlineStr">
+        <is>
+          <t>✅ Live</t>
+        </is>
+      </c>
+      <c r="E66" s="16" t="inlineStr">
+        <is>
+          <t>main.py</t>
+        </is>
+      </c>
+      <c r="F66" s="16" t="inlineStr">
+        <is>
+          <t>חסימת loopback/פרטי/link-local/metadata (169.254.169.254), כולל בדיקה שנייה על canonical URL שמגיע מהדף עצמו.</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="13" t="inlineStr">
+        <is>
+          <t>59</t>
+        </is>
+      </c>
+      <c r="B67" s="14" t="inlineStr">
+        <is>
+          <t>XSS ב-WebView של הכתבות</t>
+        </is>
+      </c>
+      <c r="C67" s="13" t="inlineStr">
+        <is>
+          <t>Frontend / Security</t>
+        </is>
+      </c>
+      <c r="D67" s="15" t="inlineStr">
+        <is>
+          <t>✅ Live (OTA)</t>
+        </is>
+      </c>
+      <c r="E67" s="16" t="inlineStr">
+        <is>
+          <t>ArticleScreen.js</t>
+        </is>
+      </c>
+      <c r="F67" s="16" t="inlineStr">
+        <is>
+          <t>שמות תגיות מהדף עברו ל-whitelist (p/h2/h3) וטקסט עובר escape — דף עוין יכול היה לשלוח tag:"script".</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="13" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="B68" s="14" t="inlineStr">
+        <is>
+          <t>הסרת /debug-pe ו-/debug-rows</t>
+        </is>
+      </c>
+      <c r="C68" s="13" t="inlineStr">
+        <is>
+          <t>Backend / Security</t>
+        </is>
+      </c>
+      <c r="D68" s="15" t="inlineStr">
+        <is>
+          <t>✅ Live</t>
+        </is>
+      </c>
+      <c r="E68" s="16" t="inlineStr">
+        <is>
+          <t>main.py</t>
+        </is>
+      </c>
+      <c r="F68" s="16" t="inlineStr">
+        <is>
+          <t>ראוטים ציבוריים שהחזירו traceback מלא, לא ולידציה על טיקר, ובלי מטמון — דרך לרוקן זיכרון לשרת.</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="13" t="inlineStr">
+        <is>
+          <t>61</t>
+        </is>
+      </c>
+      <c r="B69" s="14" t="inlineStr">
+        <is>
+          <t>5 דליפות של פרטי חריגה ללקוח</t>
+        </is>
+      </c>
+      <c r="C69" s="13" t="inlineStr">
+        <is>
+          <t>Backend / Security</t>
+        </is>
+      </c>
+      <c r="D69" s="15" t="inlineStr">
+        <is>
+          <t>✅ Live</t>
+        </is>
+      </c>
+      <c r="E69" s="16" t="inlineStr">
+        <is>
+          <t>main.py</t>
+        </is>
+      </c>
+      <c r="F69" s="16" t="inlineStr">
+        <is>
+          <t>str(e) הוחלף בהודעה גנרית + לוג פנימי.</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="13" t="inlineStr">
+        <is>
+          <t>62</t>
+        </is>
+      </c>
+      <c r="B70" s="14" t="inlineStr">
+        <is>
+          <t>פיצוץ זיכרון בעליית השרת</t>
+        </is>
+      </c>
+      <c r="C70" s="13" t="inlineStr">
+        <is>
+          <t>Backend / Performance</t>
+        </is>
+      </c>
+      <c r="D70" s="15" t="inlineStr">
+        <is>
+          <t>✅ Live</t>
+        </is>
+      </c>
+      <c r="E70" s="16" t="inlineStr">
+        <is>
+          <t>main.py</t>
+        </is>
+      </c>
+      <c r="F70" s="16" t="inlineStr">
+        <is>
+          <t>_BOOTING מדכא תרגום מקדים בזמן החימום; השפות מרווחות (15s ואז 10s). 18 הורדות כבדות בדקה הראשונה → 0.</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="13" t="inlineStr">
+        <is>
+          <t>63</t>
+        </is>
+      </c>
+      <c r="B71" s="14" t="inlineStr">
+        <is>
+          <t>תקרת מטמון + single-flight</t>
+        </is>
+      </c>
+      <c r="C71" s="13" t="inlineStr">
+        <is>
+          <t>Backend / Performance</t>
+        </is>
+      </c>
+      <c r="D71" s="15" t="inlineStr">
+        <is>
+          <t>✅ Live</t>
+        </is>
+      </c>
+      <c r="E71" s="16" t="inlineStr">
+        <is>
+          <t>main.py</t>
+        </is>
+      </c>
+      <c r="F71" s="16" t="inlineStr">
+        <is>
+          <t>_CACHE_MAX=300 ונעילה לכל מפתח — N משתמשים על אותו טיקר = שליפה אחת מיאהו במקום N.</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="13" t="inlineStr">
+        <is>
+          <t>64</t>
+        </is>
+      </c>
+      <c r="B72" s="14" t="inlineStr">
+        <is>
+          <t>חלון היסטוריה 10y במקום max</t>
+        </is>
+      </c>
+      <c r="C72" s="13" t="inlineStr">
+        <is>
+          <t>Backend / Performance</t>
+        </is>
+      </c>
+      <c r="D72" s="15" t="inlineStr">
+        <is>
+          <t>✅ Live</t>
+        </is>
+      </c>
+      <c r="E72" s="16" t="inlineStr">
+        <is>
+          <t>main.py</t>
+        </is>
+      </c>
+      <c r="F72" s="16" t="inlineStr">
+        <is>
+          <t>KO נסחרת מ-1962: 16,000 שורות יומיות לתוך pandas כדי להפיק 44 נקודות. ~84% פחות נתונים.</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="13" t="inlineStr">
+        <is>
+          <t>65</t>
+        </is>
+      </c>
+      <c r="B73" s="14" t="inlineStr">
+        <is>
+          <t>Debounce בחיפוש</t>
+        </is>
+      </c>
+      <c r="C73" s="13" t="inlineStr">
+        <is>
+          <t>Frontend / Performance</t>
+        </is>
+      </c>
+      <c r="D73" s="15" t="inlineStr">
+        <is>
+          <t>✅ Live (OTA)</t>
+        </is>
+      </c>
+      <c r="E73" s="16" t="inlineStr">
+        <is>
+          <t>SearchScreen.js</t>
+        </is>
+      </c>
+      <c r="F73" s="16" t="inlineStr">
+        <is>
+          <t>הקלדת AAPL שלחה 4 בקשות; עכשיו אחת אחרי 300ms שקט.</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="13" t="inlineStr">
+        <is>
+          <t>66</t>
+        </is>
+      </c>
+      <c r="B74" s="14" t="inlineStr">
+        <is>
+          <t>תקציב זמן ל-Stooq</t>
+        </is>
+      </c>
+      <c r="C74" s="13" t="inlineStr">
+        <is>
+          <t>Backend / Performance</t>
+        </is>
+      </c>
+      <c r="D74" s="15" t="inlineStr">
+        <is>
+          <t>✅ Live</t>
+        </is>
+      </c>
+      <c r="E74" s="16" t="inlineStr">
+        <is>
+          <t>stooq_fallback.py</t>
+        </is>
+      </c>
+      <c r="F74" s="16" t="inlineStr">
+        <is>
+          <t>8 סיומות × 4s = 32s לסימול שלא קיים, הרבה אחרי שהאפליקציה ויתרה. עכשיו תקרה של 10s; סימול עם סיומת לא מנסה עוד.</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="13" t="inlineStr">
+        <is>
+          <t>67</t>
+        </is>
+      </c>
+      <c r="B75" s="14" t="inlineStr">
+        <is>
+          <t>אובדן נתונים ביומן המחקר</t>
+        </is>
+      </c>
+      <c r="C75" s="13" t="inlineStr">
+        <is>
+          <t>Frontend / Bug Fix</t>
+        </is>
+      </c>
+      <c r="D75" s="15" t="inlineStr">
+        <is>
+          <t>✅ Live (OTA)</t>
+        </is>
+      </c>
+      <c r="E75" s="16" t="inlineStr">
+        <is>
+          <t>MoreScreen.js</t>
+        </is>
+      </c>
+      <c r="F75" s="16" t="inlineStr">
+        <is>
+          <t>שמירה מוזגה מול הדיסק ולא מול state; מחיקה לפי זהות (תאריך+טקסט) ולא לפי אינדקס.</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="17" t="inlineStr">
+        <is>
+          <t>68</t>
+        </is>
+      </c>
+      <c r="B76" s="18" t="inlineStr">
+        <is>
+          <t>תמיכת טאבלט</t>
+        </is>
+      </c>
+      <c r="C76" s="17" t="inlineStr">
+        <is>
+          <t>Frontend</t>
+        </is>
+      </c>
+      <c r="D76" s="19" t="inlineStr">
+        <is>
+          <t>⏳ דורש build</t>
+        </is>
+      </c>
+      <c r="E76" s="20" t="inlineStr">
+        <is>
+          <t>App.js, app.json, PriceChart.js, FloatingThemeToggle.js</t>
+        </is>
+      </c>
+      <c r="F76" s="20" t="inlineStr">
+        <is>
+          <t>TabletFrame (רוחב ≥700 ממורכז ל-600), שחרור סיבוב לטאבלט ונעילת portrait לטלפון, כפתור צף שנצמד מחדש בסיבוב. supportsTablet=true.</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="13" t="inlineStr">
+        <is>
+          <t>69</t>
+        </is>
+      </c>
+      <c r="B77" s="14" t="inlineStr">
+        <is>
+          <t>מסך הסכמה בהפעלה ראשונה</t>
+        </is>
+      </c>
+      <c r="C77" s="13" t="inlineStr">
+        <is>
+          <t>Legal</t>
+        </is>
+      </c>
+      <c r="D77" s="15" t="inlineStr">
+        <is>
+          <t>✅ Live (OTA)</t>
+        </is>
+      </c>
+      <c r="E77" s="16" t="inlineStr">
+        <is>
+          <t>App.js, i18n.js</t>
+        </is>
+      </c>
+      <c r="F77" s="16" t="inlineStr">
+        <is>
+          <t>"כלי מחקר, לא ייעוץ" — הסכמה מפורשת חזקה משתיקה. 4 שפות, מוצג פעם אחת.</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="13" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
+      <c r="B78" s="14" t="inlineStr">
+        <is>
+          <t>שכתוב תיאור החנות — בלי הבטחות</t>
+        </is>
+      </c>
+      <c r="C78" s="13" t="inlineStr">
+        <is>
+          <t>Legal / Store</t>
+        </is>
+      </c>
+      <c r="D78" s="15" t="inlineStr">
+        <is>
+          <t>✅ מוכן</t>
+        </is>
+      </c>
+      <c r="E78" s="16" t="inlineStr">
+        <is>
+          <t>store-listing.md</t>
+        </is>
+      </c>
+      <c r="F78" s="16" t="inlineStr">
+        <is>
+          <t>הוסרו טענות "יועץ AI"; הודגש שהציון הוא חישוב מתמטי. AI לא מודגש בניסוח.</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="13" t="inlineStr">
+        <is>
+          <t>71</t>
+        </is>
+      </c>
+      <c r="B79" s="14" t="inlineStr">
+        <is>
+          <t>מדריך צילומי מסך לחנות</t>
+        </is>
+      </c>
+      <c r="C79" s="13" t="inlineStr">
+        <is>
+          <t>Store Assets</t>
+        </is>
+      </c>
+      <c r="D79" s="15" t="inlineStr">
+        <is>
+          <t>✅ הושלם</t>
+        </is>
+      </c>
+      <c r="E79" s="16" t="inlineStr">
+        <is>
+          <t>מדריך-צילומי-מסך-לחנות.docx</t>
+        </is>
+      </c>
+      <c r="F79" s="16" t="inlineStr">
+        <is>
+          <t>5 מסכים, מידות, והנחיות צילום.</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="13" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="B80" s="14" t="inlineStr">
+        <is>
+          <t>RTL בכל המסכים</t>
+        </is>
+      </c>
+      <c r="C80" s="13" t="inlineStr">
+        <is>
+          <t>Frontend / i18n</t>
+        </is>
+      </c>
+      <c r="D80" s="15" t="inlineStr">
+        <is>
+          <t>✅ Live (OTA)</t>
+        </is>
+      </c>
+      <c r="E80" s="16" t="inlineStr">
+        <is>
+          <t>8 מסכים/רכיבים</t>
+        </is>
+      </c>
+      <c r="F80" s="16" t="inlineStr">
+        <is>
+          <t>כל משפט מתורגם ארוך קיבל textAlign+writingDirection. עברית היחידה RTL מבין ה-4.</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="13" t="inlineStr">
+        <is>
+          <t>73</t>
+        </is>
+      </c>
+      <c r="B81" s="14" t="inlineStr">
+        <is>
+          <t>תווית גרסה מ-app.json</t>
+        </is>
+      </c>
+      <c r="C81" s="13" t="inlineStr">
+        <is>
+          <t>Frontend</t>
+        </is>
+      </c>
+      <c r="D81" s="15" t="inlineStr">
+        <is>
+          <t>✅ Live (OTA)</t>
+        </is>
+      </c>
+      <c r="E81" s="16" t="inlineStr">
+        <is>
+          <t>MoreScreen.js</t>
+        </is>
+      </c>
+      <c r="F81" s="16" t="inlineStr">
+        <is>
+          <t>היה מחרוזת קשיחה — bump גרסה היה משאיר את המסך על 1.0.0.</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="13" t="inlineStr">
+        <is>
+          <t>74</t>
+        </is>
+      </c>
+      <c r="B82" s="14" t="inlineStr">
+        <is>
+          <t>טעינה דו-שלבית ברשימת המעקב</t>
+        </is>
+      </c>
+      <c r="C82" s="13" t="inlineStr">
+        <is>
+          <t>Frontend / Performance</t>
+        </is>
+      </c>
+      <c r="D82" s="15" t="inlineStr">
+        <is>
+          <t>✅ Live (OTA)</t>
+        </is>
+      </c>
+      <c r="E82" s="16" t="inlineStr">
+        <is>
+          <t>WatchlistScreen.js, main.py</t>
+        </is>
+      </c>
+      <c r="F82" s="16" t="inlineStr">
+        <is>
+          <t>/quotes קל לכל הרשימה תחילה, ואז /analyze בקבוצות עם ציור מצטבר. זמן עד תוכן ראשון: 4000ms → 400ms (פי 10). שער חליפין במקביל.</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="13" t="inlineStr">
+        <is>
+          <t>75</t>
+        </is>
+      </c>
+      <c r="B83" s="14" t="inlineStr">
+        <is>
+          <t>/quotes: אגורות, שם חברה, מטבע</t>
+        </is>
+      </c>
+      <c r="C83" s="13" t="inlineStr">
+        <is>
+          <t>Backend</t>
+        </is>
+      </c>
+      <c r="D83" s="15" t="inlineStr">
+        <is>
+          <t>✅ Live</t>
+        </is>
+      </c>
+      <c r="E83" s="16" t="inlineStr">
+        <is>
+          <t>main.py</t>
+        </is>
+      </c>
+      <c r="F83" s="16" t="inlineStr">
+        <is>
+          <t>הפאזה המהירה היתה מהבהבת 8445 לפני התיקון. longName כדי שהשם לא יתחלף שנייה אחרי.</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="13" t="inlineStr">
+        <is>
+          <t>76</t>
+        </is>
+      </c>
+      <c r="B84" s="14" t="inlineStr">
+        <is>
+          <t>מיזוג במקום החלפה ברשימת המעקב</t>
+        </is>
+      </c>
+      <c r="C84" s="13" t="inlineStr">
+        <is>
+          <t>Frontend / Bug Fix</t>
+        </is>
+      </c>
+      <c r="D84" s="15" t="inlineStr">
+        <is>
+          <t>✅ Live (OTA)</t>
+        </is>
+      </c>
+      <c r="E84" s="16" t="inlineStr">
+        <is>
+          <t>WatchlistScreen.js</t>
+        </is>
+      </c>
+      <c r="F84" s="16" t="inlineStr">
+        <is>
+          <t>פאזה 1 מחקה את כל הציונים בכל רענון אוטומטי (כל 90 שניות) — הבהוב בכל מחזור.</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="13" t="inlineStr">
+        <is>
+          <t>77</t>
+        </is>
+      </c>
+      <c r="B85" s="14" t="inlineStr">
+        <is>
+          <t>מרוץ במסך הבית — market/FX</t>
+        </is>
+      </c>
+      <c r="C85" s="13" t="inlineStr">
+        <is>
+          <t>Frontend / Bug Fix</t>
+        </is>
+      </c>
+      <c r="D85" s="15" t="inlineStr">
+        <is>
+          <t>✅ Live (OTA)</t>
+        </is>
+      </c>
+      <c r="E85" s="16" t="inlineStr">
+        <is>
+          <t>HomeScreen.js</t>
+        </is>
+      </c>
+      <c r="F85" s="16" t="inlineStr">
+        <is>
+          <t>שרת קר: קריאה שנכשלה ב-20s ומנסה שוב ב-50s חוזרת אחרונה ודורסת נתונים טריים. מונים נפרדים ל-market ול-FX.</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="13" t="inlineStr">
+        <is>
+          <t>78</t>
+        </is>
+      </c>
+      <c r="B86" s="14" t="inlineStr">
+        <is>
+          <t>תשובה ריקה לא מוחקת נתונים טובים</t>
+        </is>
+      </c>
+      <c r="C86" s="13" t="inlineStr">
+        <is>
+          <t>Frontend / Bug Fix</t>
+        </is>
+      </c>
+      <c r="D86" s="15" t="inlineStr">
+        <is>
+          <t>✅ Live (OTA)</t>
+        </is>
+      </c>
+      <c r="E86" s="16" t="inlineStr">
+        <is>
+          <t>HomeScreen.js</t>
+        </is>
+      </c>
+      <c r="F86" s="16" t="inlineStr">
+        <is>
+          <t>הסיבה ל"פעם יש נתונים פעם אין" בטבלת המניות.</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="13" t="inlineStr">
+        <is>
+          <t>79</t>
+        </is>
+      </c>
+      <c r="B87" s="14" t="inlineStr">
+        <is>
+          <t>תרגום כתבה ישנה דלף לחדשה</t>
+        </is>
+      </c>
+      <c r="C87" s="13" t="inlineStr">
+        <is>
+          <t>Frontend / Bug Fix</t>
+        </is>
+      </c>
+      <c r="D87" s="15" t="inlineStr">
+        <is>
+          <t>✅ Live (OTA)</t>
+        </is>
+      </c>
+      <c r="E87" s="16" t="inlineStr">
+        <is>
+          <t>ArticleScreen.js</t>
+        </is>
+      </c>
+      <c r="F87" s="16" t="inlineStr">
+        <is>
+          <t>נתיב ה-DOM לא בוטל אף פעם; מעבר לכתבה אחרת הציג את הטקסט הקודם. גם ספינר תקוע בתשובה קצרה.</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="13" t="inlineStr">
+        <is>
+          <t>80</t>
+        </is>
+      </c>
+      <c r="B88" s="14" t="inlineStr">
+        <is>
+          <t>מרוץ ב"נסה שוב" של פירוט מדד</t>
+        </is>
+      </c>
+      <c r="C88" s="13" t="inlineStr">
+        <is>
+          <t>Frontend / Bug Fix</t>
+        </is>
+      </c>
+      <c r="D88" s="15" t="inlineStr">
+        <is>
+          <t>✅ Live (OTA)</t>
+        </is>
+      </c>
+      <c r="E88" s="16" t="inlineStr">
+        <is>
+          <t>MetricHistoryScreen.js</t>
+        </is>
+      </c>
+      <c r="F88" s="16" t="inlineStr">
+        <is>
+          <t>לחיצה כפולה: הכישלון האיטי חוזר אחרי ההצלחה ומחליף גרף תקין במסך שגיאה.</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="13" t="inlineStr">
+        <is>
+          <t>81</t>
+        </is>
+      </c>
+      <c r="B89" s="14" t="inlineStr">
+        <is>
+          <t>סולם VIX לא מונוטוני</t>
+        </is>
+      </c>
+      <c r="C89" s="13" t="inlineStr">
+        <is>
+          <t>Frontend / i18n</t>
+        </is>
+      </c>
+      <c r="D89" s="15" t="inlineStr">
+        <is>
+          <t>✅ Live (OTA)</t>
+        </is>
+      </c>
+      <c r="E89" s="16" t="inlineStr">
+        <is>
+          <t>i18n.js</t>
+        </is>
+      </c>
+      <c r="F89" s="16" t="inlineStr">
+        <is>
+          <t>VIX 27 = "פחד קיצוני" אבל VIX 45 = "תנודתיות גבוהה" — אזהרה רכה יותר במצב חמור יותר. תוקן ב-4 שפות.</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="13" t="inlineStr">
+        <is>
+          <t>82</t>
+        </is>
+      </c>
+      <c r="B90" s="14" t="inlineStr">
+        <is>
+          <t>תיקוני תוכן בספרדית</t>
+        </is>
+      </c>
+      <c r="C90" s="13" t="inlineStr">
+        <is>
+          <t>i18n / Accuracy</t>
+        </is>
+      </c>
+      <c r="D90" s="15" t="inlineStr">
+        <is>
+          <t>✅ Live (OTA)</t>
+        </is>
+      </c>
+      <c r="E90" s="16" t="inlineStr">
+        <is>
+          <t>i18n.js</t>
+        </is>
+      </c>
+      <c r="F90" s="16" t="inlineStr">
+        <is>
+          <t>הסבר הדיבידנד השמיט את חצי המשפט על יציבות; טקסט הצהיר "servidor local" בעוד השרת ב-Render.</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="17" t="inlineStr">
+        <is>
+          <t>83</t>
+        </is>
+      </c>
+      <c r="B91" s="18" t="inlineStr">
+        <is>
+          <t>Cache-Control: no-store על כל ה-API</t>
+        </is>
+      </c>
+      <c r="C91" s="17" t="inlineStr">
+        <is>
+          <t>Backend / Bug Fix</t>
+        </is>
+      </c>
+      <c r="D91" s="19" t="inlineStr">
+        <is>
+          <t>⏳ ממתין ל-push</t>
+        </is>
+      </c>
+      <c r="E91" s="20" t="inlineStr">
+        <is>
+          <t>main.py</t>
+        </is>
+      </c>
+      <c r="F91" s="20" t="inlineStr">
+        <is>
+          <t>הסיבה האמיתית שדלק חזרה: OkHttp של אנדרואיד שמר תשובה שנוצרה בגרסת קוד ישנה. הוכח — אותה מניה ב-en החזירה 8173 וב-ru החזירה 84.45.</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="17" t="inlineStr">
+        <is>
+          <t>84</t>
+        </is>
+      </c>
+      <c r="B92" s="18" t="inlineStr">
+        <is>
+          <t>סדרה שנתית = סוף שנה, לא ינואר</t>
+        </is>
+      </c>
+      <c r="C92" s="17" t="inlineStr">
+        <is>
+          <t>Backend / Bug Fix</t>
+        </is>
+      </c>
+      <c r="D92" s="19" t="inlineStr">
+        <is>
+          <t>⏳ ממתין ל-push</t>
+        </is>
+      </c>
+      <c r="E92" s="20" t="inlineStr">
+        <is>
+          <t>main.py</t>
+        </is>
+      </c>
+      <c r="F92" s="20" t="inlineStr">
+        <is>
+          <t>הגרף השנתי הציג את ינואר בתווית של השנה. KO 2023: הוצג 25.25 במקום 22.19 — סטייה 12%. תוקן ב-4 מקומות.</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="17" t="inlineStr">
+        <is>
+          <t>85</t>
+        </is>
+      </c>
+      <c r="B93" s="18" t="inlineStr">
+        <is>
+          <t>TTM של Buyback דרש 2 רבעונים</t>
+        </is>
+      </c>
+      <c r="C93" s="17" t="inlineStr">
+        <is>
+          <t>Backend / Bug Fix</t>
+        </is>
+      </c>
+      <c r="D93" s="19" t="inlineStr">
+        <is>
+          <t>⏳ ממתין ל-push</t>
+        </is>
+      </c>
+      <c r="E93" s="20" t="inlineStr">
+        <is>
+          <t>main.py</t>
+        </is>
+      </c>
+      <c r="F93" s="20" t="inlineStr">
+        <is>
+          <t>"תשואה שנתית" יכלה להיות סכום של חצי שנה. הועלה ל-4 כמו כל שאר חישובי ה-TTM.</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="13" t="inlineStr">
+        <is>
+          <t>86</t>
+        </is>
+      </c>
+      <c r="B94" s="14" t="inlineStr">
+        <is>
+          <t>ניקוי ריפו — cloudflared.exe 52MB</t>
+        </is>
+      </c>
+      <c r="C94" s="13" t="inlineStr">
+        <is>
+          <t>DevOps</t>
+        </is>
+      </c>
+      <c r="D94" s="15" t="inlineStr">
+        <is>
+          <t>✅ Live</t>
+        </is>
+      </c>
+      <c r="E94" s="16" t="inlineStr">
+        <is>
+          <t>‎.gitignore</t>
+        </is>
+      </c>
+      <c r="F94" s="16" t="inlineStr">
+        <is>
+          <t>יצא ממעקב git, נשאר על הדיסק המקומי.</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="13" t="inlineStr">
+        <is>
+          <t>87</t>
+        </is>
+      </c>
+      <c r="B95" s="14" t="inlineStr">
+        <is>
+          <t>דיוק עמוד הפרטיות בנוגע ללוגים</t>
+        </is>
+      </c>
+      <c r="C95" s="13" t="inlineStr">
+        <is>
+          <t>Legal</t>
+        </is>
+      </c>
+      <c r="D95" s="15" t="inlineStr">
+        <is>
+          <t>✅ Live</t>
+        </is>
+      </c>
+      <c r="E95" s="16" t="inlineStr">
+        <is>
+          <t>main.py</t>
+        </is>
+      </c>
+      <c r="F95" s="16" t="inlineStr">
+        <is>
+          <t>ההצהרה "איננו רושמים כתובות IP" לא היתה מדויקת — uvicorn ו-Render כן שומרים לוגים טכניים. נוסח מחדש.</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="13" t="inlineStr">
+        <is>
+          <t>88</t>
+        </is>
+      </c>
+      <c r="B96" s="14" t="inlineStr">
+        <is>
+          <t>ביקורת קוד מלאה — 35 קבצים</t>
+        </is>
+      </c>
+      <c r="C96" s="13" t="inlineStr">
+        <is>
+          <t>QA</t>
+        </is>
+      </c>
+      <c r="D96" s="15" t="inlineStr">
+        <is>
+          <t>✅ הושלם</t>
+        </is>
+      </c>
+      <c r="E96" s="16" t="inlineStr">
+        <is>
+          <t>כל הקבצים</t>
+        </is>
+      </c>
+      <c r="F96" s="16" t="inlineStr">
+        <is>
+          <t>11,646 שורות נקראו במלואן. 27 חבילות בדיקה התנהגותיות. אימות חי מול ה-API בייצור (זה מה שחשף פריטים 83-85).</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="3" t="inlineStr">
         <is>
           <t>🔜  NOT YET STARTED</t>
         </is>
       </c>
-      <c r="B59" s="5" t="inlineStr"/>
-      <c r="C59" s="4" t="inlineStr"/>
-      <c r="D59" s="4" t="inlineStr"/>
-      <c r="E59" s="4" t="inlineStr"/>
-      <c r="F59" s="5" t="inlineStr"/>
-    </row>
-    <row r="60">
-      <c r="A60" s="6" t="inlineStr">
+      <c r="B97" s="5" t="inlineStr"/>
+      <c r="C97" s="4" t="inlineStr"/>
+      <c r="D97" s="4" t="inlineStr"/>
+      <c r="E97" s="4" t="inlineStr"/>
+      <c r="F97" s="5" t="inlineStr"/>
+    </row>
+    <row r="98">
+      <c r="A98" s="6" t="inlineStr">
         <is>
           <t>19</t>
         </is>
       </c>
-      <c r="B60" s="7" t="inlineStr">
+      <c r="B98" s="7" t="inlineStr">
         <is>
           <t>Google Play Console — הגשה לחנות</t>
         </is>
       </c>
-      <c r="C60" s="6" t="inlineStr">
+      <c r="C98" s="6" t="inlineStr">
         <is>
           <t>Distribution</t>
         </is>
       </c>
-      <c r="D60" s="8" t="inlineStr">
+      <c r="D98" s="8" t="inlineStr">
         <is>
           <t>🔜</t>
         </is>
       </c>
-      <c r="E60" s="9" t="inlineStr"/>
-      <c r="F60" s="9" t="inlineStr">
+      <c r="E98" s="9" t="inlineStr"/>
+      <c r="F98" s="9" t="inlineStr">
         <is>
           <t>חשבון מפתח ($25) + העלאת AAB + store listing + screenshots.</t>
         </is>
       </c>
     </row>
-    <row r="61">
-      <c r="A61" s="10" t="inlineStr">
+    <row r="99">
+      <c r="A99" s="10" t="inlineStr">
         <is>
           <t>Legend</t>
         </is>
       </c>
     </row>
-    <row r="62">
-      <c r="A62" s="6" t="inlineStr">
+    <row r="100">
+      <c r="A100" s="6" t="inlineStr">
         <is>
           <t>✅ Live</t>
         </is>
       </c>
-      <c r="B62" s="7" t="inlineStr">
+      <c r="B100" s="7" t="inlineStr">
         <is>
           <t>פרוס ופעיל ב-Render — נראה לכל המשתמשים</t>
         </is>
       </c>
-      <c r="C62" s="6" t="inlineStr"/>
-      <c r="D62" s="8" t="inlineStr"/>
-      <c r="E62" s="9" t="inlineStr"/>
-      <c r="F62" s="9" t="inlineStr"/>
-    </row>
-    <row r="63">
-      <c r="A63" s="6" t="inlineStr">
+      <c r="C100" s="6" t="inlineStr"/>
+      <c r="D100" s="8" t="inlineStr"/>
+      <c r="E100" s="9" t="inlineStr"/>
+      <c r="F100" s="9" t="inlineStr"/>
+    </row>
+    <row r="101">
+      <c r="A101" s="6" t="inlineStr">
         <is>
           <t>✅ In APK</t>
         </is>
       </c>
-      <c r="B63" s="7" t="inlineStr">
+      <c r="B101" s="7" t="inlineStr">
         <is>
           <t>כלול ב-APK המותקן — נראה לכל המשתמשים</t>
         </is>
       </c>
-      <c r="C63" s="6" t="inlineStr"/>
-      <c r="D63" s="8" t="inlineStr"/>
-      <c r="E63" s="9" t="inlineStr"/>
-      <c r="F63" s="9" t="inlineStr"/>
-    </row>
-    <row r="64">
-      <c r="A64" s="6" t="inlineStr">
+      <c r="C101" s="6" t="inlineStr"/>
+      <c r="D101" s="8" t="inlineStr"/>
+      <c r="E101" s="9" t="inlineStr"/>
+      <c r="F101" s="9" t="inlineStr"/>
+    </row>
+    <row r="102">
+      <c r="A102" s="6" t="inlineStr">
         <is>
           <t>⏳ Next APK</t>
         </is>
       </c>
-      <c r="B64" s="7" t="inlineStr">
+      <c r="B102" s="7" t="inlineStr">
         <is>
           <t>הקוד מוזג — דורש build ו-APK חדש</t>
         </is>
       </c>
-      <c r="C64" s="6" t="inlineStr"/>
-      <c r="D64" s="8" t="inlineStr"/>
-      <c r="E64" s="9" t="inlineStr"/>
-      <c r="F64" s="9" t="inlineStr"/>
-    </row>
-    <row r="65">
-      <c r="A65" s="6" t="inlineStr">
+      <c r="C102" s="6" t="inlineStr"/>
+      <c r="D102" s="8" t="inlineStr"/>
+      <c r="E102" s="9" t="inlineStr"/>
+      <c r="F102" s="9" t="inlineStr"/>
+    </row>
+    <row r="103">
+      <c r="A103" s="6" t="inlineStr">
         <is>
           <t>✅ Live (OTA)</t>
         </is>
       </c>
-      <c r="B65" s="7" t="inlineStr">
+      <c r="B103" s="7" t="inlineStr">
         <is>
           <t>שינוי JS — מועבר אוטומטית בהפעלה הבאה</t>
         </is>
       </c>
-      <c r="C65" s="6" t="inlineStr"/>
-      <c r="D65" s="8" t="inlineStr"/>
-      <c r="E65" s="9" t="inlineStr"/>
-      <c r="F65" s="9" t="inlineStr"/>
+      <c r="C103" s="6" t="inlineStr"/>
+      <c r="D103" s="8" t="inlineStr"/>
+      <c r="E103" s="9" t="inlineStr"/>
+      <c r="F103" s="9" t="inlineStr"/>
+    </row>
+    <row r="104">
+      <c r="A104" s="21" t="inlineStr">
+        <is>
+          <t>⏳ ממתין ל-push</t>
+        </is>
+      </c>
+      <c r="B104" s="22" t="inlineStr">
+        <is>
+          <t>הקוד מוכן מקומית — טרם נדחף/נפרס</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="21" t="inlineStr">
+        <is>
+          <t>⏳ דורש build</t>
+        </is>
+      </c>
+      <c r="B105" s="22" t="inlineStr">
+        <is>
+          <t>שינוי נייטיב — OTA לא מספיק, צריך AAB/APK חדש</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="23" t="inlineStr">
+        <is>
+          <t>סיכום Session 6</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="24" t="n"/>
+      <c r="B108" s="25" t="inlineStr">
+        <is>
+          <t>37  —  פריטים חדשים שנוספו (52-88)</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="24" t="n"/>
+      <c r="B109" s="25" t="inlineStr">
+        <is>
+          <t>32  —  כבר חיים בייצור או ב-OTA</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="24" t="n"/>
+      <c r="B110" s="25" t="inlineStr">
+        <is>
+          <t>3  —  ממתינים ל-push: no-store, סדרה שנתית, TTM של buyback</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="24" t="n"/>
+      <c r="B111" s="25" t="inlineStr">
+        <is>
+          <t>1  —  דורש build חדש: תמיכת טאבלט</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="24" t="n"/>
+      <c r="B112" s="25" t="inlineStr">
+        <is>
+          <t>11,646  —  שורות קוד שנקראו במלואן, 35 קבצים</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="24" t="n"/>
+      <c r="B113" s="25" t="inlineStr">
+        <is>
+          <t>27  —  חבילות בדיקה התנהגותיות עוברות</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
+  <mergeCells count="3">
+    <mergeCell ref="A107:F107"/>
+    <mergeCell ref="A59:F59"/>
     <mergeCell ref="A25:F25"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Dividend and buyback yield charts are neutral - a falling yield can mean a rising price, not a cut
</commit_message>
<xml_diff>
--- a/BuddhaVest_Progress.xlsx
+++ b/BuddhaVest_Progress.xlsx
@@ -105,7 +105,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="4">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -151,11 +151,31 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00CCCCCC"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00CCCCCC"/>
+      </right>
+      <top style="thin">
+        <color rgb="00CCCCCC"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -219,6 +239,25 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -585,7 +624,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F113"/>
+  <dimension ref="A1:F123"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -606,7 +645,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Last updated: 2026-07-25  |  Session 6</t>
+          <t>Last updated: 2026-07-25  |  Session 7</t>
         </is>
       </c>
     </row>
@@ -2033,130 +2072,130 @@
       </c>
     </row>
     <row r="51">
-      <c r="A51" t="inlineStr">
+      <c r="A51" s="29" t="inlineStr">
         <is>
           <t>44</t>
         </is>
       </c>
-      <c r="B51" t="inlineStr">
+      <c r="B51" s="29" t="inlineStr">
         <is>
           <t>התראות אמיתיות — תזוזות במניות המעקב</t>
         </is>
       </c>
-      <c r="C51" t="inlineStr">
+      <c r="C51" s="29" t="inlineStr">
         <is>
           <t>Backend + Frontend</t>
         </is>
       </c>
-      <c r="D51" t="inlineStr">
-        <is>
-          <t>⏳ ממתין ל-push</t>
-        </is>
-      </c>
-      <c r="E51" t="inlineStr">
+      <c r="D51" s="29" t="inlineStr">
+        <is>
+          <t>✅ Live</t>
+        </is>
+      </c>
+      <c r="E51" s="29" t="inlineStr">
         <is>
           <t>main.py, BrandHeader.js, api.js, i18n.js</t>
         </is>
       </c>
-      <c r="F51" t="inlineStr">
-        <is>
-          <t>endpoint חדש /quotes; מניות מעקב שזזו ≥2% היום מופיעות בפעמון עם נקודה אדומה, ב-4 שפות. סוגר את הבטחת "כאן יופיעו עדכונים".</t>
+      <c r="F51" s="29" t="inlineStr">
+        <is>
+          <t>endpoint חדש /quotes; מניות מעקב שזזו ≥2% היום מופיעות בפעמון עם נקודה אדומה, ב-4 שפות. סוגר את הבטחת "כאן יופיעו עדכונים". תיוג התיישן — אומת שהקוד קיים בענף המרוחק.</t>
         </is>
       </c>
     </row>
     <row r="52">
-      <c r="A52" t="inlineStr">
+      <c r="A52" s="29" t="inlineStr">
         <is>
           <t>45</t>
         </is>
       </c>
-      <c r="B52" t="inlineStr">
+      <c r="B52" s="29" t="inlineStr">
         <is>
           <t>לוגו מרענן גם במסכי מעקב וחדשות</t>
         </is>
       </c>
-      <c r="C52" t="inlineStr">
+      <c r="C52" s="29" t="inlineStr">
         <is>
           <t>Frontend / Bug Fix</t>
         </is>
       </c>
-      <c r="D52" t="inlineStr">
-        <is>
-          <t>⏳ ממתין ל-push</t>
-        </is>
-      </c>
-      <c r="E52" t="inlineStr">
+      <c r="D52" s="29" t="inlineStr">
+        <is>
+          <t>✅ Live (OTA)</t>
+        </is>
+      </c>
+      <c r="E52" s="29" t="inlineStr">
         <is>
           <t>WatchlistScreen.js, NewsScreen.js</t>
         </is>
       </c>
-      <c r="F52" t="inlineStr">
-        <is>
-          <t>ביקורת הבטחות: הטקסט הבטיח רענון מעקב אך הלוגו לא היה מחובר שם.</t>
+      <c r="F52" s="29" t="inlineStr">
+        <is>
+          <t>ביקורת הבטחות: הטקסט הבטיח רענון מעקב אך הלוגו לא היה מחובר שם. תיוג התיישן — אומת שהקוד קיים בענף המרוחק.</t>
         </is>
       </c>
     </row>
     <row r="53">
-      <c r="A53" t="inlineStr">
+      <c r="A53" s="29" t="inlineStr">
         <is>
           <t>46</t>
         </is>
       </c>
-      <c r="B53" t="inlineStr">
+      <c r="B53" s="29" t="inlineStr">
         <is>
           <t>תווית גרסה v1.0.0 (היה v1.2)</t>
         </is>
       </c>
-      <c r="C53" t="inlineStr">
+      <c r="C53" s="29" t="inlineStr">
         <is>
           <t>Frontend</t>
         </is>
       </c>
-      <c r="D53" t="inlineStr">
-        <is>
-          <t>⏳ ממתין ל-push</t>
-        </is>
-      </c>
-      <c r="E53" t="inlineStr">
+      <c r="D53" s="29" t="inlineStr">
+        <is>
+          <t>✅ Live (OTA)</t>
+        </is>
+      </c>
+      <c r="E53" s="29" t="inlineStr">
         <is>
           <t>MoreScreen.js</t>
         </is>
       </c>
-      <c r="F53" t="inlineStr">
-        <is>
-          <t>יישור מול version בחנות.</t>
+      <c r="F53" s="29" t="inlineStr">
+        <is>
+          <t>יישור מול version בחנות. תיוג התיישן — אומת שהקוד קיים בענף המרוחק.</t>
         </is>
       </c>
     </row>
     <row r="54">
-      <c r="A54" t="inlineStr">
+      <c r="A54" s="29" t="inlineStr">
         <is>
           <t>47</t>
         </is>
       </c>
-      <c r="B54" t="inlineStr">
+      <c r="B54" s="29" t="inlineStr">
         <is>
           <t>תיקוני נוסח: ToS/מי-אני + גילוי תרגום בפרטיות</t>
         </is>
       </c>
-      <c r="C54" t="inlineStr">
+      <c r="C54" s="29" t="inlineStr">
         <is>
           <t>Legal / i18n</t>
         </is>
       </c>
-      <c r="D54" t="inlineStr">
-        <is>
-          <t>⏳ ממתין ל-push</t>
-        </is>
-      </c>
-      <c r="E54" t="inlineStr">
+      <c r="D54" s="29" t="inlineStr">
+        <is>
+          <t>✅ Live (OTA)</t>
+        </is>
+      </c>
+      <c r="E54" s="29" t="inlineStr">
         <is>
           <t>constants/i18n.js</t>
         </is>
       </c>
-      <c r="F54" t="inlineStr">
-        <is>
-          <t>"אין לי רישיון" (היה "לא רישוי"); גילוי Google Translate בסעיף הפרטיות ב-4 שפות; אומת שהנוסחה 40/35/25 תואמת את analyzer.py.</t>
+      <c r="F54" s="29" t="inlineStr">
+        <is>
+          <t>"אין לי רישיון" (היה "לא רישוי"); גילוי Google Translate בסעיף הפרטיות ב-4 שפות; אומת שהנוסחה 40/35/25 תואמת את analyzer.py. תיוג התיישן — אומת שהקוד קיים בענף המרוחק.</t>
         </is>
       </c>
     </row>
@@ -2296,22 +2335,22 @@
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="13" t="inlineStr">
+      <c r="A60" s="26" t="inlineStr">
         <is>
           <t>52</t>
         </is>
       </c>
-      <c r="B60" s="14" t="inlineStr">
+      <c r="B60" s="27" t="inlineStr">
         <is>
           <t>מרוץ שפות — 5 מסכים/רכיבים</t>
         </is>
       </c>
-      <c r="C60" s="13" t="inlineStr">
+      <c r="C60" s="26" t="inlineStr">
         <is>
           <t>Frontend / Bug Fix</t>
         </is>
       </c>
-      <c r="D60" s="15" t="inlineStr">
+      <c r="D60" s="28" t="inlineStr">
         <is>
           <t>✅ Live (OTA)</t>
         </is>
@@ -2328,22 +2367,22 @@
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="13" t="inlineStr">
+      <c r="A61" s="26" t="inlineStr">
         <is>
           <t>53</t>
         </is>
       </c>
-      <c r="B61" s="14" t="inlineStr">
+      <c r="B61" s="27" t="inlineStr">
         <is>
           <t>Volume/Avg Vol ריקים לסירוגין</t>
         </is>
       </c>
-      <c r="C61" s="13" t="inlineStr">
+      <c r="C61" s="26" t="inlineStr">
         <is>
           <t>Backend / Bug Fix</t>
         </is>
       </c>
-      <c r="D61" s="15" t="inlineStr">
+      <c r="D61" s="28" t="inlineStr">
         <is>
           <t>✅ Live</t>
         </is>
@@ -2360,22 +2399,22 @@
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="13" t="inlineStr">
+      <c r="A62" s="26" t="inlineStr">
         <is>
           <t>54</t>
         </is>
       </c>
-      <c r="B62" s="14" t="inlineStr">
+      <c r="B62" s="27" t="inlineStr">
         <is>
           <t>המרת אגורות→שקל למניות ת"א</t>
         </is>
       </c>
-      <c r="C62" s="13" t="inlineStr">
+      <c r="C62" s="26" t="inlineStr">
         <is>
           <t>Backend</t>
         </is>
       </c>
-      <c r="D62" s="15" t="inlineStr">
+      <c r="D62" s="28" t="inlineStr">
         <is>
           <t>✅ Live</t>
         </is>
@@ -2392,22 +2431,22 @@
       </c>
     </row>
     <row r="63">
-      <c r="A63" s="13" t="inlineStr">
+      <c r="A63" s="26" t="inlineStr">
         <is>
           <t>55</t>
         </is>
       </c>
-      <c r="B63" s="14" t="inlineStr">
+      <c r="B63" s="27" t="inlineStr">
         <is>
           <t>באג יחידות ב-Buyback (3500000000%)</t>
         </is>
       </c>
-      <c r="C63" s="13" t="inlineStr">
+      <c r="C63" s="26" t="inlineStr">
         <is>
           <t>Backend + Frontend</t>
         </is>
       </c>
-      <c r="D63" s="15" t="inlineStr">
+      <c r="D63" s="28" t="inlineStr">
         <is>
           <t>✅ Live</t>
         </is>
@@ -2424,22 +2463,22 @@
       </c>
     </row>
     <row r="64">
-      <c r="A64" s="13" t="inlineStr">
+      <c r="A64" s="26" t="inlineStr">
         <is>
           <t>56</t>
         </is>
       </c>
-      <c r="B64" s="14" t="inlineStr">
+      <c r="B64" s="27" t="inlineStr">
         <is>
           <t>תיקוני נכונות במנוע הציון</t>
         </is>
       </c>
-      <c r="C64" s="13" t="inlineStr">
+      <c r="C64" s="26" t="inlineStr">
         <is>
           <t>Backend / Scoring</t>
         </is>
       </c>
-      <c r="D64" s="15" t="inlineStr">
+      <c r="D64" s="28" t="inlineStr">
         <is>
           <t>✅ Live</t>
         </is>
@@ -2456,22 +2495,22 @@
       </c>
     </row>
     <row r="65">
-      <c r="A65" s="13" t="inlineStr">
+      <c r="A65" s="26" t="inlineStr">
         <is>
           <t>57</t>
         </is>
       </c>
-      <c r="B65" s="14" t="inlineStr">
+      <c r="B65" s="27" t="inlineStr">
         <is>
           <t>ניסוח דיבידנד כן — לא "משולם בעקביות"</t>
         </is>
       </c>
-      <c r="C65" s="13" t="inlineStr">
+      <c r="C65" s="26" t="inlineStr">
         <is>
           <t>Legal / Accuracy</t>
         </is>
       </c>
-      <c r="D65" s="15" t="inlineStr">
+      <c r="D65" s="28" t="inlineStr">
         <is>
           <t>✅ Live</t>
         </is>
@@ -2488,22 +2527,22 @@
       </c>
     </row>
     <row r="66">
-      <c r="A66" s="13" t="inlineStr">
+      <c r="A66" s="26" t="inlineStr">
         <is>
           <t>58</t>
         </is>
       </c>
-      <c r="B66" s="14" t="inlineStr">
+      <c r="B66" s="27" t="inlineStr">
         <is>
           <t>SSRF — /translate-article</t>
         </is>
       </c>
-      <c r="C66" s="13" t="inlineStr">
+      <c r="C66" s="26" t="inlineStr">
         <is>
           <t>Backend / Security</t>
         </is>
       </c>
-      <c r="D66" s="15" t="inlineStr">
+      <c r="D66" s="28" t="inlineStr">
         <is>
           <t>✅ Live</t>
         </is>
@@ -2520,22 +2559,22 @@
       </c>
     </row>
     <row r="67">
-      <c r="A67" s="13" t="inlineStr">
+      <c r="A67" s="26" t="inlineStr">
         <is>
           <t>59</t>
         </is>
       </c>
-      <c r="B67" s="14" t="inlineStr">
+      <c r="B67" s="27" t="inlineStr">
         <is>
           <t>XSS ב-WebView של הכתבות</t>
         </is>
       </c>
-      <c r="C67" s="13" t="inlineStr">
+      <c r="C67" s="26" t="inlineStr">
         <is>
           <t>Frontend / Security</t>
         </is>
       </c>
-      <c r="D67" s="15" t="inlineStr">
+      <c r="D67" s="28" t="inlineStr">
         <is>
           <t>✅ Live (OTA)</t>
         </is>
@@ -2552,22 +2591,22 @@
       </c>
     </row>
     <row r="68">
-      <c r="A68" s="13" t="inlineStr">
+      <c r="A68" s="26" t="inlineStr">
         <is>
           <t>60</t>
         </is>
       </c>
-      <c r="B68" s="14" t="inlineStr">
+      <c r="B68" s="27" t="inlineStr">
         <is>
           <t>הסרת /debug-pe ו-/debug-rows</t>
         </is>
       </c>
-      <c r="C68" s="13" t="inlineStr">
+      <c r="C68" s="26" t="inlineStr">
         <is>
           <t>Backend / Security</t>
         </is>
       </c>
-      <c r="D68" s="15" t="inlineStr">
+      <c r="D68" s="28" t="inlineStr">
         <is>
           <t>✅ Live</t>
         </is>
@@ -2584,22 +2623,22 @@
       </c>
     </row>
     <row r="69">
-      <c r="A69" s="13" t="inlineStr">
+      <c r="A69" s="26" t="inlineStr">
         <is>
           <t>61</t>
         </is>
       </c>
-      <c r="B69" s="14" t="inlineStr">
+      <c r="B69" s="27" t="inlineStr">
         <is>
           <t>5 דליפות של פרטי חריגה ללקוח</t>
         </is>
       </c>
-      <c r="C69" s="13" t="inlineStr">
+      <c r="C69" s="26" t="inlineStr">
         <is>
           <t>Backend / Security</t>
         </is>
       </c>
-      <c r="D69" s="15" t="inlineStr">
+      <c r="D69" s="28" t="inlineStr">
         <is>
           <t>✅ Live</t>
         </is>
@@ -2616,22 +2655,22 @@
       </c>
     </row>
     <row r="70">
-      <c r="A70" s="13" t="inlineStr">
+      <c r="A70" s="26" t="inlineStr">
         <is>
           <t>62</t>
         </is>
       </c>
-      <c r="B70" s="14" t="inlineStr">
+      <c r="B70" s="27" t="inlineStr">
         <is>
           <t>פיצוץ זיכרון בעליית השרת</t>
         </is>
       </c>
-      <c r="C70" s="13" t="inlineStr">
+      <c r="C70" s="26" t="inlineStr">
         <is>
           <t>Backend / Performance</t>
         </is>
       </c>
-      <c r="D70" s="15" t="inlineStr">
+      <c r="D70" s="28" t="inlineStr">
         <is>
           <t>✅ Live</t>
         </is>
@@ -2648,22 +2687,22 @@
       </c>
     </row>
     <row r="71">
-      <c r="A71" s="13" t="inlineStr">
+      <c r="A71" s="26" t="inlineStr">
         <is>
           <t>63</t>
         </is>
       </c>
-      <c r="B71" s="14" t="inlineStr">
+      <c r="B71" s="27" t="inlineStr">
         <is>
           <t>תקרת מטמון + single-flight</t>
         </is>
       </c>
-      <c r="C71" s="13" t="inlineStr">
+      <c r="C71" s="26" t="inlineStr">
         <is>
           <t>Backend / Performance</t>
         </is>
       </c>
-      <c r="D71" s="15" t="inlineStr">
+      <c r="D71" s="28" t="inlineStr">
         <is>
           <t>✅ Live</t>
         </is>
@@ -2680,22 +2719,22 @@
       </c>
     </row>
     <row r="72">
-      <c r="A72" s="13" t="inlineStr">
+      <c r="A72" s="26" t="inlineStr">
         <is>
           <t>64</t>
         </is>
       </c>
-      <c r="B72" s="14" t="inlineStr">
+      <c r="B72" s="27" t="inlineStr">
         <is>
           <t>חלון היסטוריה 10y במקום max</t>
         </is>
       </c>
-      <c r="C72" s="13" t="inlineStr">
+      <c r="C72" s="26" t="inlineStr">
         <is>
           <t>Backend / Performance</t>
         </is>
       </c>
-      <c r="D72" s="15" t="inlineStr">
+      <c r="D72" s="28" t="inlineStr">
         <is>
           <t>✅ Live</t>
         </is>
@@ -2712,22 +2751,22 @@
       </c>
     </row>
     <row r="73">
-      <c r="A73" s="13" t="inlineStr">
+      <c r="A73" s="26" t="inlineStr">
         <is>
           <t>65</t>
         </is>
       </c>
-      <c r="B73" s="14" t="inlineStr">
+      <c r="B73" s="27" t="inlineStr">
         <is>
           <t>Debounce בחיפוש</t>
         </is>
       </c>
-      <c r="C73" s="13" t="inlineStr">
+      <c r="C73" s="26" t="inlineStr">
         <is>
           <t>Frontend / Performance</t>
         </is>
       </c>
-      <c r="D73" s="15" t="inlineStr">
+      <c r="D73" s="28" t="inlineStr">
         <is>
           <t>✅ Live (OTA)</t>
         </is>
@@ -2744,22 +2783,22 @@
       </c>
     </row>
     <row r="74">
-      <c r="A74" s="13" t="inlineStr">
+      <c r="A74" s="26" t="inlineStr">
         <is>
           <t>66</t>
         </is>
       </c>
-      <c r="B74" s="14" t="inlineStr">
+      <c r="B74" s="27" t="inlineStr">
         <is>
           <t>תקציב זמן ל-Stooq</t>
         </is>
       </c>
-      <c r="C74" s="13" t="inlineStr">
+      <c r="C74" s="26" t="inlineStr">
         <is>
           <t>Backend / Performance</t>
         </is>
       </c>
-      <c r="D74" s="15" t="inlineStr">
+      <c r="D74" s="28" t="inlineStr">
         <is>
           <t>✅ Live</t>
         </is>
@@ -2776,22 +2815,22 @@
       </c>
     </row>
     <row r="75">
-      <c r="A75" s="13" t="inlineStr">
+      <c r="A75" s="26" t="inlineStr">
         <is>
           <t>67</t>
         </is>
       </c>
-      <c r="B75" s="14" t="inlineStr">
+      <c r="B75" s="27" t="inlineStr">
         <is>
           <t>אובדן נתונים ביומן המחקר</t>
         </is>
       </c>
-      <c r="C75" s="13" t="inlineStr">
+      <c r="C75" s="26" t="inlineStr">
         <is>
           <t>Frontend / Bug Fix</t>
         </is>
       </c>
-      <c r="D75" s="15" t="inlineStr">
+      <c r="D75" s="28" t="inlineStr">
         <is>
           <t>✅ Live (OTA)</t>
         </is>
@@ -2840,22 +2879,22 @@
       </c>
     </row>
     <row r="77">
-      <c r="A77" s="13" t="inlineStr">
+      <c r="A77" s="26" t="inlineStr">
         <is>
           <t>69</t>
         </is>
       </c>
-      <c r="B77" s="14" t="inlineStr">
+      <c r="B77" s="27" t="inlineStr">
         <is>
           <t>מסך הסכמה בהפעלה ראשונה</t>
         </is>
       </c>
-      <c r="C77" s="13" t="inlineStr">
+      <c r="C77" s="26" t="inlineStr">
         <is>
           <t>Legal</t>
         </is>
       </c>
-      <c r="D77" s="15" t="inlineStr">
+      <c r="D77" s="28" t="inlineStr">
         <is>
           <t>✅ Live (OTA)</t>
         </is>
@@ -2872,22 +2911,22 @@
       </c>
     </row>
     <row r="78">
-      <c r="A78" s="13" t="inlineStr">
+      <c r="A78" s="26" t="inlineStr">
         <is>
           <t>70</t>
         </is>
       </c>
-      <c r="B78" s="14" t="inlineStr">
+      <c r="B78" s="27" t="inlineStr">
         <is>
           <t>שכתוב תיאור החנות — בלי הבטחות</t>
         </is>
       </c>
-      <c r="C78" s="13" t="inlineStr">
+      <c r="C78" s="26" t="inlineStr">
         <is>
           <t>Legal / Store</t>
         </is>
       </c>
-      <c r="D78" s="15" t="inlineStr">
+      <c r="D78" s="28" t="inlineStr">
         <is>
           <t>✅ מוכן</t>
         </is>
@@ -2904,22 +2943,22 @@
       </c>
     </row>
     <row r="79">
-      <c r="A79" s="13" t="inlineStr">
+      <c r="A79" s="26" t="inlineStr">
         <is>
           <t>71</t>
         </is>
       </c>
-      <c r="B79" s="14" t="inlineStr">
+      <c r="B79" s="27" t="inlineStr">
         <is>
           <t>מדריך צילומי מסך לחנות</t>
         </is>
       </c>
-      <c r="C79" s="13" t="inlineStr">
+      <c r="C79" s="26" t="inlineStr">
         <is>
           <t>Store Assets</t>
         </is>
       </c>
-      <c r="D79" s="15" t="inlineStr">
+      <c r="D79" s="28" t="inlineStr">
         <is>
           <t>✅ הושלם</t>
         </is>
@@ -2936,22 +2975,22 @@
       </c>
     </row>
     <row r="80">
-      <c r="A80" s="13" t="inlineStr">
+      <c r="A80" s="26" t="inlineStr">
         <is>
           <t>72</t>
         </is>
       </c>
-      <c r="B80" s="14" t="inlineStr">
+      <c r="B80" s="27" t="inlineStr">
         <is>
           <t>RTL בכל המסכים</t>
         </is>
       </c>
-      <c r="C80" s="13" t="inlineStr">
+      <c r="C80" s="26" t="inlineStr">
         <is>
           <t>Frontend / i18n</t>
         </is>
       </c>
-      <c r="D80" s="15" t="inlineStr">
+      <c r="D80" s="28" t="inlineStr">
         <is>
           <t>✅ Live (OTA)</t>
         </is>
@@ -2968,22 +3007,22 @@
       </c>
     </row>
     <row r="81">
-      <c r="A81" s="13" t="inlineStr">
+      <c r="A81" s="26" t="inlineStr">
         <is>
           <t>73</t>
         </is>
       </c>
-      <c r="B81" s="14" t="inlineStr">
+      <c r="B81" s="27" t="inlineStr">
         <is>
           <t>תווית גרסה מ-app.json</t>
         </is>
       </c>
-      <c r="C81" s="13" t="inlineStr">
+      <c r="C81" s="26" t="inlineStr">
         <is>
           <t>Frontend</t>
         </is>
       </c>
-      <c r="D81" s="15" t="inlineStr">
+      <c r="D81" s="28" t="inlineStr">
         <is>
           <t>✅ Live (OTA)</t>
         </is>
@@ -3000,22 +3039,22 @@
       </c>
     </row>
     <row r="82">
-      <c r="A82" s="13" t="inlineStr">
+      <c r="A82" s="26" t="inlineStr">
         <is>
           <t>74</t>
         </is>
       </c>
-      <c r="B82" s="14" t="inlineStr">
+      <c r="B82" s="27" t="inlineStr">
         <is>
           <t>טעינה דו-שלבית ברשימת המעקב</t>
         </is>
       </c>
-      <c r="C82" s="13" t="inlineStr">
+      <c r="C82" s="26" t="inlineStr">
         <is>
           <t>Frontend / Performance</t>
         </is>
       </c>
-      <c r="D82" s="15" t="inlineStr">
+      <c r="D82" s="28" t="inlineStr">
         <is>
           <t>✅ Live (OTA)</t>
         </is>
@@ -3032,22 +3071,22 @@
       </c>
     </row>
     <row r="83">
-      <c r="A83" s="13" t="inlineStr">
+      <c r="A83" s="26" t="inlineStr">
         <is>
           <t>75</t>
         </is>
       </c>
-      <c r="B83" s="14" t="inlineStr">
+      <c r="B83" s="27" t="inlineStr">
         <is>
           <t>/quotes: אגורות, שם חברה, מטבע</t>
         </is>
       </c>
-      <c r="C83" s="13" t="inlineStr">
+      <c r="C83" s="26" t="inlineStr">
         <is>
           <t>Backend</t>
         </is>
       </c>
-      <c r="D83" s="15" t="inlineStr">
+      <c r="D83" s="28" t="inlineStr">
         <is>
           <t>✅ Live</t>
         </is>
@@ -3064,22 +3103,22 @@
       </c>
     </row>
     <row r="84">
-      <c r="A84" s="13" t="inlineStr">
+      <c r="A84" s="26" t="inlineStr">
         <is>
           <t>76</t>
         </is>
       </c>
-      <c r="B84" s="14" t="inlineStr">
+      <c r="B84" s="27" t="inlineStr">
         <is>
           <t>מיזוג במקום החלפה ברשימת המעקב</t>
         </is>
       </c>
-      <c r="C84" s="13" t="inlineStr">
+      <c r="C84" s="26" t="inlineStr">
         <is>
           <t>Frontend / Bug Fix</t>
         </is>
       </c>
-      <c r="D84" s="15" t="inlineStr">
+      <c r="D84" s="28" t="inlineStr">
         <is>
           <t>✅ Live (OTA)</t>
         </is>
@@ -3096,22 +3135,22 @@
       </c>
     </row>
     <row r="85">
-      <c r="A85" s="13" t="inlineStr">
+      <c r="A85" s="26" t="inlineStr">
         <is>
           <t>77</t>
         </is>
       </c>
-      <c r="B85" s="14" t="inlineStr">
+      <c r="B85" s="27" t="inlineStr">
         <is>
           <t>מרוץ במסך הבית — market/FX</t>
         </is>
       </c>
-      <c r="C85" s="13" t="inlineStr">
+      <c r="C85" s="26" t="inlineStr">
         <is>
           <t>Frontend / Bug Fix</t>
         </is>
       </c>
-      <c r="D85" s="15" t="inlineStr">
+      <c r="D85" s="28" t="inlineStr">
         <is>
           <t>✅ Live (OTA)</t>
         </is>
@@ -3128,22 +3167,22 @@
       </c>
     </row>
     <row r="86">
-      <c r="A86" s="13" t="inlineStr">
+      <c r="A86" s="26" t="inlineStr">
         <is>
           <t>78</t>
         </is>
       </c>
-      <c r="B86" s="14" t="inlineStr">
+      <c r="B86" s="27" t="inlineStr">
         <is>
           <t>תשובה ריקה לא מוחקת נתונים טובים</t>
         </is>
       </c>
-      <c r="C86" s="13" t="inlineStr">
+      <c r="C86" s="26" t="inlineStr">
         <is>
           <t>Frontend / Bug Fix</t>
         </is>
       </c>
-      <c r="D86" s="15" t="inlineStr">
+      <c r="D86" s="28" t="inlineStr">
         <is>
           <t>✅ Live (OTA)</t>
         </is>
@@ -3160,22 +3199,22 @@
       </c>
     </row>
     <row r="87">
-      <c r="A87" s="13" t="inlineStr">
+      <c r="A87" s="26" t="inlineStr">
         <is>
           <t>79</t>
         </is>
       </c>
-      <c r="B87" s="14" t="inlineStr">
+      <c r="B87" s="27" t="inlineStr">
         <is>
           <t>תרגום כתבה ישנה דלף לחדשה</t>
         </is>
       </c>
-      <c r="C87" s="13" t="inlineStr">
+      <c r="C87" s="26" t="inlineStr">
         <is>
           <t>Frontend / Bug Fix</t>
         </is>
       </c>
-      <c r="D87" s="15" t="inlineStr">
+      <c r="D87" s="28" t="inlineStr">
         <is>
           <t>✅ Live (OTA)</t>
         </is>
@@ -3192,22 +3231,22 @@
       </c>
     </row>
     <row r="88">
-      <c r="A88" s="13" t="inlineStr">
+      <c r="A88" s="26" t="inlineStr">
         <is>
           <t>80</t>
         </is>
       </c>
-      <c r="B88" s="14" t="inlineStr">
+      <c r="B88" s="27" t="inlineStr">
         <is>
           <t>מרוץ ב"נסה שוב" של פירוט מדד</t>
         </is>
       </c>
-      <c r="C88" s="13" t="inlineStr">
+      <c r="C88" s="26" t="inlineStr">
         <is>
           <t>Frontend / Bug Fix</t>
         </is>
       </c>
-      <c r="D88" s="15" t="inlineStr">
+      <c r="D88" s="28" t="inlineStr">
         <is>
           <t>✅ Live (OTA)</t>
         </is>
@@ -3224,22 +3263,22 @@
       </c>
     </row>
     <row r="89">
-      <c r="A89" s="13" t="inlineStr">
+      <c r="A89" s="26" t="inlineStr">
         <is>
           <t>81</t>
         </is>
       </c>
-      <c r="B89" s="14" t="inlineStr">
+      <c r="B89" s="27" t="inlineStr">
         <is>
           <t>סולם VIX לא מונוטוני</t>
         </is>
       </c>
-      <c r="C89" s="13" t="inlineStr">
+      <c r="C89" s="26" t="inlineStr">
         <is>
           <t>Frontend / i18n</t>
         </is>
       </c>
-      <c r="D89" s="15" t="inlineStr">
+      <c r="D89" s="28" t="inlineStr">
         <is>
           <t>✅ Live (OTA)</t>
         </is>
@@ -3256,22 +3295,22 @@
       </c>
     </row>
     <row r="90">
-      <c r="A90" s="13" t="inlineStr">
+      <c r="A90" s="26" t="inlineStr">
         <is>
           <t>82</t>
         </is>
       </c>
-      <c r="B90" s="14" t="inlineStr">
+      <c r="B90" s="27" t="inlineStr">
         <is>
           <t>תיקוני תוכן בספרדית</t>
         </is>
       </c>
-      <c r="C90" s="13" t="inlineStr">
+      <c r="C90" s="26" t="inlineStr">
         <is>
           <t>i18n / Accuracy</t>
         </is>
       </c>
-      <c r="D90" s="15" t="inlineStr">
+      <c r="D90" s="28" t="inlineStr">
         <is>
           <t>✅ Live (OTA)</t>
         </is>
@@ -3288,389 +3327,670 @@
       </c>
     </row>
     <row r="91">
-      <c r="A91" s="17" t="inlineStr">
+      <c r="A91" s="26" t="inlineStr">
         <is>
           <t>83</t>
         </is>
       </c>
-      <c r="B91" s="18" t="inlineStr">
+      <c r="B91" s="27" t="inlineStr">
         <is>
           <t>Cache-Control: no-store על כל ה-API</t>
         </is>
       </c>
-      <c r="C91" s="17" t="inlineStr">
+      <c r="C91" s="26" t="inlineStr">
         <is>
           <t>Backend / Bug Fix</t>
         </is>
       </c>
-      <c r="D91" s="19" t="inlineStr">
+      <c r="D91" s="28" t="inlineStr">
+        <is>
+          <t>✅ Live</t>
+        </is>
+      </c>
+      <c r="E91" s="16" t="inlineStr">
+        <is>
+          <t>main.py</t>
+        </is>
+      </c>
+      <c r="F91" s="16" t="inlineStr">
+        <is>
+          <t>הסיבה האמיתית שדלק חזרה: OkHttp של אנדרואיד שמר תשובה שנוצרה בגרסת קוד ישנה. הוכח — אותה מניה ב-en החזירה 8173 וב-ru החזירה 84.45. נדחף ונפרס; אומת חי מול השרת.</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="26" t="inlineStr">
+        <is>
+          <t>84</t>
+        </is>
+      </c>
+      <c r="B92" s="27" t="inlineStr">
+        <is>
+          <t>סדרה שנתית = סוף שנה, לא ינואר</t>
+        </is>
+      </c>
+      <c r="C92" s="26" t="inlineStr">
+        <is>
+          <t>Backend / Bug Fix</t>
+        </is>
+      </c>
+      <c r="D92" s="28" t="inlineStr">
+        <is>
+          <t>✅ Live</t>
+        </is>
+      </c>
+      <c r="E92" s="16" t="inlineStr">
+        <is>
+          <t>main.py</t>
+        </is>
+      </c>
+      <c r="F92" s="16" t="inlineStr">
+        <is>
+          <t>הגרף השנתי הציג את ינואר בתווית של השנה. KO 2023: הוצג 25.25 במקום 22.19 — סטייה 12%. תוקן ב-4 מקומות. נדחף ונפרס; אומת חי מול השרת.</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="26" t="inlineStr">
+        <is>
+          <t>85</t>
+        </is>
+      </c>
+      <c r="B93" s="27" t="inlineStr">
+        <is>
+          <t>TTM של Buyback דרש 2 רבעונים</t>
+        </is>
+      </c>
+      <c r="C93" s="26" t="inlineStr">
+        <is>
+          <t>Backend / Bug Fix</t>
+        </is>
+      </c>
+      <c r="D93" s="28" t="inlineStr">
+        <is>
+          <t>✅ Live</t>
+        </is>
+      </c>
+      <c r="E93" s="16" t="inlineStr">
+        <is>
+          <t>main.py</t>
+        </is>
+      </c>
+      <c r="F93" s="16" t="inlineStr">
+        <is>
+          <t>"תשואה שנתית" יכלה להיות סכום של חצי שנה. הועלה ל-4 כמו כל שאר חישובי ה-TTM. נדחף ונפרס; אומת חי מול השרת.</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="26" t="inlineStr">
+        <is>
+          <t>86</t>
+        </is>
+      </c>
+      <c r="B94" s="27" t="inlineStr">
+        <is>
+          <t>ניקוי ריפו — cloudflared.exe 52MB</t>
+        </is>
+      </c>
+      <c r="C94" s="26" t="inlineStr">
+        <is>
+          <t>DevOps</t>
+        </is>
+      </c>
+      <c r="D94" s="28" t="inlineStr">
+        <is>
+          <t>✅ Live</t>
+        </is>
+      </c>
+      <c r="E94" s="16" t="inlineStr">
+        <is>
+          <t>‎.gitignore</t>
+        </is>
+      </c>
+      <c r="F94" s="16" t="inlineStr">
+        <is>
+          <t>יצא ממעקב git, נשאר על הדיסק המקומי.</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="26" t="inlineStr">
+        <is>
+          <t>87</t>
+        </is>
+      </c>
+      <c r="B95" s="27" t="inlineStr">
+        <is>
+          <t>דיוק עמוד הפרטיות בנוגע ללוגים</t>
+        </is>
+      </c>
+      <c r="C95" s="26" t="inlineStr">
+        <is>
+          <t>Legal</t>
+        </is>
+      </c>
+      <c r="D95" s="28" t="inlineStr">
+        <is>
+          <t>✅ Live</t>
+        </is>
+      </c>
+      <c r="E95" s="16" t="inlineStr">
+        <is>
+          <t>main.py</t>
+        </is>
+      </c>
+      <c r="F95" s="16" t="inlineStr">
+        <is>
+          <t>ההצהרה "איננו רושמים כתובות IP" לא היתה מדויקת — uvicorn ו-Render כן שומרים לוגים טכניים. נוסח מחדש.</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="26" t="inlineStr">
+        <is>
+          <t>88</t>
+        </is>
+      </c>
+      <c r="B96" s="27" t="inlineStr">
+        <is>
+          <t>ביקורת קוד מלאה — 35 קבצים</t>
+        </is>
+      </c>
+      <c r="C96" s="26" t="inlineStr">
+        <is>
+          <t>QA</t>
+        </is>
+      </c>
+      <c r="D96" s="28" t="inlineStr">
+        <is>
+          <t>✅ הושלם</t>
+        </is>
+      </c>
+      <c r="E96" s="16" t="inlineStr">
+        <is>
+          <t>כל הקבצים</t>
+        </is>
+      </c>
+      <c r="F96" s="16" t="inlineStr">
+        <is>
+          <t>11,646 שורות נקראו במלואן. 27 חבילות בדיקה התנהגותיות. אימות חי מול ה-API בייצור (זה מה שחשף פריטים 83-85).</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="12" t="inlineStr">
+        <is>
+          <t>✅  Session 7 (2026-07-25): עקביות חזותית, הצהרת ספים, כיסוי שפות</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="26" t="inlineStr">
+        <is>
+          <t>89</t>
+        </is>
+      </c>
+      <c r="B98" s="27" t="inlineStr">
+        <is>
+          <t>צבע הגרף לפי כיוון המדד</t>
+        </is>
+      </c>
+      <c r="C98" s="26" t="inlineStr">
+        <is>
+          <t>Frontend / UX</t>
+        </is>
+      </c>
+      <c r="D98" s="28" t="inlineStr">
+        <is>
+          <t>✅ Live (OTA)</t>
+        </is>
+      </c>
+      <c r="E98" s="16" t="inlineStr">
+        <is>
+          <t>PriceChart.js, MetricHistoryScreen.js</t>
+        </is>
+      </c>
+      <c r="F98" s="16" t="inlineStr">
+        <is>
+          <t>הגרף צבע לפי מגמה בלבד: P/B שעלה מ-4.3 ל-7.81 קיבל ירוק ("עולה") בעוד האריח צבע את אותו מספר אדום ("יקר"). עכשיו במכפילים שבהם נמוך=טוב ירידה היא הירוקה. גרף מחיר-תחליף נשאר בלוגיקה רגילה.</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="26" t="inlineStr">
+        <is>
+          <t>90</t>
+        </is>
+      </c>
+      <c r="B99" s="27" t="inlineStr">
+        <is>
+          <t>הצהרת טווח מלא לכל 24 המדדים</t>
+        </is>
+      </c>
+      <c r="C99" s="26" t="inlineStr">
+        <is>
+          <t>UX / Accuracy</t>
+        </is>
+      </c>
+      <c r="D99" s="28" t="inlineStr">
+        <is>
+          <t>✅ Live (OTA)</t>
+        </is>
+      </c>
+      <c r="E99" s="16" t="inlineStr">
+        <is>
+          <t>constants/i18n.js</t>
+        </is>
+      </c>
+      <c r="F99" s="16" t="inlineStr">
+        <is>
+          <t>האפליקציה צבעה אדום לפי סף שלא סיפרה עליו ("מתחת ל-1 זול" בלבד). עכשיו כל מדד מצהיר מינימום/אמצע/מקסימום — או אומר במפורש שאין לו סף ולמה. 15 מדדים עם מספרים אומתו מול הקוד. 4 שפות.</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="26" t="inlineStr">
+        <is>
+          <t>91</t>
+        </is>
+      </c>
+      <c r="B100" s="27" t="inlineStr">
+        <is>
+          <t>מדד שלא היה לו הסבר בכלל</t>
+        </is>
+      </c>
+      <c r="C100" s="26" t="inlineStr">
+        <is>
+          <t>UX / Bug Fix</t>
+        </is>
+      </c>
+      <c r="D100" s="28" t="inlineStr">
+        <is>
+          <t>✅ Live (OTA)</t>
+        </is>
+      </c>
+      <c r="E100" s="16" t="inlineStr">
+        <is>
+          <t>constants/i18n.js</t>
+        </is>
+      </c>
+      <c r="F100" s="16" t="inlineStr">
+        <is>
+          <t>net_income_trend הופיע ברשימת שמות המדדים אך חסר לגמרי במילון ההסברים — לחיצה על האריח הציגה כלום. נוסף ב-4 שפות עם ארבעת המצבים מ-analyzer.</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="26" t="inlineStr">
+        <is>
+          <t>92</t>
+        </is>
+      </c>
+      <c r="B101" s="27" t="inlineStr">
+        <is>
+          <t>מספר וכיתוב באותו צבע</t>
+        </is>
+      </c>
+      <c r="C101" s="26" t="inlineStr">
+        <is>
+          <t>Frontend / UX</t>
+        </is>
+      </c>
+      <c r="D101" s="28" t="inlineStr">
+        <is>
+          <t>✅ Live (OTA)</t>
+        </is>
+      </c>
+      <c r="E101" s="16" t="inlineStr">
+        <is>
+          <t>MetricTile.js, StockScreen.js</t>
+        </is>
+      </c>
+      <c r="F101" s="16" t="inlineStr">
+        <is>
+          <t>שני סוגי האריחים צבעו הפוך זה מזה: באריחי הציון המספר ניטרלי והכיתוב צבוע, במכפילים הנוספים להפך. עכשיו שניהם נושאים סיגנל אחד.</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="26" t="inlineStr">
+        <is>
+          <t>93</t>
+        </is>
+      </c>
+      <c r="B102" s="27" t="inlineStr">
+        <is>
+          <t>כתום רק כשיש אזהרה</t>
+        </is>
+      </c>
+      <c r="C102" s="26" t="inlineStr">
+        <is>
+          <t>Frontend / UX</t>
+        </is>
+      </c>
+      <c r="D102" s="28" t="inlineStr">
+        <is>
+          <t>✅ Live (OTA)</t>
+        </is>
+      </c>
+      <c r="E102" s="16" t="inlineStr">
+        <is>
+          <t>MetricHistoryScreen.js</t>
+        </is>
+      </c>
+      <c r="F102" s="16" t="inlineStr">
+        <is>
+          <t>colors.purple הוא בפועל #f59e0b (כתום), ו-tileScoreColor(null) החזיר אותו — כך שכל תיבות ההסבר במסך הפירוט נראו כאזהרה. אין ציון = אין פסק דין = ניטרלי.</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="26" t="inlineStr">
+        <is>
+          <t>94</t>
+        </is>
+      </c>
+      <c r="B103" s="27" t="inlineStr">
+        <is>
+          <t>הצבע שורד את המעבר בין מסכים</t>
+        </is>
+      </c>
+      <c r="C103" s="26" t="inlineStr">
+        <is>
+          <t>Frontend / Bug Fix</t>
+        </is>
+      </c>
+      <c r="D103" s="28" t="inlineStr">
+        <is>
+          <t>✅ Live (OTA)</t>
+        </is>
+      </c>
+      <c r="E103" s="16" t="inlineStr">
+        <is>
+          <t>StockScreen.js, MetricHistoryScreen.js</t>
+        </is>
+      </c>
+      <c r="F103" s="16" t="inlineStr">
+        <is>
+          <t>P/B 7.81 היה אדום באריח והופך כתום במסך הפירוט, כי המכפילים הנוספים מגיעים בלי ציון. האריח מעביר עכשיו tileSignal.</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="26" t="inlineStr">
+        <is>
+          <t>95</t>
+        </is>
+      </c>
+      <c r="B104" s="27" t="inlineStr">
+        <is>
+          <t>חומת ההסכמה של גוגל — רוסית וספרדית</t>
+        </is>
+      </c>
+      <c r="C104" s="26" t="inlineStr">
+        <is>
+          <t>Frontend / i18n</t>
+        </is>
+      </c>
+      <c r="D104" s="28" t="inlineStr">
+        <is>
+          <t>✅ Live (OTA)</t>
+        </is>
+      </c>
+      <c r="E104" s="16" t="inlineStr">
+        <is>
+          <t>screens/ArticleScreen.js</t>
+        </is>
+      </c>
+      <c r="F104" s="16" t="inlineStr">
+        <is>
+          <t>הסקריפט מזהה את כפתור האישור לפי טקסט, וגוגל מציגה את החומה בשפת המכשיר. נתמכו רק אנגלית ועברית — מכשיר ברוסית/ספרדית נתקע על מסך ההסכמה במקום להגיע לכתבה. נוספו принять/согласен/принимаю ו-aceptar/acepto/de acuerdo, אומת על 11 וריאציות.</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="26" t="inlineStr">
+        <is>
+          <t>96</t>
+        </is>
+      </c>
+      <c r="B105" s="27" t="inlineStr">
+        <is>
+          <t>ביקורת כיסוי-שפות לכל השינויים</t>
+        </is>
+      </c>
+      <c r="C105" s="26" t="inlineStr">
+        <is>
+          <t>QA / i18n</t>
+        </is>
+      </c>
+      <c r="D105" s="28" t="inlineStr">
+        <is>
+          <t>✅ הושלם</t>
+        </is>
+      </c>
+      <c r="E105" s="16" t="inlineStr">
+        <is>
+          <t>כל הקבצים</t>
+        </is>
+      </c>
+      <c r="F105" s="16" t="inlineStr">
+        <is>
+          <t>כל שינוי בהפעלה סווג: תלוי-שפה נבדק ל-4, לא-תלוי אומת שהוא באמת לא תלוי. חיפוש מחרוזות חד-לשוניות חשף את פריט 95. 29 חבילות בדיקה.</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="30" t="inlineStr">
+        <is>
+          <t>97</t>
+        </is>
+      </c>
+      <c r="B106" s="31" t="inlineStr">
+        <is>
+          <t>מדדים דו-משמעיים — הגרף לא טוען טענה</t>
+        </is>
+      </c>
+      <c r="C106" s="30" t="inlineStr">
+        <is>
+          <t>Frontend / Accuracy</t>
+        </is>
+      </c>
+      <c r="D106" s="32" t="inlineStr">
+        <is>
+          <t>✅ Live (OTA)</t>
+        </is>
+      </c>
+      <c r="E106" s="16" t="inlineStr">
+        <is>
+          <t>PriceChart.js, MetricHistoryScreen.js</t>
+        </is>
+      </c>
+      <c r="F106" s="16" t="inlineStr">
+        <is>
+          <t>תשואת דיבידנד/רכישה חוזרת יורדת גם כשהתשלום נחתך (רע) וגם כשהמחיר עולה מהר יותר (טוב). וולמארט העלתה דיבידנד 52 שנה ברציפות והתשואה ירדה 3.2%→0.9% — הגרף צבע את זה אדום. מהתשואה לבדה אי אפשר להבחין, אז הקו כחול = מידע ולא פסק דין.</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="3" t="inlineStr">
+        <is>
+          <t>🔜  NOT YET STARTED</t>
+        </is>
+      </c>
+      <c r="B107" s="5" t="inlineStr"/>
+      <c r="C107" s="4" t="inlineStr"/>
+      <c r="D107" s="4" t="inlineStr"/>
+      <c r="E107" s="4" t="inlineStr"/>
+      <c r="F107" s="5" t="inlineStr"/>
+    </row>
+    <row r="108">
+      <c r="A108" s="6" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="B108" s="4" t="n"/>
+      <c r="C108" s="4" t="n"/>
+      <c r="D108" s="4" t="n"/>
+      <c r="E108" s="4" t="n"/>
+      <c r="F108" s="5" t="n"/>
+    </row>
+    <row r="109">
+      <c r="A109" s="10" t="inlineStr">
+        <is>
+          <t>Legend</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="6" t="inlineStr">
+        <is>
+          <t>✅ Live</t>
+        </is>
+      </c>
+      <c r="B110" s="7" t="inlineStr">
+        <is>
+          <t>פרוס ופעיל ב-Render — נראה לכל המשתמשים</t>
+        </is>
+      </c>
+      <c r="C110" s="6" t="inlineStr"/>
+      <c r="D110" s="8" t="inlineStr"/>
+      <c r="E110" s="9" t="inlineStr"/>
+      <c r="F110" s="9" t="inlineStr"/>
+    </row>
+    <row r="111">
+      <c r="A111" s="6" t="inlineStr">
+        <is>
+          <t>✅ In APK</t>
+        </is>
+      </c>
+      <c r="B111" s="7" t="inlineStr">
+        <is>
+          <t>כלול ב-APK המותקן — נראה לכל המשתמשים</t>
+        </is>
+      </c>
+      <c r="C111" s="6" t="inlineStr"/>
+      <c r="D111" s="8" t="inlineStr"/>
+      <c r="E111" s="9" t="inlineStr"/>
+      <c r="F111" s="9" t="inlineStr"/>
+    </row>
+    <row r="112">
+      <c r="A112" s="6" t="inlineStr">
+        <is>
+          <t>⏳ Next APK</t>
+        </is>
+      </c>
+      <c r="B112" s="7" t="inlineStr">
+        <is>
+          <t>הקוד מוזג — דורש build ו-APK חדש</t>
+        </is>
+      </c>
+      <c r="C112" s="6" t="inlineStr"/>
+      <c r="D112" s="8" t="inlineStr"/>
+      <c r="E112" s="9" t="inlineStr"/>
+      <c r="F112" s="9" t="inlineStr"/>
+    </row>
+    <row r="113">
+      <c r="A113" s="6" t="inlineStr">
+        <is>
+          <t>✅ Live (OTA)</t>
+        </is>
+      </c>
+      <c r="B113" s="7" t="inlineStr">
+        <is>
+          <t>שינוי JS — מועבר אוטומטית בהפעלה הבאה</t>
+        </is>
+      </c>
+      <c r="C113" s="6" t="inlineStr"/>
+      <c r="D113" s="8" t="inlineStr"/>
+      <c r="E113" s="9" t="inlineStr"/>
+      <c r="F113" s="9" t="inlineStr"/>
+    </row>
+    <row r="114">
+      <c r="A114" s="21" t="inlineStr">
         <is>
           <t>⏳ ממתין ל-push</t>
         </is>
       </c>
-      <c r="E91" s="20" t="inlineStr">
-        <is>
-          <t>main.py</t>
-        </is>
-      </c>
-      <c r="F91" s="20" t="inlineStr">
-        <is>
-          <t>הסיבה האמיתית שדלק חזרה: OkHttp של אנדרואיד שמר תשובה שנוצרה בגרסת קוד ישנה. הוכח — אותה מניה ב-en החזירה 8173 וב-ru החזירה 84.45.</t>
-        </is>
-      </c>
-    </row>
-    <row r="92">
-      <c r="A92" s="17" t="inlineStr">
-        <is>
-          <t>84</t>
-        </is>
-      </c>
-      <c r="B92" s="18" t="inlineStr">
-        <is>
-          <t>סדרה שנתית = סוף שנה, לא ינואר</t>
-        </is>
-      </c>
-      <c r="C92" s="17" t="inlineStr">
-        <is>
-          <t>Backend / Bug Fix</t>
-        </is>
-      </c>
-      <c r="D92" s="19" t="inlineStr">
-        <is>
-          <t>⏳ ממתין ל-push</t>
-        </is>
-      </c>
-      <c r="E92" s="20" t="inlineStr">
-        <is>
-          <t>main.py</t>
-        </is>
-      </c>
-      <c r="F92" s="20" t="inlineStr">
-        <is>
-          <t>הגרף השנתי הציג את ינואר בתווית של השנה. KO 2023: הוצג 25.25 במקום 22.19 — סטייה 12%. תוקן ב-4 מקומות.</t>
-        </is>
-      </c>
-    </row>
-    <row r="93">
-      <c r="A93" s="17" t="inlineStr">
-        <is>
-          <t>85</t>
-        </is>
-      </c>
-      <c r="B93" s="18" t="inlineStr">
-        <is>
-          <t>TTM של Buyback דרש 2 רבעונים</t>
-        </is>
-      </c>
-      <c r="C93" s="17" t="inlineStr">
-        <is>
-          <t>Backend / Bug Fix</t>
-        </is>
-      </c>
-      <c r="D93" s="19" t="inlineStr">
-        <is>
-          <t>⏳ ממתין ל-push</t>
-        </is>
-      </c>
-      <c r="E93" s="20" t="inlineStr">
-        <is>
-          <t>main.py</t>
-        </is>
-      </c>
-      <c r="F93" s="20" t="inlineStr">
-        <is>
-          <t>"תשואה שנתית" יכלה להיות סכום של חצי שנה. הועלה ל-4 כמו כל שאר חישובי ה-TTM.</t>
-        </is>
-      </c>
-    </row>
-    <row r="94">
-      <c r="A94" s="13" t="inlineStr">
-        <is>
-          <t>86</t>
-        </is>
-      </c>
-      <c r="B94" s="14" t="inlineStr">
-        <is>
-          <t>ניקוי ריפו — cloudflared.exe 52MB</t>
-        </is>
-      </c>
-      <c r="C94" s="13" t="inlineStr">
-        <is>
-          <t>DevOps</t>
-        </is>
-      </c>
-      <c r="D94" s="15" t="inlineStr">
-        <is>
-          <t>✅ Live</t>
-        </is>
-      </c>
-      <c r="E94" s="16" t="inlineStr">
-        <is>
-          <t>‎.gitignore</t>
-        </is>
-      </c>
-      <c r="F94" s="16" t="inlineStr">
-        <is>
-          <t>יצא ממעקב git, נשאר על הדיסק המקומי.</t>
-        </is>
-      </c>
-    </row>
-    <row r="95">
-      <c r="A95" s="13" t="inlineStr">
-        <is>
-          <t>87</t>
-        </is>
-      </c>
-      <c r="B95" s="14" t="inlineStr">
-        <is>
-          <t>דיוק עמוד הפרטיות בנוגע ללוגים</t>
-        </is>
-      </c>
-      <c r="C95" s="13" t="inlineStr">
-        <is>
-          <t>Legal</t>
-        </is>
-      </c>
-      <c r="D95" s="15" t="inlineStr">
-        <is>
-          <t>✅ Live</t>
-        </is>
-      </c>
-      <c r="E95" s="16" t="inlineStr">
-        <is>
-          <t>main.py</t>
-        </is>
-      </c>
-      <c r="F95" s="16" t="inlineStr">
-        <is>
-          <t>ההצהרה "איננו רושמים כתובות IP" לא היתה מדויקת — uvicorn ו-Render כן שומרים לוגים טכניים. נוסח מחדש.</t>
-        </is>
-      </c>
-    </row>
-    <row r="96">
-      <c r="A96" s="13" t="inlineStr">
-        <is>
-          <t>88</t>
-        </is>
-      </c>
-      <c r="B96" s="14" t="inlineStr">
-        <is>
-          <t>ביקורת קוד מלאה — 35 קבצים</t>
-        </is>
-      </c>
-      <c r="C96" s="13" t="inlineStr">
-        <is>
-          <t>QA</t>
-        </is>
-      </c>
-      <c r="D96" s="15" t="inlineStr">
-        <is>
-          <t>✅ הושלם</t>
-        </is>
-      </c>
-      <c r="E96" s="16" t="inlineStr">
-        <is>
-          <t>כל הקבצים</t>
-        </is>
-      </c>
-      <c r="F96" s="16" t="inlineStr">
-        <is>
-          <t>11,646 שורות נקראו במלואן. 27 חבילות בדיקה התנהגותיות. אימות חי מול ה-API בייצור (זה מה שחשף פריטים 83-85).</t>
-        </is>
-      </c>
-    </row>
-    <row r="97">
-      <c r="A97" s="3" t="inlineStr">
-        <is>
-          <t>🔜  NOT YET STARTED</t>
-        </is>
-      </c>
-      <c r="B97" s="5" t="inlineStr"/>
-      <c r="C97" s="4" t="inlineStr"/>
-      <c r="D97" s="4" t="inlineStr"/>
-      <c r="E97" s="4" t="inlineStr"/>
-      <c r="F97" s="5" t="inlineStr"/>
-    </row>
-    <row r="98">
-      <c r="A98" s="6" t="inlineStr">
-        <is>
-          <t>19</t>
-        </is>
-      </c>
-      <c r="B98" s="7" t="inlineStr">
-        <is>
-          <t>Google Play Console — הגשה לחנות</t>
-        </is>
-      </c>
-      <c r="C98" s="6" t="inlineStr">
-        <is>
-          <t>Distribution</t>
-        </is>
-      </c>
-      <c r="D98" s="8" t="inlineStr">
-        <is>
-          <t>🔜</t>
-        </is>
-      </c>
-      <c r="E98" s="9" t="inlineStr"/>
-      <c r="F98" s="9" t="inlineStr">
-        <is>
-          <t>חשבון מפתח ($25) + העלאת AAB + store listing + screenshots.</t>
-        </is>
-      </c>
-    </row>
-    <row r="99">
-      <c r="A99" s="10" t="inlineStr">
-        <is>
-          <t>Legend</t>
-        </is>
-      </c>
-    </row>
-    <row r="100">
-      <c r="A100" s="6" t="inlineStr">
-        <is>
-          <t>✅ Live</t>
-        </is>
-      </c>
-      <c r="B100" s="7" t="inlineStr">
-        <is>
-          <t>פרוס ופעיל ב-Render — נראה לכל המשתמשים</t>
-        </is>
-      </c>
-      <c r="C100" s="6" t="inlineStr"/>
-      <c r="D100" s="8" t="inlineStr"/>
-      <c r="E100" s="9" t="inlineStr"/>
-      <c r="F100" s="9" t="inlineStr"/>
-    </row>
-    <row r="101">
-      <c r="A101" s="6" t="inlineStr">
-        <is>
-          <t>✅ In APK</t>
-        </is>
-      </c>
-      <c r="B101" s="7" t="inlineStr">
-        <is>
-          <t>כלול ב-APK המותקן — נראה לכל המשתמשים</t>
-        </is>
-      </c>
-      <c r="C101" s="6" t="inlineStr"/>
-      <c r="D101" s="8" t="inlineStr"/>
-      <c r="E101" s="9" t="inlineStr"/>
-      <c r="F101" s="9" t="inlineStr"/>
-    </row>
-    <row r="102">
-      <c r="A102" s="6" t="inlineStr">
-        <is>
-          <t>⏳ Next APK</t>
-        </is>
-      </c>
-      <c r="B102" s="7" t="inlineStr">
-        <is>
-          <t>הקוד מוזג — דורש build ו-APK חדש</t>
-        </is>
-      </c>
-      <c r="C102" s="6" t="inlineStr"/>
-      <c r="D102" s="8" t="inlineStr"/>
-      <c r="E102" s="9" t="inlineStr"/>
-      <c r="F102" s="9" t="inlineStr"/>
-    </row>
-    <row r="103">
-      <c r="A103" s="6" t="inlineStr">
-        <is>
-          <t>✅ Live (OTA)</t>
-        </is>
-      </c>
-      <c r="B103" s="7" t="inlineStr">
-        <is>
-          <t>שינוי JS — מועבר אוטומטית בהפעלה הבאה</t>
-        </is>
-      </c>
-      <c r="C103" s="6" t="inlineStr"/>
-      <c r="D103" s="8" t="inlineStr"/>
-      <c r="E103" s="9" t="inlineStr"/>
-      <c r="F103" s="9" t="inlineStr"/>
-    </row>
-    <row r="104">
-      <c r="A104" s="21" t="inlineStr">
-        <is>
-          <t>⏳ ממתין ל-push</t>
-        </is>
-      </c>
-      <c r="B104" s="22" t="inlineStr">
+      <c r="B114" s="22" t="inlineStr">
         <is>
           <t>הקוד מוכן מקומית — טרם נדחף/נפרס</t>
         </is>
       </c>
     </row>
-    <row r="105">
-      <c r="A105" s="21" t="inlineStr">
+    <row r="115">
+      <c r="A115" s="21" t="inlineStr">
         <is>
           <t>⏳ דורש build</t>
         </is>
       </c>
-      <c r="B105" s="22" t="inlineStr">
+      <c r="B115" s="22" t="inlineStr">
         <is>
           <t>שינוי נייטיב — OTA לא מספיק, צריך AAB/APK חדש</t>
         </is>
       </c>
     </row>
-    <row r="107">
-      <c r="A107" s="23" t="inlineStr">
-        <is>
-          <t>סיכום Session 6</t>
-        </is>
-      </c>
-    </row>
-    <row r="108">
-      <c r="A108" s="24" t="n"/>
-      <c r="B108" s="25" t="inlineStr">
-        <is>
-          <t>37  —  פריטים חדשים שנוספו (52-88)</t>
-        </is>
-      </c>
-    </row>
-    <row r="109">
-      <c r="A109" s="24" t="n"/>
-      <c r="B109" s="25" t="inlineStr">
-        <is>
-          <t>32  —  כבר חיים בייצור או ב-OTA</t>
-        </is>
-      </c>
-    </row>
-    <row r="110">
-      <c r="A110" s="24" t="n"/>
-      <c r="B110" s="25" t="inlineStr">
-        <is>
-          <t>3  —  ממתינים ל-push: no-store, סדרה שנתית, TTM של buyback</t>
-        </is>
-      </c>
-    </row>
-    <row r="111">
-      <c r="A111" s="24" t="n"/>
-      <c r="B111" s="25" t="inlineStr">
-        <is>
-          <t>1  —  דורש build חדש: תמיכת טאבלט</t>
-        </is>
-      </c>
-    </row>
-    <row r="112">
-      <c r="A112" s="24" t="n"/>
-      <c r="B112" s="25" t="inlineStr">
-        <is>
-          <t>11,646  —  שורות קוד שנקראו במלואן, 35 קבצים</t>
-        </is>
-      </c>
-    </row>
-    <row r="113">
-      <c r="A113" s="24" t="n"/>
-      <c r="B113" s="25" t="inlineStr">
-        <is>
-          <t>27  —  חבילות בדיקה התנהגותיות עוברות</t>
+    <row r="116"/>
+    <row r="117">
+      <c r="A117" s="23" t="inlineStr">
+        <is>
+          <t>סיכום Session 6-7</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="24" t="n"/>
+      <c r="B118" s="25" t="inlineStr">
+        <is>
+          <t>45  —  פריטים חדשים שנוספו (52-96)</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="24" t="n"/>
+      <c r="B119" s="25" t="inlineStr">
+        <is>
+          <t>44  —  חיים בייצור או ב-OTA</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="24" t="n"/>
+      <c r="B120" s="25" t="inlineStr">
+        <is>
+          <t>1  —  דורש build חדש: תמיכת טאבלט (פריט 68)</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="24" t="n"/>
+      <c r="B121" s="25" t="inlineStr">
+        <is>
+          <t>11,781  —  שורות קוד שנקראו במלואן, 36 קבצים</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="24" t="n"/>
+      <c r="B122" s="25" t="inlineStr">
+        <is>
+          <t>29  —  חבילות בדיקה התנהגותיות עוברות</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="24" t="n"/>
+      <c r="B123" s="25" t="inlineStr">
+        <is>
+          <t>18  —  ראוטים בשרת · 316 מפתחות i18n × 4 שפות</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="4">
+    <mergeCell ref="A97:F97"/>
     <mergeCell ref="A107:F107"/>
     <mergeCell ref="A59:F59"/>
     <mergeCell ref="A25:F25"/>

</xml_diff>

<commit_message>
Chart colour is the tile verdict, not the trend - P/B 6.84 is red on both screens
</commit_message>
<xml_diff>
--- a/BuddhaVest_Progress.xlsx
+++ b/BuddhaVest_Progress.xlsx
@@ -175,7 +175,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -250,6 +250,15 @@
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
@@ -624,7 +633,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F123"/>
+  <dimension ref="A1:F124"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2335,22 +2344,22 @@
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="26" t="inlineStr">
+      <c r="A60" s="30" t="inlineStr">
         <is>
           <t>52</t>
         </is>
       </c>
-      <c r="B60" s="27" t="inlineStr">
+      <c r="B60" s="31" t="inlineStr">
         <is>
           <t>מרוץ שפות — 5 מסכים/רכיבים</t>
         </is>
       </c>
-      <c r="C60" s="26" t="inlineStr">
+      <c r="C60" s="30" t="inlineStr">
         <is>
           <t>Frontend / Bug Fix</t>
         </is>
       </c>
-      <c r="D60" s="28" t="inlineStr">
+      <c r="D60" s="32" t="inlineStr">
         <is>
           <t>✅ Live (OTA)</t>
         </is>
@@ -2367,22 +2376,22 @@
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="26" t="inlineStr">
+      <c r="A61" s="30" t="inlineStr">
         <is>
           <t>53</t>
         </is>
       </c>
-      <c r="B61" s="27" t="inlineStr">
+      <c r="B61" s="31" t="inlineStr">
         <is>
           <t>Volume/Avg Vol ריקים לסירוגין</t>
         </is>
       </c>
-      <c r="C61" s="26" t="inlineStr">
+      <c r="C61" s="30" t="inlineStr">
         <is>
           <t>Backend / Bug Fix</t>
         </is>
       </c>
-      <c r="D61" s="28" t="inlineStr">
+      <c r="D61" s="32" t="inlineStr">
         <is>
           <t>✅ Live</t>
         </is>
@@ -2399,22 +2408,22 @@
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="26" t="inlineStr">
+      <c r="A62" s="30" t="inlineStr">
         <is>
           <t>54</t>
         </is>
       </c>
-      <c r="B62" s="27" t="inlineStr">
+      <c r="B62" s="31" t="inlineStr">
         <is>
           <t>המרת אגורות→שקל למניות ת"א</t>
         </is>
       </c>
-      <c r="C62" s="26" t="inlineStr">
+      <c r="C62" s="30" t="inlineStr">
         <is>
           <t>Backend</t>
         </is>
       </c>
-      <c r="D62" s="28" t="inlineStr">
+      <c r="D62" s="32" t="inlineStr">
         <is>
           <t>✅ Live</t>
         </is>
@@ -2431,22 +2440,22 @@
       </c>
     </row>
     <row r="63">
-      <c r="A63" s="26" t="inlineStr">
+      <c r="A63" s="30" t="inlineStr">
         <is>
           <t>55</t>
         </is>
       </c>
-      <c r="B63" s="27" t="inlineStr">
+      <c r="B63" s="31" t="inlineStr">
         <is>
           <t>באג יחידות ב-Buyback (3500000000%)</t>
         </is>
       </c>
-      <c r="C63" s="26" t="inlineStr">
+      <c r="C63" s="30" t="inlineStr">
         <is>
           <t>Backend + Frontend</t>
         </is>
       </c>
-      <c r="D63" s="28" t="inlineStr">
+      <c r="D63" s="32" t="inlineStr">
         <is>
           <t>✅ Live</t>
         </is>
@@ -2463,22 +2472,22 @@
       </c>
     </row>
     <row r="64">
-      <c r="A64" s="26" t="inlineStr">
+      <c r="A64" s="30" t="inlineStr">
         <is>
           <t>56</t>
         </is>
       </c>
-      <c r="B64" s="27" t="inlineStr">
+      <c r="B64" s="31" t="inlineStr">
         <is>
           <t>תיקוני נכונות במנוע הציון</t>
         </is>
       </c>
-      <c r="C64" s="26" t="inlineStr">
+      <c r="C64" s="30" t="inlineStr">
         <is>
           <t>Backend / Scoring</t>
         </is>
       </c>
-      <c r="D64" s="28" t="inlineStr">
+      <c r="D64" s="32" t="inlineStr">
         <is>
           <t>✅ Live</t>
         </is>
@@ -2495,22 +2504,22 @@
       </c>
     </row>
     <row r="65">
-      <c r="A65" s="26" t="inlineStr">
+      <c r="A65" s="30" t="inlineStr">
         <is>
           <t>57</t>
         </is>
       </c>
-      <c r="B65" s="27" t="inlineStr">
+      <c r="B65" s="31" t="inlineStr">
         <is>
           <t>ניסוח דיבידנד כן — לא "משולם בעקביות"</t>
         </is>
       </c>
-      <c r="C65" s="26" t="inlineStr">
+      <c r="C65" s="30" t="inlineStr">
         <is>
           <t>Legal / Accuracy</t>
         </is>
       </c>
-      <c r="D65" s="28" t="inlineStr">
+      <c r="D65" s="32" t="inlineStr">
         <is>
           <t>✅ Live</t>
         </is>
@@ -2527,22 +2536,22 @@
       </c>
     </row>
     <row r="66">
-      <c r="A66" s="26" t="inlineStr">
+      <c r="A66" s="30" t="inlineStr">
         <is>
           <t>58</t>
         </is>
       </c>
-      <c r="B66" s="27" t="inlineStr">
+      <c r="B66" s="31" t="inlineStr">
         <is>
           <t>SSRF — /translate-article</t>
         </is>
       </c>
-      <c r="C66" s="26" t="inlineStr">
+      <c r="C66" s="30" t="inlineStr">
         <is>
           <t>Backend / Security</t>
         </is>
       </c>
-      <c r="D66" s="28" t="inlineStr">
+      <c r="D66" s="32" t="inlineStr">
         <is>
           <t>✅ Live</t>
         </is>
@@ -2559,22 +2568,22 @@
       </c>
     </row>
     <row r="67">
-      <c r="A67" s="26" t="inlineStr">
+      <c r="A67" s="30" t="inlineStr">
         <is>
           <t>59</t>
         </is>
       </c>
-      <c r="B67" s="27" t="inlineStr">
+      <c r="B67" s="31" t="inlineStr">
         <is>
           <t>XSS ב-WebView של הכתבות</t>
         </is>
       </c>
-      <c r="C67" s="26" t="inlineStr">
+      <c r="C67" s="30" t="inlineStr">
         <is>
           <t>Frontend / Security</t>
         </is>
       </c>
-      <c r="D67" s="28" t="inlineStr">
+      <c r="D67" s="32" t="inlineStr">
         <is>
           <t>✅ Live (OTA)</t>
         </is>
@@ -2591,22 +2600,22 @@
       </c>
     </row>
     <row r="68">
-      <c r="A68" s="26" t="inlineStr">
+      <c r="A68" s="30" t="inlineStr">
         <is>
           <t>60</t>
         </is>
       </c>
-      <c r="B68" s="27" t="inlineStr">
+      <c r="B68" s="31" t="inlineStr">
         <is>
           <t>הסרת /debug-pe ו-/debug-rows</t>
         </is>
       </c>
-      <c r="C68" s="26" t="inlineStr">
+      <c r="C68" s="30" t="inlineStr">
         <is>
           <t>Backend / Security</t>
         </is>
       </c>
-      <c r="D68" s="28" t="inlineStr">
+      <c r="D68" s="32" t="inlineStr">
         <is>
           <t>✅ Live</t>
         </is>
@@ -2623,22 +2632,22 @@
       </c>
     </row>
     <row r="69">
-      <c r="A69" s="26" t="inlineStr">
+      <c r="A69" s="30" t="inlineStr">
         <is>
           <t>61</t>
         </is>
       </c>
-      <c r="B69" s="27" t="inlineStr">
+      <c r="B69" s="31" t="inlineStr">
         <is>
           <t>5 דליפות של פרטי חריגה ללקוח</t>
         </is>
       </c>
-      <c r="C69" s="26" t="inlineStr">
+      <c r="C69" s="30" t="inlineStr">
         <is>
           <t>Backend / Security</t>
         </is>
       </c>
-      <c r="D69" s="28" t="inlineStr">
+      <c r="D69" s="32" t="inlineStr">
         <is>
           <t>✅ Live</t>
         </is>
@@ -2655,22 +2664,22 @@
       </c>
     </row>
     <row r="70">
-      <c r="A70" s="26" t="inlineStr">
+      <c r="A70" s="30" t="inlineStr">
         <is>
           <t>62</t>
         </is>
       </c>
-      <c r="B70" s="27" t="inlineStr">
+      <c r="B70" s="31" t="inlineStr">
         <is>
           <t>פיצוץ זיכרון בעליית השרת</t>
         </is>
       </c>
-      <c r="C70" s="26" t="inlineStr">
+      <c r="C70" s="30" t="inlineStr">
         <is>
           <t>Backend / Performance</t>
         </is>
       </c>
-      <c r="D70" s="28" t="inlineStr">
+      <c r="D70" s="32" t="inlineStr">
         <is>
           <t>✅ Live</t>
         </is>
@@ -2687,22 +2696,22 @@
       </c>
     </row>
     <row r="71">
-      <c r="A71" s="26" t="inlineStr">
+      <c r="A71" s="30" t="inlineStr">
         <is>
           <t>63</t>
         </is>
       </c>
-      <c r="B71" s="27" t="inlineStr">
+      <c r="B71" s="31" t="inlineStr">
         <is>
           <t>תקרת מטמון + single-flight</t>
         </is>
       </c>
-      <c r="C71" s="26" t="inlineStr">
+      <c r="C71" s="30" t="inlineStr">
         <is>
           <t>Backend / Performance</t>
         </is>
       </c>
-      <c r="D71" s="28" t="inlineStr">
+      <c r="D71" s="32" t="inlineStr">
         <is>
           <t>✅ Live</t>
         </is>
@@ -2719,22 +2728,22 @@
       </c>
     </row>
     <row r="72">
-      <c r="A72" s="26" t="inlineStr">
+      <c r="A72" s="30" t="inlineStr">
         <is>
           <t>64</t>
         </is>
       </c>
-      <c r="B72" s="27" t="inlineStr">
+      <c r="B72" s="31" t="inlineStr">
         <is>
           <t>חלון היסטוריה 10y במקום max</t>
         </is>
       </c>
-      <c r="C72" s="26" t="inlineStr">
+      <c r="C72" s="30" t="inlineStr">
         <is>
           <t>Backend / Performance</t>
         </is>
       </c>
-      <c r="D72" s="28" t="inlineStr">
+      <c r="D72" s="32" t="inlineStr">
         <is>
           <t>✅ Live</t>
         </is>
@@ -2751,22 +2760,22 @@
       </c>
     </row>
     <row r="73">
-      <c r="A73" s="26" t="inlineStr">
+      <c r="A73" s="30" t="inlineStr">
         <is>
           <t>65</t>
         </is>
       </c>
-      <c r="B73" s="27" t="inlineStr">
+      <c r="B73" s="31" t="inlineStr">
         <is>
           <t>Debounce בחיפוש</t>
         </is>
       </c>
-      <c r="C73" s="26" t="inlineStr">
+      <c r="C73" s="30" t="inlineStr">
         <is>
           <t>Frontend / Performance</t>
         </is>
       </c>
-      <c r="D73" s="28" t="inlineStr">
+      <c r="D73" s="32" t="inlineStr">
         <is>
           <t>✅ Live (OTA)</t>
         </is>
@@ -2783,22 +2792,22 @@
       </c>
     </row>
     <row r="74">
-      <c r="A74" s="26" t="inlineStr">
+      <c r="A74" s="30" t="inlineStr">
         <is>
           <t>66</t>
         </is>
       </c>
-      <c r="B74" s="27" t="inlineStr">
+      <c r="B74" s="31" t="inlineStr">
         <is>
           <t>תקציב זמן ל-Stooq</t>
         </is>
       </c>
-      <c r="C74" s="26" t="inlineStr">
+      <c r="C74" s="30" t="inlineStr">
         <is>
           <t>Backend / Performance</t>
         </is>
       </c>
-      <c r="D74" s="28" t="inlineStr">
+      <c r="D74" s="32" t="inlineStr">
         <is>
           <t>✅ Live</t>
         </is>
@@ -2815,22 +2824,22 @@
       </c>
     </row>
     <row r="75">
-      <c r="A75" s="26" t="inlineStr">
+      <c r="A75" s="30" t="inlineStr">
         <is>
           <t>67</t>
         </is>
       </c>
-      <c r="B75" s="27" t="inlineStr">
+      <c r="B75" s="31" t="inlineStr">
         <is>
           <t>אובדן נתונים ביומן המחקר</t>
         </is>
       </c>
-      <c r="C75" s="26" t="inlineStr">
+      <c r="C75" s="30" t="inlineStr">
         <is>
           <t>Frontend / Bug Fix</t>
         </is>
       </c>
-      <c r="D75" s="28" t="inlineStr">
+      <c r="D75" s="32" t="inlineStr">
         <is>
           <t>✅ Live (OTA)</t>
         </is>
@@ -2879,22 +2888,22 @@
       </c>
     </row>
     <row r="77">
-      <c r="A77" s="26" t="inlineStr">
+      <c r="A77" s="30" t="inlineStr">
         <is>
           <t>69</t>
         </is>
       </c>
-      <c r="B77" s="27" t="inlineStr">
+      <c r="B77" s="31" t="inlineStr">
         <is>
           <t>מסך הסכמה בהפעלה ראשונה</t>
         </is>
       </c>
-      <c r="C77" s="26" t="inlineStr">
+      <c r="C77" s="30" t="inlineStr">
         <is>
           <t>Legal</t>
         </is>
       </c>
-      <c r="D77" s="28" t="inlineStr">
+      <c r="D77" s="32" t="inlineStr">
         <is>
           <t>✅ Live (OTA)</t>
         </is>
@@ -2911,22 +2920,22 @@
       </c>
     </row>
     <row r="78">
-      <c r="A78" s="26" t="inlineStr">
+      <c r="A78" s="30" t="inlineStr">
         <is>
           <t>70</t>
         </is>
       </c>
-      <c r="B78" s="27" t="inlineStr">
+      <c r="B78" s="31" t="inlineStr">
         <is>
           <t>שכתוב תיאור החנות — בלי הבטחות</t>
         </is>
       </c>
-      <c r="C78" s="26" t="inlineStr">
+      <c r="C78" s="30" t="inlineStr">
         <is>
           <t>Legal / Store</t>
         </is>
       </c>
-      <c r="D78" s="28" t="inlineStr">
+      <c r="D78" s="32" t="inlineStr">
         <is>
           <t>✅ מוכן</t>
         </is>
@@ -2943,22 +2952,22 @@
       </c>
     </row>
     <row r="79">
-      <c r="A79" s="26" t="inlineStr">
+      <c r="A79" s="30" t="inlineStr">
         <is>
           <t>71</t>
         </is>
       </c>
-      <c r="B79" s="27" t="inlineStr">
+      <c r="B79" s="31" t="inlineStr">
         <is>
           <t>מדריך צילומי מסך לחנות</t>
         </is>
       </c>
-      <c r="C79" s="26" t="inlineStr">
+      <c r="C79" s="30" t="inlineStr">
         <is>
           <t>Store Assets</t>
         </is>
       </c>
-      <c r="D79" s="28" t="inlineStr">
+      <c r="D79" s="32" t="inlineStr">
         <is>
           <t>✅ הושלם</t>
         </is>
@@ -2975,22 +2984,22 @@
       </c>
     </row>
     <row r="80">
-      <c r="A80" s="26" t="inlineStr">
+      <c r="A80" s="30" t="inlineStr">
         <is>
           <t>72</t>
         </is>
       </c>
-      <c r="B80" s="27" t="inlineStr">
+      <c r="B80" s="31" t="inlineStr">
         <is>
           <t>RTL בכל המסכים</t>
         </is>
       </c>
-      <c r="C80" s="26" t="inlineStr">
+      <c r="C80" s="30" t="inlineStr">
         <is>
           <t>Frontend / i18n</t>
         </is>
       </c>
-      <c r="D80" s="28" t="inlineStr">
+      <c r="D80" s="32" t="inlineStr">
         <is>
           <t>✅ Live (OTA)</t>
         </is>
@@ -3007,22 +3016,22 @@
       </c>
     </row>
     <row r="81">
-      <c r="A81" s="26" t="inlineStr">
+      <c r="A81" s="30" t="inlineStr">
         <is>
           <t>73</t>
         </is>
       </c>
-      <c r="B81" s="27" t="inlineStr">
+      <c r="B81" s="31" t="inlineStr">
         <is>
           <t>תווית גרסה מ-app.json</t>
         </is>
       </c>
-      <c r="C81" s="26" t="inlineStr">
+      <c r="C81" s="30" t="inlineStr">
         <is>
           <t>Frontend</t>
         </is>
       </c>
-      <c r="D81" s="28" t="inlineStr">
+      <c r="D81" s="32" t="inlineStr">
         <is>
           <t>✅ Live (OTA)</t>
         </is>
@@ -3039,22 +3048,22 @@
       </c>
     </row>
     <row r="82">
-      <c r="A82" s="26" t="inlineStr">
+      <c r="A82" s="30" t="inlineStr">
         <is>
           <t>74</t>
         </is>
       </c>
-      <c r="B82" s="27" t="inlineStr">
+      <c r="B82" s="31" t="inlineStr">
         <is>
           <t>טעינה דו-שלבית ברשימת המעקב</t>
         </is>
       </c>
-      <c r="C82" s="26" t="inlineStr">
+      <c r="C82" s="30" t="inlineStr">
         <is>
           <t>Frontend / Performance</t>
         </is>
       </c>
-      <c r="D82" s="28" t="inlineStr">
+      <c r="D82" s="32" t="inlineStr">
         <is>
           <t>✅ Live (OTA)</t>
         </is>
@@ -3071,22 +3080,22 @@
       </c>
     </row>
     <row r="83">
-      <c r="A83" s="26" t="inlineStr">
+      <c r="A83" s="30" t="inlineStr">
         <is>
           <t>75</t>
         </is>
       </c>
-      <c r="B83" s="27" t="inlineStr">
+      <c r="B83" s="31" t="inlineStr">
         <is>
           <t>/quotes: אגורות, שם חברה, מטבע</t>
         </is>
       </c>
-      <c r="C83" s="26" t="inlineStr">
+      <c r="C83" s="30" t="inlineStr">
         <is>
           <t>Backend</t>
         </is>
       </c>
-      <c r="D83" s="28" t="inlineStr">
+      <c r="D83" s="32" t="inlineStr">
         <is>
           <t>✅ Live</t>
         </is>
@@ -3103,22 +3112,22 @@
       </c>
     </row>
     <row r="84">
-      <c r="A84" s="26" t="inlineStr">
+      <c r="A84" s="30" t="inlineStr">
         <is>
           <t>76</t>
         </is>
       </c>
-      <c r="B84" s="27" t="inlineStr">
+      <c r="B84" s="31" t="inlineStr">
         <is>
           <t>מיזוג במקום החלפה ברשימת המעקב</t>
         </is>
       </c>
-      <c r="C84" s="26" t="inlineStr">
+      <c r="C84" s="30" t="inlineStr">
         <is>
           <t>Frontend / Bug Fix</t>
         </is>
       </c>
-      <c r="D84" s="28" t="inlineStr">
+      <c r="D84" s="32" t="inlineStr">
         <is>
           <t>✅ Live (OTA)</t>
         </is>
@@ -3135,22 +3144,22 @@
       </c>
     </row>
     <row r="85">
-      <c r="A85" s="26" t="inlineStr">
+      <c r="A85" s="30" t="inlineStr">
         <is>
           <t>77</t>
         </is>
       </c>
-      <c r="B85" s="27" t="inlineStr">
+      <c r="B85" s="31" t="inlineStr">
         <is>
           <t>מרוץ במסך הבית — market/FX</t>
         </is>
       </c>
-      <c r="C85" s="26" t="inlineStr">
+      <c r="C85" s="30" t="inlineStr">
         <is>
           <t>Frontend / Bug Fix</t>
         </is>
       </c>
-      <c r="D85" s="28" t="inlineStr">
+      <c r="D85" s="32" t="inlineStr">
         <is>
           <t>✅ Live (OTA)</t>
         </is>
@@ -3167,22 +3176,22 @@
       </c>
     </row>
     <row r="86">
-      <c r="A86" s="26" t="inlineStr">
+      <c r="A86" s="30" t="inlineStr">
         <is>
           <t>78</t>
         </is>
       </c>
-      <c r="B86" s="27" t="inlineStr">
+      <c r="B86" s="31" t="inlineStr">
         <is>
           <t>תשובה ריקה לא מוחקת נתונים טובים</t>
         </is>
       </c>
-      <c r="C86" s="26" t="inlineStr">
+      <c r="C86" s="30" t="inlineStr">
         <is>
           <t>Frontend / Bug Fix</t>
         </is>
       </c>
-      <c r="D86" s="28" t="inlineStr">
+      <c r="D86" s="32" t="inlineStr">
         <is>
           <t>✅ Live (OTA)</t>
         </is>
@@ -3199,22 +3208,22 @@
       </c>
     </row>
     <row r="87">
-      <c r="A87" s="26" t="inlineStr">
+      <c r="A87" s="30" t="inlineStr">
         <is>
           <t>79</t>
         </is>
       </c>
-      <c r="B87" s="27" t="inlineStr">
+      <c r="B87" s="31" t="inlineStr">
         <is>
           <t>תרגום כתבה ישנה דלף לחדשה</t>
         </is>
       </c>
-      <c r="C87" s="26" t="inlineStr">
+      <c r="C87" s="30" t="inlineStr">
         <is>
           <t>Frontend / Bug Fix</t>
         </is>
       </c>
-      <c r="D87" s="28" t="inlineStr">
+      <c r="D87" s="32" t="inlineStr">
         <is>
           <t>✅ Live (OTA)</t>
         </is>
@@ -3231,22 +3240,22 @@
       </c>
     </row>
     <row r="88">
-      <c r="A88" s="26" t="inlineStr">
+      <c r="A88" s="30" t="inlineStr">
         <is>
           <t>80</t>
         </is>
       </c>
-      <c r="B88" s="27" t="inlineStr">
+      <c r="B88" s="31" t="inlineStr">
         <is>
           <t>מרוץ ב"נסה שוב" של פירוט מדד</t>
         </is>
       </c>
-      <c r="C88" s="26" t="inlineStr">
+      <c r="C88" s="30" t="inlineStr">
         <is>
           <t>Frontend / Bug Fix</t>
         </is>
       </c>
-      <c r="D88" s="28" t="inlineStr">
+      <c r="D88" s="32" t="inlineStr">
         <is>
           <t>✅ Live (OTA)</t>
         </is>
@@ -3263,22 +3272,22 @@
       </c>
     </row>
     <row r="89">
-      <c r="A89" s="26" t="inlineStr">
+      <c r="A89" s="30" t="inlineStr">
         <is>
           <t>81</t>
         </is>
       </c>
-      <c r="B89" s="27" t="inlineStr">
+      <c r="B89" s="31" t="inlineStr">
         <is>
           <t>סולם VIX לא מונוטוני</t>
         </is>
       </c>
-      <c r="C89" s="26" t="inlineStr">
+      <c r="C89" s="30" t="inlineStr">
         <is>
           <t>Frontend / i18n</t>
         </is>
       </c>
-      <c r="D89" s="28" t="inlineStr">
+      <c r="D89" s="32" t="inlineStr">
         <is>
           <t>✅ Live (OTA)</t>
         </is>
@@ -3295,22 +3304,22 @@
       </c>
     </row>
     <row r="90">
-      <c r="A90" s="26" t="inlineStr">
+      <c r="A90" s="30" t="inlineStr">
         <is>
           <t>82</t>
         </is>
       </c>
-      <c r="B90" s="27" t="inlineStr">
+      <c r="B90" s="31" t="inlineStr">
         <is>
           <t>תיקוני תוכן בספרדית</t>
         </is>
       </c>
-      <c r="C90" s="26" t="inlineStr">
+      <c r="C90" s="30" t="inlineStr">
         <is>
           <t>i18n / Accuracy</t>
         </is>
       </c>
-      <c r="D90" s="28" t="inlineStr">
+      <c r="D90" s="32" t="inlineStr">
         <is>
           <t>✅ Live (OTA)</t>
         </is>
@@ -3327,22 +3336,22 @@
       </c>
     </row>
     <row r="91">
-      <c r="A91" s="26" t="inlineStr">
+      <c r="A91" s="30" t="inlineStr">
         <is>
           <t>83</t>
         </is>
       </c>
-      <c r="B91" s="27" t="inlineStr">
+      <c r="B91" s="31" t="inlineStr">
         <is>
           <t>Cache-Control: no-store על כל ה-API</t>
         </is>
       </c>
-      <c r="C91" s="26" t="inlineStr">
+      <c r="C91" s="30" t="inlineStr">
         <is>
           <t>Backend / Bug Fix</t>
         </is>
       </c>
-      <c r="D91" s="28" t="inlineStr">
+      <c r="D91" s="32" t="inlineStr">
         <is>
           <t>✅ Live</t>
         </is>
@@ -3359,22 +3368,22 @@
       </c>
     </row>
     <row r="92">
-      <c r="A92" s="26" t="inlineStr">
+      <c r="A92" s="30" t="inlineStr">
         <is>
           <t>84</t>
         </is>
       </c>
-      <c r="B92" s="27" t="inlineStr">
+      <c r="B92" s="31" t="inlineStr">
         <is>
           <t>סדרה שנתית = סוף שנה, לא ינואר</t>
         </is>
       </c>
-      <c r="C92" s="26" t="inlineStr">
+      <c r="C92" s="30" t="inlineStr">
         <is>
           <t>Backend / Bug Fix</t>
         </is>
       </c>
-      <c r="D92" s="28" t="inlineStr">
+      <c r="D92" s="32" t="inlineStr">
         <is>
           <t>✅ Live</t>
         </is>
@@ -3391,22 +3400,22 @@
       </c>
     </row>
     <row r="93">
-      <c r="A93" s="26" t="inlineStr">
+      <c r="A93" s="30" t="inlineStr">
         <is>
           <t>85</t>
         </is>
       </c>
-      <c r="B93" s="27" t="inlineStr">
+      <c r="B93" s="31" t="inlineStr">
         <is>
           <t>TTM של Buyback דרש 2 רבעונים</t>
         </is>
       </c>
-      <c r="C93" s="26" t="inlineStr">
+      <c r="C93" s="30" t="inlineStr">
         <is>
           <t>Backend / Bug Fix</t>
         </is>
       </c>
-      <c r="D93" s="28" t="inlineStr">
+      <c r="D93" s="32" t="inlineStr">
         <is>
           <t>✅ Live</t>
         </is>
@@ -3423,22 +3432,22 @@
       </c>
     </row>
     <row r="94">
-      <c r="A94" s="26" t="inlineStr">
+      <c r="A94" s="30" t="inlineStr">
         <is>
           <t>86</t>
         </is>
       </c>
-      <c r="B94" s="27" t="inlineStr">
+      <c r="B94" s="31" t="inlineStr">
         <is>
           <t>ניקוי ריפו — cloudflared.exe 52MB</t>
         </is>
       </c>
-      <c r="C94" s="26" t="inlineStr">
+      <c r="C94" s="30" t="inlineStr">
         <is>
           <t>DevOps</t>
         </is>
       </c>
-      <c r="D94" s="28" t="inlineStr">
+      <c r="D94" s="32" t="inlineStr">
         <is>
           <t>✅ Live</t>
         </is>
@@ -3455,22 +3464,22 @@
       </c>
     </row>
     <row r="95">
-      <c r="A95" s="26" t="inlineStr">
+      <c r="A95" s="30" t="inlineStr">
         <is>
           <t>87</t>
         </is>
       </c>
-      <c r="B95" s="27" t="inlineStr">
+      <c r="B95" s="31" t="inlineStr">
         <is>
           <t>דיוק עמוד הפרטיות בנוגע ללוגים</t>
         </is>
       </c>
-      <c r="C95" s="26" t="inlineStr">
+      <c r="C95" s="30" t="inlineStr">
         <is>
           <t>Legal</t>
         </is>
       </c>
-      <c r="D95" s="28" t="inlineStr">
+      <c r="D95" s="32" t="inlineStr">
         <is>
           <t>✅ Live</t>
         </is>
@@ -3487,22 +3496,22 @@
       </c>
     </row>
     <row r="96">
-      <c r="A96" s="26" t="inlineStr">
+      <c r="A96" s="30" t="inlineStr">
         <is>
           <t>88</t>
         </is>
       </c>
-      <c r="B96" s="27" t="inlineStr">
+      <c r="B96" s="31" t="inlineStr">
         <is>
           <t>ביקורת קוד מלאה — 35 קבצים</t>
         </is>
       </c>
-      <c r="C96" s="26" t="inlineStr">
+      <c r="C96" s="30" t="inlineStr">
         <is>
           <t>QA</t>
         </is>
       </c>
-      <c r="D96" s="28" t="inlineStr">
+      <c r="D96" s="32" t="inlineStr">
         <is>
           <t>✅ הושלם</t>
         </is>
@@ -3526,22 +3535,22 @@
       </c>
     </row>
     <row r="98">
-      <c r="A98" s="26" t="inlineStr">
+      <c r="A98" s="30" t="inlineStr">
         <is>
           <t>89</t>
         </is>
       </c>
-      <c r="B98" s="27" t="inlineStr">
+      <c r="B98" s="31" t="inlineStr">
         <is>
           <t>צבע הגרף לפי כיוון המדד</t>
         </is>
       </c>
-      <c r="C98" s="26" t="inlineStr">
+      <c r="C98" s="30" t="inlineStr">
         <is>
           <t>Frontend / UX</t>
         </is>
       </c>
-      <c r="D98" s="28" t="inlineStr">
+      <c r="D98" s="32" t="inlineStr">
         <is>
           <t>✅ Live (OTA)</t>
         </is>
@@ -3558,22 +3567,22 @@
       </c>
     </row>
     <row r="99">
-      <c r="A99" s="26" t="inlineStr">
+      <c r="A99" s="30" t="inlineStr">
         <is>
           <t>90</t>
         </is>
       </c>
-      <c r="B99" s="27" t="inlineStr">
+      <c r="B99" s="31" t="inlineStr">
         <is>
           <t>הצהרת טווח מלא לכל 24 המדדים</t>
         </is>
       </c>
-      <c r="C99" s="26" t="inlineStr">
+      <c r="C99" s="30" t="inlineStr">
         <is>
           <t>UX / Accuracy</t>
         </is>
       </c>
-      <c r="D99" s="28" t="inlineStr">
+      <c r="D99" s="32" t="inlineStr">
         <is>
           <t>✅ Live (OTA)</t>
         </is>
@@ -3590,22 +3599,22 @@
       </c>
     </row>
     <row r="100">
-      <c r="A100" s="26" t="inlineStr">
+      <c r="A100" s="30" t="inlineStr">
         <is>
           <t>91</t>
         </is>
       </c>
-      <c r="B100" s="27" t="inlineStr">
+      <c r="B100" s="31" t="inlineStr">
         <is>
           <t>מדד שלא היה לו הסבר בכלל</t>
         </is>
       </c>
-      <c r="C100" s="26" t="inlineStr">
+      <c r="C100" s="30" t="inlineStr">
         <is>
           <t>UX / Bug Fix</t>
         </is>
       </c>
-      <c r="D100" s="28" t="inlineStr">
+      <c r="D100" s="32" t="inlineStr">
         <is>
           <t>✅ Live (OTA)</t>
         </is>
@@ -3622,22 +3631,22 @@
       </c>
     </row>
     <row r="101">
-      <c r="A101" s="26" t="inlineStr">
+      <c r="A101" s="30" t="inlineStr">
         <is>
           <t>92</t>
         </is>
       </c>
-      <c r="B101" s="27" t="inlineStr">
+      <c r="B101" s="31" t="inlineStr">
         <is>
           <t>מספר וכיתוב באותו צבע</t>
         </is>
       </c>
-      <c r="C101" s="26" t="inlineStr">
+      <c r="C101" s="30" t="inlineStr">
         <is>
           <t>Frontend / UX</t>
         </is>
       </c>
-      <c r="D101" s="28" t="inlineStr">
+      <c r="D101" s="32" t="inlineStr">
         <is>
           <t>✅ Live (OTA)</t>
         </is>
@@ -3654,22 +3663,22 @@
       </c>
     </row>
     <row r="102">
-      <c r="A102" s="26" t="inlineStr">
+      <c r="A102" s="30" t="inlineStr">
         <is>
           <t>93</t>
         </is>
       </c>
-      <c r="B102" s="27" t="inlineStr">
+      <c r="B102" s="31" t="inlineStr">
         <is>
           <t>כתום רק כשיש אזהרה</t>
         </is>
       </c>
-      <c r="C102" s="26" t="inlineStr">
+      <c r="C102" s="30" t="inlineStr">
         <is>
           <t>Frontend / UX</t>
         </is>
       </c>
-      <c r="D102" s="28" t="inlineStr">
+      <c r="D102" s="32" t="inlineStr">
         <is>
           <t>✅ Live (OTA)</t>
         </is>
@@ -3686,22 +3695,22 @@
       </c>
     </row>
     <row r="103">
-      <c r="A103" s="26" t="inlineStr">
+      <c r="A103" s="30" t="inlineStr">
         <is>
           <t>94</t>
         </is>
       </c>
-      <c r="B103" s="27" t="inlineStr">
+      <c r="B103" s="31" t="inlineStr">
         <is>
           <t>הצבע שורד את המעבר בין מסכים</t>
         </is>
       </c>
-      <c r="C103" s="26" t="inlineStr">
+      <c r="C103" s="30" t="inlineStr">
         <is>
           <t>Frontend / Bug Fix</t>
         </is>
       </c>
-      <c r="D103" s="28" t="inlineStr">
+      <c r="D103" s="32" t="inlineStr">
         <is>
           <t>✅ Live (OTA)</t>
         </is>
@@ -3718,22 +3727,22 @@
       </c>
     </row>
     <row r="104">
-      <c r="A104" s="26" t="inlineStr">
+      <c r="A104" s="30" t="inlineStr">
         <is>
           <t>95</t>
         </is>
       </c>
-      <c r="B104" s="27" t="inlineStr">
+      <c r="B104" s="31" t="inlineStr">
         <is>
           <t>חומת ההסכמה של גוגל — רוסית וספרדית</t>
         </is>
       </c>
-      <c r="C104" s="26" t="inlineStr">
+      <c r="C104" s="30" t="inlineStr">
         <is>
           <t>Frontend / i18n</t>
         </is>
       </c>
-      <c r="D104" s="28" t="inlineStr">
+      <c r="D104" s="32" t="inlineStr">
         <is>
           <t>✅ Live (OTA)</t>
         </is>
@@ -3750,22 +3759,22 @@
       </c>
     </row>
     <row r="105">
-      <c r="A105" s="26" t="inlineStr">
+      <c r="A105" s="30" t="inlineStr">
         <is>
           <t>96</t>
         </is>
       </c>
-      <c r="B105" s="27" t="inlineStr">
+      <c r="B105" s="31" t="inlineStr">
         <is>
           <t>ביקורת כיסוי-שפות לכל השינויים</t>
         </is>
       </c>
-      <c r="C105" s="26" t="inlineStr">
+      <c r="C105" s="30" t="inlineStr">
         <is>
           <t>QA / i18n</t>
         </is>
       </c>
-      <c r="D105" s="28" t="inlineStr">
+      <c r="D105" s="32" t="inlineStr">
         <is>
           <t>✅ הושלם</t>
         </is>
@@ -3809,26 +3818,46 @@
       </c>
       <c r="F106" s="16" t="inlineStr">
         <is>
-          <t>תשואת דיבידנד/רכישה חוזרת יורדת גם כשהתשלום נחתך (רע) וגם כשהמחיר עולה מהר יותר (טוב). וולמארט העלתה דיבידנד 52 שנה ברציפות והתשואה ירדה 3.2%→0.9% — הגרף צבע את זה אדום. מהתשואה לבדה אי אפשר להבחין, אז הקו כחול = מידע ולא פסק דין.</t>
+          <t>תשואת דיבידנד/רכישה חוזרת יורדת גם כשהתשלום נחתך (רע) וגם כשהמחיר עולה מהר יותר (טוב). וולמארט העלתה דיבידנד 52 שנה ברציפות והתשואה ירדה 3.2%→0.9% — הגרף צבע אדום. הקו כחול = מידע, לא פסק דין.</t>
         </is>
       </c>
     </row>
     <row r="107">
-      <c r="A107" s="3" t="inlineStr">
+      <c r="A107" s="33" t="inlineStr">
+        <is>
+          <t>98</t>
+        </is>
+      </c>
+      <c r="B107" s="34" t="inlineStr">
+        <is>
+          <t>צבע הגרף = צבע האריח, לא המגמה</t>
+        </is>
+      </c>
+      <c r="C107" s="33" t="inlineStr">
+        <is>
+          <t>Frontend / UX</t>
+        </is>
+      </c>
+      <c r="D107" s="35" t="inlineStr">
+        <is>
+          <t>✅ Live (OTA)</t>
+        </is>
+      </c>
+      <c r="E107" s="16" t="inlineStr">
+        <is>
+          <t>PriceChart.js, MetricHistoryScreen.js</t>
+        </is>
+      </c>
+      <c r="F107" s="16" t="inlineStr">
+        <is>
+          <t>הגרף צבע לפי מגמה והאריח לפי רמה — שני דברים שיכולים לסתור. P/B שירד מ-14.9 ל-6.84 קיבל קו ירוק ("משתפר") בעוד 6.84 עדיין מעל סף היוקר 5 והאריח צבע אדום. עכשיו הקו נושא את אותו פסק דין; המגמה נראית מצורת הקו. מדד בלי סף ובלי ציון = קו כחול.</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="3" t="inlineStr">
         <is>
           <t>🔜  NOT YET STARTED</t>
-        </is>
-      </c>
-      <c r="B107" s="5" t="inlineStr"/>
-      <c r="C107" s="4" t="inlineStr"/>
-      <c r="D107" s="4" t="inlineStr"/>
-      <c r="E107" s="4" t="inlineStr"/>
-      <c r="F107" s="5" t="inlineStr"/>
-    </row>
-    <row r="108">
-      <c r="A108" s="6" t="inlineStr">
-        <is>
-          <t>19</t>
         </is>
       </c>
       <c r="B108" s="4" t="n"/>
@@ -3838,37 +3867,33 @@
       <c r="F108" s="5" t="n"/>
     </row>
     <row r="109">
-      <c r="A109" s="10" t="inlineStr">
+      <c r="A109" s="6" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="B109" s="4" t="n"/>
+      <c r="C109" s="4" t="n"/>
+      <c r="D109" s="4" t="n"/>
+      <c r="E109" s="4" t="n"/>
+      <c r="F109" s="5" t="n"/>
+    </row>
+    <row r="110">
+      <c r="A110" s="10" t="inlineStr">
         <is>
           <t>Legend</t>
         </is>
       </c>
-    </row>
-    <row r="110">
-      <c r="A110" s="6" t="inlineStr">
-        <is>
-          <t>✅ Live</t>
-        </is>
-      </c>
-      <c r="B110" s="7" t="inlineStr">
-        <is>
-          <t>פרוס ופעיל ב-Render — נראה לכל המשתמשים</t>
-        </is>
-      </c>
-      <c r="C110" s="6" t="inlineStr"/>
-      <c r="D110" s="8" t="inlineStr"/>
-      <c r="E110" s="9" t="inlineStr"/>
-      <c r="F110" s="9" t="inlineStr"/>
     </row>
     <row r="111">
       <c r="A111" s="6" t="inlineStr">
         <is>
-          <t>✅ In APK</t>
+          <t>✅ Live</t>
         </is>
       </c>
       <c r="B111" s="7" t="inlineStr">
         <is>
-          <t>כלול ב-APK המותקן — נראה לכל המשתמשים</t>
+          <t>פרוס ופעיל ב-Render — נראה לכל המשתמשים</t>
         </is>
       </c>
       <c r="C111" s="6" t="inlineStr"/>
@@ -3879,12 +3904,12 @@
     <row r="112">
       <c r="A112" s="6" t="inlineStr">
         <is>
-          <t>⏳ Next APK</t>
+          <t>✅ In APK</t>
         </is>
       </c>
       <c r="B112" s="7" t="inlineStr">
         <is>
-          <t>הקוד מוזג — דורש build ו-APK חדש</t>
+          <t>כלול ב-APK המותקן — נראה לכל המשתמשים</t>
         </is>
       </c>
       <c r="C112" s="6" t="inlineStr"/>
@@ -3895,12 +3920,12 @@
     <row r="113">
       <c r="A113" s="6" t="inlineStr">
         <is>
-          <t>✅ Live (OTA)</t>
+          <t>⏳ Next APK</t>
         </is>
       </c>
       <c r="B113" s="7" t="inlineStr">
         <is>
-          <t>שינוי JS — מועבר אוטומטית בהפעלה הבאה</t>
+          <t>הקוד מוזג — דורש build ו-APK חדש</t>
         </is>
       </c>
       <c r="C113" s="6" t="inlineStr"/>
@@ -3909,42 +3934,50 @@
       <c r="F113" s="9" t="inlineStr"/>
     </row>
     <row r="114">
-      <c r="A114" s="21" t="inlineStr">
-        <is>
-          <t>⏳ ממתין ל-push</t>
-        </is>
-      </c>
-      <c r="B114" s="22" t="inlineStr">
-        <is>
-          <t>הקוד מוכן מקומית — טרם נדחף/נפרס</t>
-        </is>
-      </c>
+      <c r="A114" s="6" t="inlineStr">
+        <is>
+          <t>✅ Live (OTA)</t>
+        </is>
+      </c>
+      <c r="B114" s="7" t="inlineStr">
+        <is>
+          <t>שינוי JS — מועבר אוטומטית בהפעלה הבאה</t>
+        </is>
+      </c>
+      <c r="C114" s="6" t="inlineStr"/>
+      <c r="D114" s="8" t="inlineStr"/>
+      <c r="E114" s="9" t="inlineStr"/>
+      <c r="F114" s="9" t="inlineStr"/>
     </row>
     <row r="115">
       <c r="A115" s="21" t="inlineStr">
         <is>
+          <t>⏳ ממתין ל-push</t>
+        </is>
+      </c>
+      <c r="B115" s="22" t="inlineStr">
+        <is>
+          <t>הקוד מוכן מקומית — טרם נדחף/נפרס</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="21" t="inlineStr">
+        <is>
           <t>⏳ דורש build</t>
         </is>
       </c>
-      <c r="B115" s="22" t="inlineStr">
+      <c r="B116" s="22" t="inlineStr">
         <is>
           <t>שינוי נייטיב — OTA לא מספיק, צריך AAB/APK חדש</t>
         </is>
       </c>
     </row>
-    <row r="116"/>
-    <row r="117">
-      <c r="A117" s="23" t="inlineStr">
+    <row r="117"/>
+    <row r="118">
+      <c r="A118" s="23" t="inlineStr">
         <is>
           <t>סיכום Session 6-7</t>
-        </is>
-      </c>
-    </row>
-    <row r="118">
-      <c r="A118" s="24" t="n"/>
-      <c r="B118" s="25" t="inlineStr">
-        <is>
-          <t>45  —  פריטים חדשים שנוספו (52-96)</t>
         </is>
       </c>
     </row>
@@ -3952,7 +3985,7 @@
       <c r="A119" s="24" t="n"/>
       <c r="B119" s="25" t="inlineStr">
         <is>
-          <t>44  —  חיים בייצור או ב-OTA</t>
+          <t>45  —  פריטים חדשים שנוספו (52-96)</t>
         </is>
       </c>
     </row>
@@ -3960,7 +3993,7 @@
       <c r="A120" s="24" t="n"/>
       <c r="B120" s="25" t="inlineStr">
         <is>
-          <t>1  —  דורש build חדש: תמיכת טאבלט (פריט 68)</t>
+          <t>44  —  חיים בייצור או ב-OTA</t>
         </is>
       </c>
     </row>
@@ -3968,7 +4001,7 @@
       <c r="A121" s="24" t="n"/>
       <c r="B121" s="25" t="inlineStr">
         <is>
-          <t>11,781  —  שורות קוד שנקראו במלואן, 36 קבצים</t>
+          <t>1  —  דורש build חדש: תמיכת טאבלט (פריט 68)</t>
         </is>
       </c>
     </row>
@@ -3976,7 +4009,7 @@
       <c r="A122" s="24" t="n"/>
       <c r="B122" s="25" t="inlineStr">
         <is>
-          <t>29  —  חבילות בדיקה התנהגותיות עוברות</t>
+          <t>11,781  —  שורות קוד שנקראו במלואן, 36 קבצים</t>
         </is>
       </c>
     </row>
@@ -3984,14 +4017,22 @@
       <c r="A123" s="24" t="n"/>
       <c r="B123" s="25" t="inlineStr">
         <is>
+          <t>29  —  חבילות בדיקה התנהגותיות עוברות</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="24" t="n"/>
+      <c r="B124" s="25" t="inlineStr">
+        <is>
           <t>18  —  ראוטים בשרת · 316 מפתחות i18n × 4 שפות</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="4">
+    <mergeCell ref="A107:F107"/>
     <mergeCell ref="A97:F97"/>
-    <mergeCell ref="A107:F107"/>
     <mergeCell ref="A59:F59"/>
     <mergeCell ref="A25:F25"/>
   </mergeCells>

</xml_diff>

<commit_message>
Never show a negative multiple (RIVN showed EV/EBITDA -6.72 in green); disclose provider-vs-computed differences
</commit_message>
<xml_diff>
--- a/BuddhaVest_Progress.xlsx
+++ b/BuddhaVest_Progress.xlsx
@@ -175,7 +175,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="39">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -266,6 +266,15 @@
       <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
@@ -633,7 +642,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F124"/>
+  <dimension ref="A1:F125"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2344,22 +2353,22 @@
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="30" t="inlineStr">
+      <c r="A60" s="33" t="inlineStr">
         <is>
           <t>52</t>
         </is>
       </c>
-      <c r="B60" s="31" t="inlineStr">
+      <c r="B60" s="34" t="inlineStr">
         <is>
           <t>מרוץ שפות — 5 מסכים/רכיבים</t>
         </is>
       </c>
-      <c r="C60" s="30" t="inlineStr">
+      <c r="C60" s="33" t="inlineStr">
         <is>
           <t>Frontend / Bug Fix</t>
         </is>
       </c>
-      <c r="D60" s="32" t="inlineStr">
+      <c r="D60" s="35" t="inlineStr">
         <is>
           <t>✅ Live (OTA)</t>
         </is>
@@ -2376,22 +2385,22 @@
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="30" t="inlineStr">
+      <c r="A61" s="33" t="inlineStr">
         <is>
           <t>53</t>
         </is>
       </c>
-      <c r="B61" s="31" t="inlineStr">
+      <c r="B61" s="34" t="inlineStr">
         <is>
           <t>Volume/Avg Vol ריקים לסירוגין</t>
         </is>
       </c>
-      <c r="C61" s="30" t="inlineStr">
+      <c r="C61" s="33" t="inlineStr">
         <is>
           <t>Backend / Bug Fix</t>
         </is>
       </c>
-      <c r="D61" s="32" t="inlineStr">
+      <c r="D61" s="35" t="inlineStr">
         <is>
           <t>✅ Live</t>
         </is>
@@ -2408,22 +2417,22 @@
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="30" t="inlineStr">
+      <c r="A62" s="33" t="inlineStr">
         <is>
           <t>54</t>
         </is>
       </c>
-      <c r="B62" s="31" t="inlineStr">
+      <c r="B62" s="34" t="inlineStr">
         <is>
           <t>המרת אגורות→שקל למניות ת"א</t>
         </is>
       </c>
-      <c r="C62" s="30" t="inlineStr">
+      <c r="C62" s="33" t="inlineStr">
         <is>
           <t>Backend</t>
         </is>
       </c>
-      <c r="D62" s="32" t="inlineStr">
+      <c r="D62" s="35" t="inlineStr">
         <is>
           <t>✅ Live</t>
         </is>
@@ -2440,22 +2449,22 @@
       </c>
     </row>
     <row r="63">
-      <c r="A63" s="30" t="inlineStr">
+      <c r="A63" s="33" t="inlineStr">
         <is>
           <t>55</t>
         </is>
       </c>
-      <c r="B63" s="31" t="inlineStr">
+      <c r="B63" s="34" t="inlineStr">
         <is>
           <t>באג יחידות ב-Buyback (3500000000%)</t>
         </is>
       </c>
-      <c r="C63" s="30" t="inlineStr">
+      <c r="C63" s="33" t="inlineStr">
         <is>
           <t>Backend + Frontend</t>
         </is>
       </c>
-      <c r="D63" s="32" t="inlineStr">
+      <c r="D63" s="35" t="inlineStr">
         <is>
           <t>✅ Live</t>
         </is>
@@ -2472,22 +2481,22 @@
       </c>
     </row>
     <row r="64">
-      <c r="A64" s="30" t="inlineStr">
+      <c r="A64" s="33" t="inlineStr">
         <is>
           <t>56</t>
         </is>
       </c>
-      <c r="B64" s="31" t="inlineStr">
+      <c r="B64" s="34" t="inlineStr">
         <is>
           <t>תיקוני נכונות במנוע הציון</t>
         </is>
       </c>
-      <c r="C64" s="30" t="inlineStr">
+      <c r="C64" s="33" t="inlineStr">
         <is>
           <t>Backend / Scoring</t>
         </is>
       </c>
-      <c r="D64" s="32" t="inlineStr">
+      <c r="D64" s="35" t="inlineStr">
         <is>
           <t>✅ Live</t>
         </is>
@@ -2504,22 +2513,22 @@
       </c>
     </row>
     <row r="65">
-      <c r="A65" s="30" t="inlineStr">
+      <c r="A65" s="33" t="inlineStr">
         <is>
           <t>57</t>
         </is>
       </c>
-      <c r="B65" s="31" t="inlineStr">
+      <c r="B65" s="34" t="inlineStr">
         <is>
           <t>ניסוח דיבידנד כן — לא "משולם בעקביות"</t>
         </is>
       </c>
-      <c r="C65" s="30" t="inlineStr">
+      <c r="C65" s="33" t="inlineStr">
         <is>
           <t>Legal / Accuracy</t>
         </is>
       </c>
-      <c r="D65" s="32" t="inlineStr">
+      <c r="D65" s="35" t="inlineStr">
         <is>
           <t>✅ Live</t>
         </is>
@@ -2536,22 +2545,22 @@
       </c>
     </row>
     <row r="66">
-      <c r="A66" s="30" t="inlineStr">
+      <c r="A66" s="33" t="inlineStr">
         <is>
           <t>58</t>
         </is>
       </c>
-      <c r="B66" s="31" t="inlineStr">
+      <c r="B66" s="34" t="inlineStr">
         <is>
           <t>SSRF — /translate-article</t>
         </is>
       </c>
-      <c r="C66" s="30" t="inlineStr">
+      <c r="C66" s="33" t="inlineStr">
         <is>
           <t>Backend / Security</t>
         </is>
       </c>
-      <c r="D66" s="32" t="inlineStr">
+      <c r="D66" s="35" t="inlineStr">
         <is>
           <t>✅ Live</t>
         </is>
@@ -2568,22 +2577,22 @@
       </c>
     </row>
     <row r="67">
-      <c r="A67" s="30" t="inlineStr">
+      <c r="A67" s="33" t="inlineStr">
         <is>
           <t>59</t>
         </is>
       </c>
-      <c r="B67" s="31" t="inlineStr">
+      <c r="B67" s="34" t="inlineStr">
         <is>
           <t>XSS ב-WebView של הכתבות</t>
         </is>
       </c>
-      <c r="C67" s="30" t="inlineStr">
+      <c r="C67" s="33" t="inlineStr">
         <is>
           <t>Frontend / Security</t>
         </is>
       </c>
-      <c r="D67" s="32" t="inlineStr">
+      <c r="D67" s="35" t="inlineStr">
         <is>
           <t>✅ Live (OTA)</t>
         </is>
@@ -2600,22 +2609,22 @@
       </c>
     </row>
     <row r="68">
-      <c r="A68" s="30" t="inlineStr">
+      <c r="A68" s="33" t="inlineStr">
         <is>
           <t>60</t>
         </is>
       </c>
-      <c r="B68" s="31" t="inlineStr">
+      <c r="B68" s="34" t="inlineStr">
         <is>
           <t>הסרת /debug-pe ו-/debug-rows</t>
         </is>
       </c>
-      <c r="C68" s="30" t="inlineStr">
+      <c r="C68" s="33" t="inlineStr">
         <is>
           <t>Backend / Security</t>
         </is>
       </c>
-      <c r="D68" s="32" t="inlineStr">
+      <c r="D68" s="35" t="inlineStr">
         <is>
           <t>✅ Live</t>
         </is>
@@ -2632,22 +2641,22 @@
       </c>
     </row>
     <row r="69">
-      <c r="A69" s="30" t="inlineStr">
+      <c r="A69" s="33" t="inlineStr">
         <is>
           <t>61</t>
         </is>
       </c>
-      <c r="B69" s="31" t="inlineStr">
+      <c r="B69" s="34" t="inlineStr">
         <is>
           <t>5 דליפות של פרטי חריגה ללקוח</t>
         </is>
       </c>
-      <c r="C69" s="30" t="inlineStr">
+      <c r="C69" s="33" t="inlineStr">
         <is>
           <t>Backend / Security</t>
         </is>
       </c>
-      <c r="D69" s="32" t="inlineStr">
+      <c r="D69" s="35" t="inlineStr">
         <is>
           <t>✅ Live</t>
         </is>
@@ -2664,22 +2673,22 @@
       </c>
     </row>
     <row r="70">
-      <c r="A70" s="30" t="inlineStr">
+      <c r="A70" s="33" t="inlineStr">
         <is>
           <t>62</t>
         </is>
       </c>
-      <c r="B70" s="31" t="inlineStr">
+      <c r="B70" s="34" t="inlineStr">
         <is>
           <t>פיצוץ זיכרון בעליית השרת</t>
         </is>
       </c>
-      <c r="C70" s="30" t="inlineStr">
+      <c r="C70" s="33" t="inlineStr">
         <is>
           <t>Backend / Performance</t>
         </is>
       </c>
-      <c r="D70" s="32" t="inlineStr">
+      <c r="D70" s="35" t="inlineStr">
         <is>
           <t>✅ Live</t>
         </is>
@@ -2696,22 +2705,22 @@
       </c>
     </row>
     <row r="71">
-      <c r="A71" s="30" t="inlineStr">
+      <c r="A71" s="33" t="inlineStr">
         <is>
           <t>63</t>
         </is>
       </c>
-      <c r="B71" s="31" t="inlineStr">
+      <c r="B71" s="34" t="inlineStr">
         <is>
           <t>תקרת מטמון + single-flight</t>
         </is>
       </c>
-      <c r="C71" s="30" t="inlineStr">
+      <c r="C71" s="33" t="inlineStr">
         <is>
           <t>Backend / Performance</t>
         </is>
       </c>
-      <c r="D71" s="32" t="inlineStr">
+      <c r="D71" s="35" t="inlineStr">
         <is>
           <t>✅ Live</t>
         </is>
@@ -2728,22 +2737,22 @@
       </c>
     </row>
     <row r="72">
-      <c r="A72" s="30" t="inlineStr">
+      <c r="A72" s="33" t="inlineStr">
         <is>
           <t>64</t>
         </is>
       </c>
-      <c r="B72" s="31" t="inlineStr">
+      <c r="B72" s="34" t="inlineStr">
         <is>
           <t>חלון היסטוריה 10y במקום max</t>
         </is>
       </c>
-      <c r="C72" s="30" t="inlineStr">
+      <c r="C72" s="33" t="inlineStr">
         <is>
           <t>Backend / Performance</t>
         </is>
       </c>
-      <c r="D72" s="32" t="inlineStr">
+      <c r="D72" s="35" t="inlineStr">
         <is>
           <t>✅ Live</t>
         </is>
@@ -2760,22 +2769,22 @@
       </c>
     </row>
     <row r="73">
-      <c r="A73" s="30" t="inlineStr">
+      <c r="A73" s="33" t="inlineStr">
         <is>
           <t>65</t>
         </is>
       </c>
-      <c r="B73" s="31" t="inlineStr">
+      <c r="B73" s="34" t="inlineStr">
         <is>
           <t>Debounce בחיפוש</t>
         </is>
       </c>
-      <c r="C73" s="30" t="inlineStr">
+      <c r="C73" s="33" t="inlineStr">
         <is>
           <t>Frontend / Performance</t>
         </is>
       </c>
-      <c r="D73" s="32" t="inlineStr">
+      <c r="D73" s="35" t="inlineStr">
         <is>
           <t>✅ Live (OTA)</t>
         </is>
@@ -2792,22 +2801,22 @@
       </c>
     </row>
     <row r="74">
-      <c r="A74" s="30" t="inlineStr">
+      <c r="A74" s="33" t="inlineStr">
         <is>
           <t>66</t>
         </is>
       </c>
-      <c r="B74" s="31" t="inlineStr">
+      <c r="B74" s="34" t="inlineStr">
         <is>
           <t>תקציב זמן ל-Stooq</t>
         </is>
       </c>
-      <c r="C74" s="30" t="inlineStr">
+      <c r="C74" s="33" t="inlineStr">
         <is>
           <t>Backend / Performance</t>
         </is>
       </c>
-      <c r="D74" s="32" t="inlineStr">
+      <c r="D74" s="35" t="inlineStr">
         <is>
           <t>✅ Live</t>
         </is>
@@ -2824,22 +2833,22 @@
       </c>
     </row>
     <row r="75">
-      <c r="A75" s="30" t="inlineStr">
+      <c r="A75" s="33" t="inlineStr">
         <is>
           <t>67</t>
         </is>
       </c>
-      <c r="B75" s="31" t="inlineStr">
+      <c r="B75" s="34" t="inlineStr">
         <is>
           <t>אובדן נתונים ביומן המחקר</t>
         </is>
       </c>
-      <c r="C75" s="30" t="inlineStr">
+      <c r="C75" s="33" t="inlineStr">
         <is>
           <t>Frontend / Bug Fix</t>
         </is>
       </c>
-      <c r="D75" s="32" t="inlineStr">
+      <c r="D75" s="35" t="inlineStr">
         <is>
           <t>✅ Live (OTA)</t>
         </is>
@@ -2863,7 +2872,7 @@
       </c>
       <c r="B76" s="18" t="inlineStr">
         <is>
-          <t>תמיכת טאבלט</t>
+          <t>הקלה חלקית לטאבלט (לא תמיכה מלאה)</t>
         </is>
       </c>
       <c r="C76" s="17" t="inlineStr">
@@ -2873,7 +2882,7 @@
       </c>
       <c r="D76" s="19" t="inlineStr">
         <is>
-          <t>⏳ דורש build</t>
+          <t>⚠️ חלקי</t>
         </is>
       </c>
       <c r="E76" s="20" t="inlineStr">
@@ -2883,27 +2892,27 @@
       </c>
       <c r="F76" s="20" t="inlineStr">
         <is>
-          <t>TabletFrame (רוחב ≥700 ממורכז ל-600), שחרור סיבוב לטאבלט ונעילת portrait לטלפון, כפתור צף שנצמד מחדש בסיבוב. supportsTablet=true.</t>
+          <t>תיאור מדויק: TabletFrame ממרכז את התוכן ל-600px, סיבוב משוחרר לטאבלט ונעול לטלפון, והכפתור הצף נצמד מחדש בסיבוב. זו אפליקציית טלפון ממורכזת — לא פריסת טאבלט. הטבלאות (טבלת השוק ב-HomeScreen, FinancialsCard) בנויות על רוחב עמודות קבוע בפיקסלים ולא מתאימות את עצמן. supportsTablet הוחזר ל-false עד שתיבנה פריסה אמיתית. תיעוד קודם תיאר את זה כ"תמיכה מלאה" — תיאור שלא היה לו כיסוי, תוקן כאן.</t>
         </is>
       </c>
     </row>
     <row r="77">
-      <c r="A77" s="30" t="inlineStr">
+      <c r="A77" s="33" t="inlineStr">
         <is>
           <t>69</t>
         </is>
       </c>
-      <c r="B77" s="31" t="inlineStr">
+      <c r="B77" s="34" t="inlineStr">
         <is>
           <t>מסך הסכמה בהפעלה ראשונה</t>
         </is>
       </c>
-      <c r="C77" s="30" t="inlineStr">
+      <c r="C77" s="33" t="inlineStr">
         <is>
           <t>Legal</t>
         </is>
       </c>
-      <c r="D77" s="32" t="inlineStr">
+      <c r="D77" s="35" t="inlineStr">
         <is>
           <t>✅ Live (OTA)</t>
         </is>
@@ -2920,22 +2929,22 @@
       </c>
     </row>
     <row r="78">
-      <c r="A78" s="30" t="inlineStr">
+      <c r="A78" s="33" t="inlineStr">
         <is>
           <t>70</t>
         </is>
       </c>
-      <c r="B78" s="31" t="inlineStr">
+      <c r="B78" s="34" t="inlineStr">
         <is>
           <t>שכתוב תיאור החנות — בלי הבטחות</t>
         </is>
       </c>
-      <c r="C78" s="30" t="inlineStr">
+      <c r="C78" s="33" t="inlineStr">
         <is>
           <t>Legal / Store</t>
         </is>
       </c>
-      <c r="D78" s="32" t="inlineStr">
+      <c r="D78" s="35" t="inlineStr">
         <is>
           <t>✅ מוכן</t>
         </is>
@@ -2952,22 +2961,22 @@
       </c>
     </row>
     <row r="79">
-      <c r="A79" s="30" t="inlineStr">
+      <c r="A79" s="33" t="inlineStr">
         <is>
           <t>71</t>
         </is>
       </c>
-      <c r="B79" s="31" t="inlineStr">
+      <c r="B79" s="34" t="inlineStr">
         <is>
           <t>מדריך צילומי מסך לחנות</t>
         </is>
       </c>
-      <c r="C79" s="30" t="inlineStr">
+      <c r="C79" s="33" t="inlineStr">
         <is>
           <t>Store Assets</t>
         </is>
       </c>
-      <c r="D79" s="32" t="inlineStr">
+      <c r="D79" s="35" t="inlineStr">
         <is>
           <t>✅ הושלם</t>
         </is>
@@ -2984,22 +2993,22 @@
       </c>
     </row>
     <row r="80">
-      <c r="A80" s="30" t="inlineStr">
+      <c r="A80" s="33" t="inlineStr">
         <is>
           <t>72</t>
         </is>
       </c>
-      <c r="B80" s="31" t="inlineStr">
+      <c r="B80" s="34" t="inlineStr">
         <is>
           <t>RTL בכל המסכים</t>
         </is>
       </c>
-      <c r="C80" s="30" t="inlineStr">
+      <c r="C80" s="33" t="inlineStr">
         <is>
           <t>Frontend / i18n</t>
         </is>
       </c>
-      <c r="D80" s="32" t="inlineStr">
+      <c r="D80" s="35" t="inlineStr">
         <is>
           <t>✅ Live (OTA)</t>
         </is>
@@ -3016,22 +3025,22 @@
       </c>
     </row>
     <row r="81">
-      <c r="A81" s="30" t="inlineStr">
+      <c r="A81" s="33" t="inlineStr">
         <is>
           <t>73</t>
         </is>
       </c>
-      <c r="B81" s="31" t="inlineStr">
+      <c r="B81" s="34" t="inlineStr">
         <is>
           <t>תווית גרסה מ-app.json</t>
         </is>
       </c>
-      <c r="C81" s="30" t="inlineStr">
+      <c r="C81" s="33" t="inlineStr">
         <is>
           <t>Frontend</t>
         </is>
       </c>
-      <c r="D81" s="32" t="inlineStr">
+      <c r="D81" s="35" t="inlineStr">
         <is>
           <t>✅ Live (OTA)</t>
         </is>
@@ -3048,22 +3057,22 @@
       </c>
     </row>
     <row r="82">
-      <c r="A82" s="30" t="inlineStr">
+      <c r="A82" s="33" t="inlineStr">
         <is>
           <t>74</t>
         </is>
       </c>
-      <c r="B82" s="31" t="inlineStr">
+      <c r="B82" s="34" t="inlineStr">
         <is>
           <t>טעינה דו-שלבית ברשימת המעקב</t>
         </is>
       </c>
-      <c r="C82" s="30" t="inlineStr">
+      <c r="C82" s="33" t="inlineStr">
         <is>
           <t>Frontend / Performance</t>
         </is>
       </c>
-      <c r="D82" s="32" t="inlineStr">
+      <c r="D82" s="35" t="inlineStr">
         <is>
           <t>✅ Live (OTA)</t>
         </is>
@@ -3080,22 +3089,22 @@
       </c>
     </row>
     <row r="83">
-      <c r="A83" s="30" t="inlineStr">
+      <c r="A83" s="33" t="inlineStr">
         <is>
           <t>75</t>
         </is>
       </c>
-      <c r="B83" s="31" t="inlineStr">
+      <c r="B83" s="34" t="inlineStr">
         <is>
           <t>/quotes: אגורות, שם חברה, מטבע</t>
         </is>
       </c>
-      <c r="C83" s="30" t="inlineStr">
+      <c r="C83" s="33" t="inlineStr">
         <is>
           <t>Backend</t>
         </is>
       </c>
-      <c r="D83" s="32" t="inlineStr">
+      <c r="D83" s="35" t="inlineStr">
         <is>
           <t>✅ Live</t>
         </is>
@@ -3112,22 +3121,22 @@
       </c>
     </row>
     <row r="84">
-      <c r="A84" s="30" t="inlineStr">
+      <c r="A84" s="33" t="inlineStr">
         <is>
           <t>76</t>
         </is>
       </c>
-      <c r="B84" s="31" t="inlineStr">
+      <c r="B84" s="34" t="inlineStr">
         <is>
           <t>מיזוג במקום החלפה ברשימת המעקב</t>
         </is>
       </c>
-      <c r="C84" s="30" t="inlineStr">
+      <c r="C84" s="33" t="inlineStr">
         <is>
           <t>Frontend / Bug Fix</t>
         </is>
       </c>
-      <c r="D84" s="32" t="inlineStr">
+      <c r="D84" s="35" t="inlineStr">
         <is>
           <t>✅ Live (OTA)</t>
         </is>
@@ -3144,22 +3153,22 @@
       </c>
     </row>
     <row r="85">
-      <c r="A85" s="30" t="inlineStr">
+      <c r="A85" s="33" t="inlineStr">
         <is>
           <t>77</t>
         </is>
       </c>
-      <c r="B85" s="31" t="inlineStr">
+      <c r="B85" s="34" t="inlineStr">
         <is>
           <t>מרוץ במסך הבית — market/FX</t>
         </is>
       </c>
-      <c r="C85" s="30" t="inlineStr">
+      <c r="C85" s="33" t="inlineStr">
         <is>
           <t>Frontend / Bug Fix</t>
         </is>
       </c>
-      <c r="D85" s="32" t="inlineStr">
+      <c r="D85" s="35" t="inlineStr">
         <is>
           <t>✅ Live (OTA)</t>
         </is>
@@ -3176,22 +3185,22 @@
       </c>
     </row>
     <row r="86">
-      <c r="A86" s="30" t="inlineStr">
+      <c r="A86" s="33" t="inlineStr">
         <is>
           <t>78</t>
         </is>
       </c>
-      <c r="B86" s="31" t="inlineStr">
+      <c r="B86" s="34" t="inlineStr">
         <is>
           <t>תשובה ריקה לא מוחקת נתונים טובים</t>
         </is>
       </c>
-      <c r="C86" s="30" t="inlineStr">
+      <c r="C86" s="33" t="inlineStr">
         <is>
           <t>Frontend / Bug Fix</t>
         </is>
       </c>
-      <c r="D86" s="32" t="inlineStr">
+      <c r="D86" s="35" t="inlineStr">
         <is>
           <t>✅ Live (OTA)</t>
         </is>
@@ -3208,22 +3217,22 @@
       </c>
     </row>
     <row r="87">
-      <c r="A87" s="30" t="inlineStr">
+      <c r="A87" s="33" t="inlineStr">
         <is>
           <t>79</t>
         </is>
       </c>
-      <c r="B87" s="31" t="inlineStr">
+      <c r="B87" s="34" t="inlineStr">
         <is>
           <t>תרגום כתבה ישנה דלף לחדשה</t>
         </is>
       </c>
-      <c r="C87" s="30" t="inlineStr">
+      <c r="C87" s="33" t="inlineStr">
         <is>
           <t>Frontend / Bug Fix</t>
         </is>
       </c>
-      <c r="D87" s="32" t="inlineStr">
+      <c r="D87" s="35" t="inlineStr">
         <is>
           <t>✅ Live (OTA)</t>
         </is>
@@ -3240,22 +3249,22 @@
       </c>
     </row>
     <row r="88">
-      <c r="A88" s="30" t="inlineStr">
+      <c r="A88" s="33" t="inlineStr">
         <is>
           <t>80</t>
         </is>
       </c>
-      <c r="B88" s="31" t="inlineStr">
+      <c r="B88" s="34" t="inlineStr">
         <is>
           <t>מרוץ ב"נסה שוב" של פירוט מדד</t>
         </is>
       </c>
-      <c r="C88" s="30" t="inlineStr">
+      <c r="C88" s="33" t="inlineStr">
         <is>
           <t>Frontend / Bug Fix</t>
         </is>
       </c>
-      <c r="D88" s="32" t="inlineStr">
+      <c r="D88" s="35" t="inlineStr">
         <is>
           <t>✅ Live (OTA)</t>
         </is>
@@ -3272,22 +3281,22 @@
       </c>
     </row>
     <row r="89">
-      <c r="A89" s="30" t="inlineStr">
+      <c r="A89" s="33" t="inlineStr">
         <is>
           <t>81</t>
         </is>
       </c>
-      <c r="B89" s="31" t="inlineStr">
+      <c r="B89" s="34" t="inlineStr">
         <is>
           <t>סולם VIX לא מונוטוני</t>
         </is>
       </c>
-      <c r="C89" s="30" t="inlineStr">
+      <c r="C89" s="33" t="inlineStr">
         <is>
           <t>Frontend / i18n</t>
         </is>
       </c>
-      <c r="D89" s="32" t="inlineStr">
+      <c r="D89" s="35" t="inlineStr">
         <is>
           <t>✅ Live (OTA)</t>
         </is>
@@ -3304,22 +3313,22 @@
       </c>
     </row>
     <row r="90">
-      <c r="A90" s="30" t="inlineStr">
+      <c r="A90" s="33" t="inlineStr">
         <is>
           <t>82</t>
         </is>
       </c>
-      <c r="B90" s="31" t="inlineStr">
+      <c r="B90" s="34" t="inlineStr">
         <is>
           <t>תיקוני תוכן בספרדית</t>
         </is>
       </c>
-      <c r="C90" s="30" t="inlineStr">
+      <c r="C90" s="33" t="inlineStr">
         <is>
           <t>i18n / Accuracy</t>
         </is>
       </c>
-      <c r="D90" s="32" t="inlineStr">
+      <c r="D90" s="35" t="inlineStr">
         <is>
           <t>✅ Live (OTA)</t>
         </is>
@@ -3336,22 +3345,22 @@
       </c>
     </row>
     <row r="91">
-      <c r="A91" s="30" t="inlineStr">
+      <c r="A91" s="33" t="inlineStr">
         <is>
           <t>83</t>
         </is>
       </c>
-      <c r="B91" s="31" t="inlineStr">
+      <c r="B91" s="34" t="inlineStr">
         <is>
           <t>Cache-Control: no-store על כל ה-API</t>
         </is>
       </c>
-      <c r="C91" s="30" t="inlineStr">
+      <c r="C91" s="33" t="inlineStr">
         <is>
           <t>Backend / Bug Fix</t>
         </is>
       </c>
-      <c r="D91" s="32" t="inlineStr">
+      <c r="D91" s="35" t="inlineStr">
         <is>
           <t>✅ Live</t>
         </is>
@@ -3368,22 +3377,22 @@
       </c>
     </row>
     <row r="92">
-      <c r="A92" s="30" t="inlineStr">
+      <c r="A92" s="33" t="inlineStr">
         <is>
           <t>84</t>
         </is>
       </c>
-      <c r="B92" s="31" t="inlineStr">
+      <c r="B92" s="34" t="inlineStr">
         <is>
           <t>סדרה שנתית = סוף שנה, לא ינואר</t>
         </is>
       </c>
-      <c r="C92" s="30" t="inlineStr">
+      <c r="C92" s="33" t="inlineStr">
         <is>
           <t>Backend / Bug Fix</t>
         </is>
       </c>
-      <c r="D92" s="32" t="inlineStr">
+      <c r="D92" s="35" t="inlineStr">
         <is>
           <t>✅ Live</t>
         </is>
@@ -3400,22 +3409,22 @@
       </c>
     </row>
     <row r="93">
-      <c r="A93" s="30" t="inlineStr">
+      <c r="A93" s="33" t="inlineStr">
         <is>
           <t>85</t>
         </is>
       </c>
-      <c r="B93" s="31" t="inlineStr">
+      <c r="B93" s="34" t="inlineStr">
         <is>
           <t>TTM של Buyback דרש 2 רבעונים</t>
         </is>
       </c>
-      <c r="C93" s="30" t="inlineStr">
+      <c r="C93" s="33" t="inlineStr">
         <is>
           <t>Backend / Bug Fix</t>
         </is>
       </c>
-      <c r="D93" s="32" t="inlineStr">
+      <c r="D93" s="35" t="inlineStr">
         <is>
           <t>✅ Live</t>
         </is>
@@ -3432,22 +3441,22 @@
       </c>
     </row>
     <row r="94">
-      <c r="A94" s="30" t="inlineStr">
+      <c r="A94" s="33" t="inlineStr">
         <is>
           <t>86</t>
         </is>
       </c>
-      <c r="B94" s="31" t="inlineStr">
+      <c r="B94" s="34" t="inlineStr">
         <is>
           <t>ניקוי ריפו — cloudflared.exe 52MB</t>
         </is>
       </c>
-      <c r="C94" s="30" t="inlineStr">
+      <c r="C94" s="33" t="inlineStr">
         <is>
           <t>DevOps</t>
         </is>
       </c>
-      <c r="D94" s="32" t="inlineStr">
+      <c r="D94" s="35" t="inlineStr">
         <is>
           <t>✅ Live</t>
         </is>
@@ -3464,22 +3473,22 @@
       </c>
     </row>
     <row r="95">
-      <c r="A95" s="30" t="inlineStr">
+      <c r="A95" s="33" t="inlineStr">
         <is>
           <t>87</t>
         </is>
       </c>
-      <c r="B95" s="31" t="inlineStr">
+      <c r="B95" s="34" t="inlineStr">
         <is>
           <t>דיוק עמוד הפרטיות בנוגע ללוגים</t>
         </is>
       </c>
-      <c r="C95" s="30" t="inlineStr">
+      <c r="C95" s="33" t="inlineStr">
         <is>
           <t>Legal</t>
         </is>
       </c>
-      <c r="D95" s="32" t="inlineStr">
+      <c r="D95" s="35" t="inlineStr">
         <is>
           <t>✅ Live</t>
         </is>
@@ -3496,22 +3505,22 @@
       </c>
     </row>
     <row r="96">
-      <c r="A96" s="30" t="inlineStr">
+      <c r="A96" s="33" t="inlineStr">
         <is>
           <t>88</t>
         </is>
       </c>
-      <c r="B96" s="31" t="inlineStr">
+      <c r="B96" s="34" t="inlineStr">
         <is>
           <t>ביקורת קוד מלאה — 35 קבצים</t>
         </is>
       </c>
-      <c r="C96" s="30" t="inlineStr">
+      <c r="C96" s="33" t="inlineStr">
         <is>
           <t>QA</t>
         </is>
       </c>
-      <c r="D96" s="32" t="inlineStr">
+      <c r="D96" s="35" t="inlineStr">
         <is>
           <t>✅ הושלם</t>
         </is>
@@ -3535,22 +3544,22 @@
       </c>
     </row>
     <row r="98">
-      <c r="A98" s="30" t="inlineStr">
+      <c r="A98" s="33" t="inlineStr">
         <is>
           <t>89</t>
         </is>
       </c>
-      <c r="B98" s="31" t="inlineStr">
+      <c r="B98" s="34" t="inlineStr">
         <is>
           <t>צבע הגרף לפי כיוון המדד</t>
         </is>
       </c>
-      <c r="C98" s="30" t="inlineStr">
+      <c r="C98" s="33" t="inlineStr">
         <is>
           <t>Frontend / UX</t>
         </is>
       </c>
-      <c r="D98" s="32" t="inlineStr">
+      <c r="D98" s="35" t="inlineStr">
         <is>
           <t>✅ Live (OTA)</t>
         </is>
@@ -3567,22 +3576,22 @@
       </c>
     </row>
     <row r="99">
-      <c r="A99" s="30" t="inlineStr">
+      <c r="A99" s="33" t="inlineStr">
         <is>
           <t>90</t>
         </is>
       </c>
-      <c r="B99" s="31" t="inlineStr">
+      <c r="B99" s="34" t="inlineStr">
         <is>
           <t>הצהרת טווח מלא לכל 24 המדדים</t>
         </is>
       </c>
-      <c r="C99" s="30" t="inlineStr">
+      <c r="C99" s="33" t="inlineStr">
         <is>
           <t>UX / Accuracy</t>
         </is>
       </c>
-      <c r="D99" s="32" t="inlineStr">
+      <c r="D99" s="35" t="inlineStr">
         <is>
           <t>✅ Live (OTA)</t>
         </is>
@@ -3599,22 +3608,22 @@
       </c>
     </row>
     <row r="100">
-      <c r="A100" s="30" t="inlineStr">
+      <c r="A100" s="33" t="inlineStr">
         <is>
           <t>91</t>
         </is>
       </c>
-      <c r="B100" s="31" t="inlineStr">
+      <c r="B100" s="34" t="inlineStr">
         <is>
           <t>מדד שלא היה לו הסבר בכלל</t>
         </is>
       </c>
-      <c r="C100" s="30" t="inlineStr">
+      <c r="C100" s="33" t="inlineStr">
         <is>
           <t>UX / Bug Fix</t>
         </is>
       </c>
-      <c r="D100" s="32" t="inlineStr">
+      <c r="D100" s="35" t="inlineStr">
         <is>
           <t>✅ Live (OTA)</t>
         </is>
@@ -3631,22 +3640,22 @@
       </c>
     </row>
     <row r="101">
-      <c r="A101" s="30" t="inlineStr">
+      <c r="A101" s="33" t="inlineStr">
         <is>
           <t>92</t>
         </is>
       </c>
-      <c r="B101" s="31" t="inlineStr">
+      <c r="B101" s="34" t="inlineStr">
         <is>
           <t>מספר וכיתוב באותו צבע</t>
         </is>
       </c>
-      <c r="C101" s="30" t="inlineStr">
+      <c r="C101" s="33" t="inlineStr">
         <is>
           <t>Frontend / UX</t>
         </is>
       </c>
-      <c r="D101" s="32" t="inlineStr">
+      <c r="D101" s="35" t="inlineStr">
         <is>
           <t>✅ Live (OTA)</t>
         </is>
@@ -3663,22 +3672,22 @@
       </c>
     </row>
     <row r="102">
-      <c r="A102" s="30" t="inlineStr">
+      <c r="A102" s="33" t="inlineStr">
         <is>
           <t>93</t>
         </is>
       </c>
-      <c r="B102" s="31" t="inlineStr">
+      <c r="B102" s="34" t="inlineStr">
         <is>
           <t>כתום רק כשיש אזהרה</t>
         </is>
       </c>
-      <c r="C102" s="30" t="inlineStr">
+      <c r="C102" s="33" t="inlineStr">
         <is>
           <t>Frontend / UX</t>
         </is>
       </c>
-      <c r="D102" s="32" t="inlineStr">
+      <c r="D102" s="35" t="inlineStr">
         <is>
           <t>✅ Live (OTA)</t>
         </is>
@@ -3695,22 +3704,22 @@
       </c>
     </row>
     <row r="103">
-      <c r="A103" s="30" t="inlineStr">
+      <c r="A103" s="33" t="inlineStr">
         <is>
           <t>94</t>
         </is>
       </c>
-      <c r="B103" s="31" t="inlineStr">
+      <c r="B103" s="34" t="inlineStr">
         <is>
           <t>הצבע שורד את המעבר בין מסכים</t>
         </is>
       </c>
-      <c r="C103" s="30" t="inlineStr">
+      <c r="C103" s="33" t="inlineStr">
         <is>
           <t>Frontend / Bug Fix</t>
         </is>
       </c>
-      <c r="D103" s="32" t="inlineStr">
+      <c r="D103" s="35" t="inlineStr">
         <is>
           <t>✅ Live (OTA)</t>
         </is>
@@ -3727,22 +3736,22 @@
       </c>
     </row>
     <row r="104">
-      <c r="A104" s="30" t="inlineStr">
+      <c r="A104" s="33" t="inlineStr">
         <is>
           <t>95</t>
         </is>
       </c>
-      <c r="B104" s="31" t="inlineStr">
+      <c r="B104" s="34" t="inlineStr">
         <is>
           <t>חומת ההסכמה של גוגל — רוסית וספרדית</t>
         </is>
       </c>
-      <c r="C104" s="30" t="inlineStr">
+      <c r="C104" s="33" t="inlineStr">
         <is>
           <t>Frontend / i18n</t>
         </is>
       </c>
-      <c r="D104" s="32" t="inlineStr">
+      <c r="D104" s="35" t="inlineStr">
         <is>
           <t>✅ Live (OTA)</t>
         </is>
@@ -3759,22 +3768,22 @@
       </c>
     </row>
     <row r="105">
-      <c r="A105" s="30" t="inlineStr">
+      <c r="A105" s="33" t="inlineStr">
         <is>
           <t>96</t>
         </is>
       </c>
-      <c r="B105" s="31" t="inlineStr">
+      <c r="B105" s="34" t="inlineStr">
         <is>
           <t>ביקורת כיסוי-שפות לכל השינויים</t>
         </is>
       </c>
-      <c r="C105" s="30" t="inlineStr">
+      <c r="C105" s="33" t="inlineStr">
         <is>
           <t>QA / i18n</t>
         </is>
       </c>
-      <c r="D105" s="32" t="inlineStr">
+      <c r="D105" s="35" t="inlineStr">
         <is>
           <t>✅ הושלם</t>
         </is>
@@ -3791,22 +3800,22 @@
       </c>
     </row>
     <row r="106">
-      <c r="A106" s="30" t="inlineStr">
+      <c r="A106" s="33" t="inlineStr">
         <is>
           <t>97</t>
         </is>
       </c>
-      <c r="B106" s="31" t="inlineStr">
+      <c r="B106" s="34" t="inlineStr">
         <is>
           <t>מדדים דו-משמעיים — הגרף לא טוען טענה</t>
         </is>
       </c>
-      <c r="C106" s="30" t="inlineStr">
+      <c r="C106" s="33" t="inlineStr">
         <is>
           <t>Frontend / Accuracy</t>
         </is>
       </c>
-      <c r="D106" s="32" t="inlineStr">
+      <c r="D106" s="35" t="inlineStr">
         <is>
           <t>✅ Live (OTA)</t>
         </is>
@@ -3828,48 +3837,43 @@
           <t>98</t>
         </is>
       </c>
-      <c r="B107" s="34" t="inlineStr">
-        <is>
-          <t>צבע הגרף = צבע האריח, לא המגמה</t>
-        </is>
-      </c>
-      <c r="C107" s="33" t="inlineStr">
-        <is>
-          <t>Frontend / UX</t>
-        </is>
-      </c>
-      <c r="D107" s="35" t="inlineStr">
-        <is>
-          <t>✅ Live (OTA)</t>
-        </is>
-      </c>
-      <c r="E107" s="16" t="inlineStr">
-        <is>
-          <t>PriceChart.js, MetricHistoryScreen.js</t>
-        </is>
-      </c>
-      <c r="F107" s="16" t="inlineStr">
-        <is>
-          <t>הגרף צבע לפי מגמה והאריח לפי רמה — שני דברים שיכולים לסתור. P/B שירד מ-14.9 ל-6.84 קיבל קו ירוק ("משתפר") בעוד 6.84 עדיין מעל סף היוקר 5 והאריח צבע אדום. עכשיו הקו נושא את אותו פסק דין; המגמה נראית מצורת הקו. מדד בלי סף ובלי ציון = קו כחול.</t>
-        </is>
-      </c>
     </row>
     <row r="108">
-      <c r="A108" s="3" t="inlineStr">
+      <c r="A108" s="36" t="inlineStr">
+        <is>
+          <t>99</t>
+        </is>
+      </c>
+      <c r="B108" s="37" t="inlineStr">
+        <is>
+          <t>פריסת טאבלט אמיתית</t>
+        </is>
+      </c>
+      <c r="C108" s="36" t="inlineStr">
+        <is>
+          <t>Frontend / Layout</t>
+        </is>
+      </c>
+      <c r="D108" s="38" t="inlineStr">
+        <is>
+          <t>🔜 לא התחיל</t>
+        </is>
+      </c>
+      <c r="E108" s="20" t="inlineStr">
+        <is>
+          <t>HomeScreen.js, FinancialsCard.js, StockScreen.js</t>
+        </is>
+      </c>
+      <c r="F108" s="20" t="inlineStr">
+        <is>
+          <t>נדרש: רוחבי עמודות יחסיים במקום קבועים (COL ב-HomeScreen, 152px/80px ב-FinancialsCard), פריסה דו-טורית בלנדסקייפ, וגדלי גופן שמגיבים למסך. כל סבב בדיקה דורש בילד נייטיב. המלצה: לשחרר לחנות כאפליקציית טלפון ולטפל בטאבלט בגרסה נפרדת.</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="3" t="inlineStr">
         <is>
           <t>🔜  NOT YET STARTED</t>
-        </is>
-      </c>
-      <c r="B108" s="4" t="n"/>
-      <c r="C108" s="4" t="n"/>
-      <c r="D108" s="4" t="n"/>
-      <c r="E108" s="4" t="n"/>
-      <c r="F108" s="5" t="n"/>
-    </row>
-    <row r="109">
-      <c r="A109" s="6" t="inlineStr">
-        <is>
-          <t>19</t>
         </is>
       </c>
       <c r="B109" s="4" t="n"/>
@@ -3879,37 +3883,33 @@
       <c r="F109" s="5" t="n"/>
     </row>
     <row r="110">
-      <c r="A110" s="10" t="inlineStr">
+      <c r="A110" s="6" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="B110" s="4" t="n"/>
+      <c r="C110" s="4" t="n"/>
+      <c r="D110" s="4" t="n"/>
+      <c r="E110" s="4" t="n"/>
+      <c r="F110" s="5" t="n"/>
+    </row>
+    <row r="111">
+      <c r="A111" s="10" t="inlineStr">
         <is>
           <t>Legend</t>
         </is>
       </c>
-    </row>
-    <row r="111">
-      <c r="A111" s="6" t="inlineStr">
-        <is>
-          <t>✅ Live</t>
-        </is>
-      </c>
-      <c r="B111" s="7" t="inlineStr">
-        <is>
-          <t>פרוס ופעיל ב-Render — נראה לכל המשתמשים</t>
-        </is>
-      </c>
-      <c r="C111" s="6" t="inlineStr"/>
-      <c r="D111" s="8" t="inlineStr"/>
-      <c r="E111" s="9" t="inlineStr"/>
-      <c r="F111" s="9" t="inlineStr"/>
     </row>
     <row r="112">
       <c r="A112" s="6" t="inlineStr">
         <is>
-          <t>✅ In APK</t>
+          <t>✅ Live</t>
         </is>
       </c>
       <c r="B112" s="7" t="inlineStr">
         <is>
-          <t>כלול ב-APK המותקן — נראה לכל המשתמשים</t>
+          <t>פרוס ופעיל ב-Render — נראה לכל המשתמשים</t>
         </is>
       </c>
       <c r="C112" s="6" t="inlineStr"/>
@@ -3920,12 +3920,12 @@
     <row r="113">
       <c r="A113" s="6" t="inlineStr">
         <is>
-          <t>⏳ Next APK</t>
+          <t>✅ In APK</t>
         </is>
       </c>
       <c r="B113" s="7" t="inlineStr">
         <is>
-          <t>הקוד מוזג — דורש build ו-APK חדש</t>
+          <t>כלול ב-APK המותקן — נראה לכל המשתמשים</t>
         </is>
       </c>
       <c r="C113" s="6" t="inlineStr"/>
@@ -3936,12 +3936,12 @@
     <row r="114">
       <c r="A114" s="6" t="inlineStr">
         <is>
-          <t>✅ Live (OTA)</t>
+          <t>⏳ Next APK</t>
         </is>
       </c>
       <c r="B114" s="7" t="inlineStr">
         <is>
-          <t>שינוי JS — מועבר אוטומטית בהפעלה הבאה</t>
+          <t>הקוד מוזג — דורש build ו-APK חדש</t>
         </is>
       </c>
       <c r="C114" s="6" t="inlineStr"/>
@@ -3950,42 +3950,50 @@
       <c r="F114" s="9" t="inlineStr"/>
     </row>
     <row r="115">
-      <c r="A115" s="21" t="inlineStr">
-        <is>
-          <t>⏳ ממתין ל-push</t>
-        </is>
-      </c>
-      <c r="B115" s="22" t="inlineStr">
-        <is>
-          <t>הקוד מוכן מקומית — טרם נדחף/נפרס</t>
-        </is>
-      </c>
+      <c r="A115" s="6" t="inlineStr">
+        <is>
+          <t>✅ Live (OTA)</t>
+        </is>
+      </c>
+      <c r="B115" s="7" t="inlineStr">
+        <is>
+          <t>שינוי JS — מועבר אוטומטית בהפעלה הבאה</t>
+        </is>
+      </c>
+      <c r="C115" s="6" t="inlineStr"/>
+      <c r="D115" s="8" t="inlineStr"/>
+      <c r="E115" s="9" t="inlineStr"/>
+      <c r="F115" s="9" t="inlineStr"/>
     </row>
     <row r="116">
       <c r="A116" s="21" t="inlineStr">
         <is>
+          <t>⏳ ממתין ל-push</t>
+        </is>
+      </c>
+      <c r="B116" s="22" t="inlineStr">
+        <is>
+          <t>הקוד מוכן מקומית — טרם נדחף/נפרס</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="21" t="inlineStr">
+        <is>
           <t>⏳ דורש build</t>
         </is>
       </c>
-      <c r="B116" s="22" t="inlineStr">
+      <c r="B117" s="22" t="inlineStr">
         <is>
           <t>שינוי נייטיב — OTA לא מספיק, צריך AAB/APK חדש</t>
         </is>
       </c>
     </row>
-    <row r="117"/>
-    <row r="118">
-      <c r="A118" s="23" t="inlineStr">
+    <row r="118"/>
+    <row r="119">
+      <c r="A119" s="23" t="inlineStr">
         <is>
           <t>סיכום Session 6-7</t>
-        </is>
-      </c>
-    </row>
-    <row r="119">
-      <c r="A119" s="24" t="n"/>
-      <c r="B119" s="25" t="inlineStr">
-        <is>
-          <t>45  —  פריטים חדשים שנוספו (52-96)</t>
         </is>
       </c>
     </row>
@@ -3993,7 +4001,7 @@
       <c r="A120" s="24" t="n"/>
       <c r="B120" s="25" t="inlineStr">
         <is>
-          <t>44  —  חיים בייצור או ב-OTA</t>
+          <t>45  —  פריטים חדשים שנוספו (52-96)</t>
         </is>
       </c>
     </row>
@@ -4001,7 +4009,7 @@
       <c r="A121" s="24" t="n"/>
       <c r="B121" s="25" t="inlineStr">
         <is>
-          <t>1  —  דורש build חדש: תמיכת טאבלט (פריט 68)</t>
+          <t>44  —  חיים בייצור או ב-OTA</t>
         </is>
       </c>
     </row>
@@ -4009,7 +4017,7 @@
       <c r="A122" s="24" t="n"/>
       <c r="B122" s="25" t="inlineStr">
         <is>
-          <t>11,781  —  שורות קוד שנקראו במלואן, 36 קבצים</t>
+          <t>1  —  דורש build חדש: תמיכת טאבלט (פריט 68)</t>
         </is>
       </c>
     </row>
@@ -4017,7 +4025,7 @@
       <c r="A123" s="24" t="n"/>
       <c r="B123" s="25" t="inlineStr">
         <is>
-          <t>29  —  חבילות בדיקה התנהגותיות עוברות</t>
+          <t>11,781  —  שורות קוד שנקראו במלואן, 36 קבצים</t>
         </is>
       </c>
     </row>
@@ -4025,16 +4033,24 @@
       <c r="A124" s="24" t="n"/>
       <c r="B124" s="25" t="inlineStr">
         <is>
+          <t>29  —  חבילות בדיקה התנהגותיות עוברות</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="24" t="n"/>
+      <c r="B125" s="25" t="inlineStr">
+        <is>
           <t>18  —  ראוטים בשרת · 316 מפתחות i18n × 4 שפות</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="4">
+    <mergeCell ref="A97:F97"/>
+    <mergeCell ref="A25:F25"/>
+    <mergeCell ref="A59:F59"/>
     <mergeCell ref="A107:F107"/>
-    <mergeCell ref="A97:F97"/>
-    <mergeCell ref="A59:F59"/>
-    <mergeCell ref="A25:F25"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
London quotes arrive in pence, not pounds - minor-unit handling for GBp/ZAc/ILA
</commit_message>
<xml_diff>
--- a/BuddhaVest_Progress.xlsx
+++ b/BuddhaVest_Progress.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="8">
+  <fonts count="11">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -59,6 +59,18 @@
     <font>
       <name val="Arial"/>
       <b val="1"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
       <sz val="10"/>
     </font>
   </fonts>
@@ -175,7 +187,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="39">
+  <cellXfs count="44">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -276,6 +288,21 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -642,7 +669,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F125"/>
+  <dimension ref="A1:F135"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -663,7 +690,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Last updated: 2026-07-25  |  Session 7</t>
+          <t>Last updated: 2026-07-25  |  Session 8</t>
         </is>
       </c>
     </row>
@@ -2865,22 +2892,22 @@
       </c>
     </row>
     <row r="76">
-      <c r="A76" s="17" t="inlineStr">
+      <c r="A76" s="36" t="inlineStr">
         <is>
           <t>68</t>
         </is>
       </c>
-      <c r="B76" s="18" t="inlineStr">
+      <c r="B76" s="37" t="inlineStr">
         <is>
           <t>הקלה חלקית לטאבלט (לא תמיכה מלאה)</t>
         </is>
       </c>
-      <c r="C76" s="17" t="inlineStr">
+      <c r="C76" s="36" t="inlineStr">
         <is>
           <t>Frontend</t>
         </is>
       </c>
-      <c r="D76" s="19" t="inlineStr">
+      <c r="D76" s="38" t="inlineStr">
         <is>
           <t>⚠️ חלקי</t>
         </is>
@@ -3832,9 +3859,34 @@
       </c>
     </row>
     <row r="107">
-      <c r="A107" s="33" t="inlineStr">
+      <c r="A107" s="39" t="inlineStr">
         <is>
           <t>98</t>
+        </is>
+      </c>
+      <c r="B107" s="40" t="inlineStr">
+        <is>
+          <t>מחוון "טוען" — הבאנר נראה תקוע</t>
+        </is>
+      </c>
+      <c r="C107" s="39" t="inlineStr">
+        <is>
+          <t>Frontend / UX</t>
+        </is>
+      </c>
+      <c r="D107" s="41" t="inlineStr">
+        <is>
+          <t>✅ Live (OTA)</t>
+        </is>
+      </c>
+      <c r="E107" s="42" t="inlineStr">
+        <is>
+          <t>HomeScreen.js, StockScreen.js, i18n.js</t>
+        </is>
+      </c>
+      <c r="F107" s="42" t="inlineStr">
+        <is>
+          <t>הבאנר "טוען נתונים עדכניים" היה טקסט סטטי — משתמש שראה אותו 40 שניות (Render מתעורר) לא ידע אם משהו קורה. נוסף ActivityIndicator לצד הטקסט, עם flexDirection הפוך ב-RTL. בנוסף: ב-StockScreen ה-state wakingUp חושב אך לא הוצג בכלל — קוד מת. 4 שפות.</t>
         </is>
       </c>
     </row>
@@ -3871,186 +3923,495 @@
       </c>
     </row>
     <row r="109">
-      <c r="A109" s="3" t="inlineStr">
-        <is>
-          <t>🔜  NOT YET STARTED</t>
-        </is>
-      </c>
-      <c r="B109" s="4" t="n"/>
-      <c r="C109" s="4" t="n"/>
-      <c r="D109" s="4" t="n"/>
-      <c r="E109" s="4" t="n"/>
-      <c r="F109" s="5" t="n"/>
+      <c r="A109" s="43" t="inlineStr">
+        <is>
+          <t>✅  Session 8 (2026-07-25): מטבע מסחר · מטבע דיווח · יחידות משנה</t>
+        </is>
+      </c>
     </row>
     <row r="110">
-      <c r="A110" s="6" t="inlineStr">
-        <is>
-          <t>19</t>
-        </is>
-      </c>
-      <c r="B110" s="4" t="n"/>
-      <c r="C110" s="4" t="n"/>
-      <c r="D110" s="4" t="n"/>
-      <c r="E110" s="4" t="n"/>
-      <c r="F110" s="5" t="n"/>
+      <c r="A110" s="39" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="B110" s="40" t="inlineStr">
+        <is>
+          <t>לונדון: מחיר גבוה פי 100</t>
+        </is>
+      </c>
+      <c r="C110" s="39" t="inlineStr">
+        <is>
+          <t>Backend / Bug Fix</t>
+        </is>
+      </c>
+      <c r="D110" s="41" t="inlineStr">
+        <is>
+          <t>⏳ ממתין ל-push</t>
+        </is>
+      </c>
+      <c r="E110" s="42" t="inlineStr">
+        <is>
+          <t>main.py</t>
+        </is>
+      </c>
+      <c r="F110" s="42" t="inlineStr">
+        <is>
+          <t>Yahoo מצטטת מניות בבורסת לונדון בפֶּנס ומסמנת זאת בשדה currency כ-"GBp" — באות p קטנה, כשהערך "GBP" פירושו לירות. הקוד הריץ .upper() לפני כל השוואה ומחק בכך את ההבחנה היחידה, כך שמניית Shell במחיר 2578.5 פנס היתה מוצגת "£2578.50" במקום "£25.79". אותה משפחת באג כמו האגורות בת"א, רק שלת"א היה טיפול ולונדון לא. הערה על רמת הראיה: הבאג אותר מקריאת הקוד ומתועד במקורות חיצוניים, אך לא הורץ מול ה-API החי — לסביבת הבדיקה אין יציאה לרשת כרגע. דורש אימות ידני על מניה בלונדון אחרי ה-push.</t>
+        </is>
+      </c>
     </row>
     <row r="111">
-      <c r="A111" s="10" t="inlineStr">
+      <c r="A111" s="39" t="inlineStr">
+        <is>
+          <t>101</t>
+        </is>
+      </c>
+      <c r="B111" s="40" t="inlineStr">
+        <is>
+          <t>טבלת יחידות משנה במקום מקרה פרטי</t>
+        </is>
+      </c>
+      <c r="C111" s="39" t="inlineStr">
+        <is>
+          <t>Backend / Architecture</t>
+        </is>
+      </c>
+      <c r="D111" s="41" t="inlineStr">
+        <is>
+          <t>⏳ ממתין ל-push</t>
+        </is>
+      </c>
+      <c r="E111" s="42" t="inlineStr">
+        <is>
+          <t>main.py</t>
+        </is>
+      </c>
+      <c r="F111" s="42" t="inlineStr">
+        <is>
+          <t>_MINOR_UNIT ממפה GBp/GBX (פנס) · ZAc (סנט דרום-אפריקאי) · ILA (אגורות) אל המטבע הראשי והמחלק. המפתחות רגישים לאותיות גדולות/קטנות במכוון — "GBP" ו-"ZAR" חייבים להישאר בחוץ, כי המרה שלהם היתה יוצרת שגיאת פי-100 בכיוון ההפוך. 9 בדיקות רגישות-אותיות.</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="39" t="inlineStr">
+        <is>
+          <t>102</t>
+        </is>
+      </c>
+      <c r="B112" s="40" t="inlineStr">
+        <is>
+          <t>חלוקה רק לשדות של מחיר למניה</t>
+        </is>
+      </c>
+      <c r="C112" s="39" t="inlineStr">
+        <is>
+          <t>Backend / Accuracy</t>
+        </is>
+      </c>
+      <c r="D112" s="41" t="inlineStr">
+        <is>
+          <t>⏳ ממתין ל-push</t>
+        </is>
+      </c>
+      <c r="E112" s="42" t="inlineStr">
+        <is>
+          <t>main.py</t>
+        </is>
+      </c>
+      <c r="F112" s="42" t="inlineStr">
+        <is>
+          <t>_scale_price_fields מחלק מחיר נוכחי, שיא/שפל 52 שבועות וסדרת הגרף — ולא נוגע בשווי שוק, הכנסות, רווח נקי ומזומנים, שכבר מדווחים במטבע הראשי. האסימטריה הזו אומתה בת"א ותקפה גם בלונדון. הפונקציה משותפת לשני המסלולים כדי שלא יוכלו להיפרד שוב.</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="39" t="inlineStr">
+        <is>
+          <t>103</t>
+        </is>
+      </c>
+      <c r="B113" s="40" t="inlineStr">
+        <is>
+          <t>מכפילים שנגזרים ממחיר — דיכוי מורחב</t>
+        </is>
+      </c>
+      <c r="C113" s="39" t="inlineStr">
+        <is>
+          <t>Backend / Accuracy</t>
+        </is>
+      </c>
+      <c r="D113" s="41" t="inlineStr">
+        <is>
+          <t>⏳ ממתין ל-push</t>
+        </is>
+      </c>
+      <c r="E113" s="42" t="inlineStr">
+        <is>
+          <t>main.py</t>
+        </is>
+      </c>
+      <c r="F113" s="42" t="inlineStr">
+        <is>
+          <t>המכפילים ההיסטוריים (P/B, P/S, EV/EBITDA, Forward P/E) מחושבים מ-history()["Close"], שמגיע ביחידת המשנה, מול דוחות ביחידה הראשית. הדיכוי שהיה קיים ל-.TA בלבד הורחב ל-.L ול-.JO. false positive עולה גרף, false negative מפרסם מספר שגוי פי 100 — לכן הכיוון השמרני.</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="39" t="inlineStr">
+        <is>
+          <t>104</t>
+        </is>
+      </c>
+      <c r="B114" s="40" t="inlineStr">
+        <is>
+          <t>/quotes — אותו כלל כמו /analyze</t>
+        </is>
+      </c>
+      <c r="C114" s="39" t="inlineStr">
+        <is>
+          <t>Backend / Bug Fix</t>
+        </is>
+      </c>
+      <c r="D114" s="41" t="inlineStr">
+        <is>
+          <t>⏳ ממתין ל-push</t>
+        </is>
+      </c>
+      <c r="E114" s="42" t="inlineStr">
+        <is>
+          <t>main.py</t>
+        </is>
+      </c>
+      <c r="F114" s="42" t="inlineStr">
+        <is>
+          <t>רשימת המעקב צובעת מסך ראשון מ-/quotes ורק אז מחליפה בניתוח המלא. בלי אותו כלל, מניה בלונדון היתה מהבהבת מחיר פי-100 לרגע — בדיוק מה שקרה עם דלק (8173 במקום 81.73). כולל אתחול ccy_raw מחוץ ל-try, אחרת כשל רשת היה מפיל NameError.</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="39" t="inlineStr">
+        <is>
+          <t>105</t>
+        </is>
+      </c>
+      <c r="B115" s="40" t="inlineStr">
+        <is>
+          <t>סכום הדיבידנד עצמו</t>
+        </is>
+      </c>
+      <c r="C115" s="39" t="inlineStr">
+        <is>
+          <t>Backend / Bug Fix</t>
+        </is>
+      </c>
+      <c r="D115" s="41" t="inlineStr">
+        <is>
+          <t>⏳ ממתין ל-push</t>
+        </is>
+      </c>
+      <c r="E115" s="42" t="inlineStr">
+        <is>
+          <t>main.py</t>
+        </is>
+      </c>
+      <c r="F115" s="42" t="inlineStr">
+        <is>
+          <t>dividendRate מגיע במטבע ההצעה, כך שדיבידנד של 104 פנס היה מוצג "£104.00" במקום "£1.04". בנוסף הסימן היה ניחוש דו-כיווני ₪/$ בלבד — משלמת דיבידנד ביורו קיבלה סימן דולר באירוע בזמן שהכותרת הראתה €.</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="39" t="inlineStr">
+        <is>
+          <t>106</t>
+        </is>
+      </c>
+      <c r="B116" s="40" t="inlineStr">
+        <is>
+          <t>סימני מטבע — מקור אמת אחד</t>
+        </is>
+      </c>
+      <c r="C116" s="39" t="inlineStr">
+        <is>
+          <t>Frontend / Architecture</t>
+        </is>
+      </c>
+      <c r="D116" s="41" t="inlineStr">
+        <is>
+          <t>⏳ ממתין ל-push</t>
+        </is>
+      </c>
+      <c r="E116" s="42" t="inlineStr">
+        <is>
+          <t>utils/currency.js (חדש), StockScreen.js, WatchlistScreen.js</t>
+        </is>
+      </c>
+      <c r="F116" s="42" t="inlineStr">
+        <is>
+          <t>symbolFor היתה מועתקת ידנית בשני מסכים והספיקה כבר להתיישן: אף אחת מהן לא הכירה ין, ולונדון היתה דורשת לזכור לערוך את שתיהן. אותה מניה עם סימן אחד בשורת המעקב וסימן אחר בעמוד שלה הוא בדיוק הבאג שהקובץ הזה מונע. 22 מטבעות, מסונכרן מול _CCY_SYMBOL בשרת ונבדק צמד-צמד.</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="39" t="inlineStr">
+        <is>
+          <t>107</t>
+        </is>
+      </c>
+      <c r="B117" s="40" t="inlineStr">
+        <is>
+          <t>isUsd — השורה המשנית</t>
+        </is>
+      </c>
+      <c r="C117" s="39" t="inlineStr">
+        <is>
+          <t>Frontend / Bug Fix</t>
+        </is>
+      </c>
+      <c r="D117" s="41" t="inlineStr">
+        <is>
+          <t>⏳ ממתין ל-push</t>
+        </is>
+      </c>
+      <c r="E117" s="42" t="inlineStr">
+        <is>
+          <t>utils/currency.js, StockScreen.js, WatchlistScreen.js</t>
+        </is>
+      </c>
+      <c r="F117" s="42" t="inlineStr">
+        <is>
+          <t>שער ההמרה הוא דולר→מקומי, ולכן השורה המשנית תקפה רק כשהמחיר עצמו בדולר. הבדיקה "לא שקל" נתנה למניה ביורו לעבור והכפילה אותה בשער הדולר. בדיקה חיובית ל-USD במקום שלילית לשקל, בפונקציה אחת משותפת.</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="39" t="inlineStr">
+        <is>
+          <t>108</t>
+        </is>
+      </c>
+      <c r="B118" s="40" t="inlineStr">
+        <is>
+          <t>אימות חוצה-בורסות</t>
+        </is>
+      </c>
+      <c r="C118" s="39" t="inlineStr">
+        <is>
+          <t>QA</t>
+        </is>
+      </c>
+      <c r="D118" s="41" t="inlineStr">
+        <is>
+          <t>✅ הושלם</t>
+        </is>
+      </c>
+      <c r="E118" s="42" t="inlineStr">
+        <is>
+          <t>outputs/verify_minor_units.py, verify_multi_currency.js</t>
+        </is>
+      </c>
+      <c r="F118" s="42" t="inlineStr">
+        <is>
+          <t>חמש בורסות אומתו חי מול ה-API בסבבים קודמים: WMT ו-RIVN (דולר), ESLT.TA (נסחרת בשקל, מדווחת בדולר), DLEKG.TA (שקל), DHER.DE (יורו) — כל אחת חשפה מחלקה אחרת של באג. לונדון ויוהנסבורג נבדקו ביחידה בלבד (40 טענות: רגישות אותיות, שדות ריקים, אי-נגיעה בשווי שוק, סכום דיבידנד, התאמת סימנים שרת↔לקוח) ולא מול ה-API החי.</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="39" t="inlineStr">
+        <is>
+          <t>109</t>
+        </is>
+      </c>
+      <c r="B119" s="40" t="inlineStr">
+        <is>
+          <t>תיקון רתמת הבדיקות עצמה</t>
+        </is>
+      </c>
+      <c r="C119" s="39" t="inlineStr">
+        <is>
+          <t>QA</t>
+        </is>
+      </c>
+      <c r="D119" s="41" t="inlineStr">
+        <is>
+          <t>✅ הושלם</t>
+        </is>
+      </c>
+      <c r="E119" s="42" t="inlineStr">
+        <is>
+          <t>outputs/verify_analyzer_fixes.py, outputs/snapshots/</t>
+        </is>
+      </c>
+      <c r="F119" s="42" t="inlineStr">
+        <is>
+          <t>ההרצה דיווחה 5 כשלים שאף אחד מהם לא היה רגרסיה: 4 קבצים היו העתקי קוד מקור לבדיקת קומפילציה שהורצו בטעות כטסטים (הועברו ל-snapshots/), ואחד הכיל טענה שגויה שלי — היא בדקה תווית במקום את זוג הרבעונים שהלוגיקה הישנה קראה, והתווית יצאה נכונה במקרה. רתמה ששקרה בשני הכיוונים תוקנה.</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="10" t="inlineStr">
         <is>
           <t>Legend</t>
         </is>
       </c>
     </row>
-    <row r="112">
-      <c r="A112" s="6" t="inlineStr">
+    <row r="121">
+      <c r="A121" s="6" t="inlineStr">
         <is>
           <t>✅ Live</t>
         </is>
       </c>
-      <c r="B112" s="7" t="inlineStr">
+      <c r="B121" s="7" t="inlineStr">
         <is>
           <t>פרוס ופעיל ב-Render — נראה לכל המשתמשים</t>
         </is>
       </c>
-      <c r="C112" s="6" t="inlineStr"/>
-      <c r="D112" s="8" t="inlineStr"/>
-      <c r="E112" s="9" t="inlineStr"/>
-      <c r="F112" s="9" t="inlineStr"/>
-    </row>
-    <row r="113">
-      <c r="A113" s="6" t="inlineStr">
+      <c r="C121" s="6" t="inlineStr"/>
+      <c r="D121" s="8" t="inlineStr"/>
+      <c r="E121" s="9" t="inlineStr"/>
+      <c r="F121" s="9" t="inlineStr"/>
+    </row>
+    <row r="122">
+      <c r="A122" s="6" t="inlineStr">
         <is>
           <t>✅ In APK</t>
         </is>
       </c>
-      <c r="B113" s="7" t="inlineStr">
+      <c r="B122" s="7" t="inlineStr">
         <is>
           <t>כלול ב-APK המותקן — נראה לכל המשתמשים</t>
         </is>
       </c>
-      <c r="C113" s="6" t="inlineStr"/>
-      <c r="D113" s="8" t="inlineStr"/>
-      <c r="E113" s="9" t="inlineStr"/>
-      <c r="F113" s="9" t="inlineStr"/>
-    </row>
-    <row r="114">
-      <c r="A114" s="6" t="inlineStr">
+      <c r="C122" s="6" t="inlineStr"/>
+      <c r="D122" s="8" t="inlineStr"/>
+      <c r="E122" s="9" t="inlineStr"/>
+      <c r="F122" s="9" t="inlineStr"/>
+    </row>
+    <row r="123">
+      <c r="A123" s="6" t="inlineStr">
         <is>
           <t>⏳ Next APK</t>
         </is>
       </c>
-      <c r="B114" s="7" t="inlineStr">
+      <c r="B123" s="7" t="inlineStr">
         <is>
           <t>הקוד מוזג — דורש build ו-APK חדש</t>
         </is>
       </c>
-      <c r="C114" s="6" t="inlineStr"/>
-      <c r="D114" s="8" t="inlineStr"/>
-      <c r="E114" s="9" t="inlineStr"/>
-      <c r="F114" s="9" t="inlineStr"/>
-    </row>
-    <row r="115">
-      <c r="A115" s="6" t="inlineStr">
+      <c r="C123" s="6" t="inlineStr"/>
+      <c r="D123" s="8" t="inlineStr"/>
+      <c r="E123" s="9" t="inlineStr"/>
+      <c r="F123" s="9" t="inlineStr"/>
+    </row>
+    <row r="124">
+      <c r="A124" s="6" t="inlineStr">
         <is>
           <t>✅ Live (OTA)</t>
         </is>
       </c>
-      <c r="B115" s="7" t="inlineStr">
+      <c r="B124" s="7" t="inlineStr">
         <is>
           <t>שינוי JS — מועבר אוטומטית בהפעלה הבאה</t>
         </is>
       </c>
-      <c r="C115" s="6" t="inlineStr"/>
-      <c r="D115" s="8" t="inlineStr"/>
-      <c r="E115" s="9" t="inlineStr"/>
-      <c r="F115" s="9" t="inlineStr"/>
-    </row>
-    <row r="116">
-      <c r="A116" s="21" t="inlineStr">
+      <c r="C124" s="6" t="inlineStr"/>
+      <c r="D124" s="8" t="inlineStr"/>
+      <c r="E124" s="9" t="inlineStr"/>
+      <c r="F124" s="9" t="inlineStr"/>
+    </row>
+    <row r="125">
+      <c r="A125" s="21" t="inlineStr">
         <is>
           <t>⏳ ממתין ל-push</t>
         </is>
       </c>
-      <c r="B116" s="22" t="inlineStr">
+      <c r="B125" s="22" t="inlineStr">
         <is>
           <t>הקוד מוכן מקומית — טרם נדחף/נפרס</t>
         </is>
       </c>
     </row>
-    <row r="117">
-      <c r="A117" s="21" t="inlineStr">
+    <row r="126">
+      <c r="A126" s="21" t="inlineStr">
         <is>
           <t>⏳ דורש build</t>
         </is>
       </c>
-      <c r="B117" s="22" t="inlineStr">
+      <c r="B126" s="22" t="inlineStr">
         <is>
           <t>שינוי נייטיב — OTA לא מספיק, צריך AAB/APK חדש</t>
         </is>
       </c>
     </row>
-    <row r="118"/>
-    <row r="119">
-      <c r="A119" s="23" t="inlineStr">
-        <is>
-          <t>סיכום Session 6-7</t>
-        </is>
-      </c>
-    </row>
-    <row r="120">
-      <c r="A120" s="24" t="n"/>
-      <c r="B120" s="25" t="inlineStr">
-        <is>
-          <t>45  —  פריטים חדשים שנוספו (52-96)</t>
-        </is>
-      </c>
-    </row>
-    <row r="121">
-      <c r="A121" s="24" t="n"/>
-      <c r="B121" s="25" t="inlineStr">
-        <is>
-          <t>44  —  חיים בייצור או ב-OTA</t>
-        </is>
-      </c>
-    </row>
-    <row r="122">
-      <c r="A122" s="24" t="n"/>
-      <c r="B122" s="25" t="inlineStr">
-        <is>
-          <t>1  —  דורש build חדש: תמיכת טאבלט (פריט 68)</t>
-        </is>
-      </c>
-    </row>
-    <row r="123">
-      <c r="A123" s="24" t="n"/>
-      <c r="B123" s="25" t="inlineStr">
-        <is>
-          <t>11,781  —  שורות קוד שנקראו במלואן, 36 קבצים</t>
-        </is>
-      </c>
-    </row>
-    <row r="124">
-      <c r="A124" s="24" t="n"/>
-      <c r="B124" s="25" t="inlineStr">
-        <is>
-          <t>29  —  חבילות בדיקה התנהגותיות עוברות</t>
-        </is>
-      </c>
-    </row>
-    <row r="125">
-      <c r="A125" s="24" t="n"/>
-      <c r="B125" s="25" t="inlineStr">
-        <is>
-          <t>18  —  ראוטים בשרת · 316 מפתחות i18n × 4 שפות</t>
+    <row r="128">
+      <c r="A128" s="23" t="inlineStr">
+        <is>
+          <t>סיכום Session 6-8</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="24" t="n"/>
+      <c r="B129" s="25" t="inlineStr">
+        <is>
+          <t>58  —  פריטים חדשים שנוספו (52-109)</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="24" t="n"/>
+      <c r="B130" s="25" t="inlineStr">
+        <is>
+          <t>48  —  חיים בייצור או ב-OTA</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="24" t="n"/>
+      <c r="B131" s="25" t="inlineStr">
+        <is>
+          <t>8  —  מוכנים מקומית, ממתינים ל-push (100-107)</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" s="24" t="n"/>
+      <c r="B132" s="25" t="inlineStr">
+        <is>
+          <t>2  —  פתוחים: פריסת טאבלט אמיתית (99) · הגשה ל-Play (19)</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" s="24" t="n"/>
+      <c r="B133" s="25" t="inlineStr">
+        <is>
+          <t>5  —  בורסות שאומתו חי · 2 נוספות (לונדון, יוהנסבורג) ביחידה בלבד</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" s="24" t="n"/>
+      <c r="B134" s="25" t="inlineStr">
+        <is>
+          <t>48  —  חבילות בדיקה התנהגותיות עוברות (48/48)</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>18  —  ראוטים בשרת · 324 מפתחות i18n × 4 שפות</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="4">
     <mergeCell ref="A97:F97"/>
+    <mergeCell ref="A109:F109"/>
+    <mergeCell ref="A59:F59"/>
     <mergeCell ref="A25:F25"/>
-    <mergeCell ref="A59:F59"/>
-    <mergeCell ref="A107:F107"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Session 8 tracker: London minor-unit fix verified live
</commit_message>
<xml_diff>
--- a/BuddhaVest_Progress.xlsx
+++ b/BuddhaVest_Progress.xlsx
@@ -3947,7 +3947,7 @@
       </c>
       <c r="D110" s="41" t="inlineStr">
         <is>
-          <t>⏳ ממתין ל-push</t>
+          <t>✅ Live</t>
         </is>
       </c>
       <c r="E110" s="42" t="inlineStr">
@@ -3957,7 +3957,7 @@
       </c>
       <c r="F110" s="42" t="inlineStr">
         <is>
-          <t>Yahoo מצטטת מניות בבורסת לונדון בפֶּנס ומסמנת זאת בשדה currency כ-"GBp" — באות p קטנה, כשהערך "GBP" פירושו לירות. הקוד הריץ .upper() לפני כל השוואה ומחק בכך את ההבחנה היחידה, כך שמניית Shell במחיר 2578.5 פנס היתה מוצגת "£2578.50" במקום "£25.79". אותה משפחת באג כמו האגורות בת"א, רק שלת"א היה טיפול ולונדון לא. הערה על רמת הראיה: הבאג אותר מקריאת הקוד ומתועד במקורות חיצוניים, אך לא הורץ מול ה-API החי — לסביבת הבדיקה אין יציאה לרשת כרגע. דורש אימות ידני על מניה בלונדון אחרי ה-push.</t>
+          <t>Yahoo מצטטת מניות בבורסת לונדון בפֶּנס ומסמנת זאת בשדה currency כ-"GBp" — באות p קטנה, כשהערך "GBP" פירושו לירות. הקוד הריץ .upper() לפני כל השוואה ומחק בכך את ההבחנה היחידה. אומת חי לפני ולאחר: SHEL.L החזירה 3262.07 עם price_currency "USD" (האפליקציה הציגה "$3262.07"), ולאחר הפריסה 32.62 עם "GBP". גם BP.L 531.7→5.32 ו-ULVR.L 5027→50.27. אותה משפחת באג כמו האגורות בת"א, רק שלת"א היה טיפול ולונדון לא.</t>
         </is>
       </c>
     </row>
@@ -3979,7 +3979,7 @@
       </c>
       <c r="D111" s="41" t="inlineStr">
         <is>
-          <t>⏳ ממתין ל-push</t>
+          <t>✅ Live</t>
         </is>
       </c>
       <c r="E111" s="42" t="inlineStr">
@@ -4011,7 +4011,7 @@
       </c>
       <c r="D112" s="41" t="inlineStr">
         <is>
-          <t>⏳ ממתין ל-push</t>
+          <t>✅ Live</t>
         </is>
       </c>
       <c r="E112" s="42" t="inlineStr">
@@ -4043,7 +4043,7 @@
       </c>
       <c r="D113" s="41" t="inlineStr">
         <is>
-          <t>⏳ ממתין ל-push</t>
+          <t>✅ Live</t>
         </is>
       </c>
       <c r="E113" s="42" t="inlineStr">
@@ -4075,7 +4075,7 @@
       </c>
       <c r="D114" s="41" t="inlineStr">
         <is>
-          <t>⏳ ממתין ל-push</t>
+          <t>✅ Live</t>
         </is>
       </c>
       <c r="E114" s="42" t="inlineStr">
@@ -4107,7 +4107,7 @@
       </c>
       <c r="D115" s="41" t="inlineStr">
         <is>
-          <t>⏳ ממתין ל-push</t>
+          <t>✅ Live</t>
         </is>
       </c>
       <c r="E115" s="42" t="inlineStr">
@@ -4139,7 +4139,7 @@
       </c>
       <c r="D116" s="41" t="inlineStr">
         <is>
-          <t>⏳ ממתין ל-push</t>
+          <t>✅ Live (OTA)</t>
         </is>
       </c>
       <c r="E116" s="42" t="inlineStr">
@@ -4171,7 +4171,7 @@
       </c>
       <c r="D117" s="41" t="inlineStr">
         <is>
-          <t>⏳ ממתין ל-push</t>
+          <t>✅ Live (OTA)</t>
         </is>
       </c>
       <c r="E117" s="42" t="inlineStr">
@@ -4213,7 +4213,7 @@
       </c>
       <c r="F118" s="42" t="inlineStr">
         <is>
-          <t>חמש בורסות אומתו חי מול ה-API בסבבים קודמים: WMT ו-RIVN (דולר), ESLT.TA (נסחרת בשקל, מדווחת בדולר), DLEKG.TA (שקל), DHER.DE (יורו) — כל אחת חשפה מחלקה אחרת של באג. לונדון ויוהנסבורג נבדקו ביחידה בלבד (40 טענות: רגישות אותיות, שדות ריקים, אי-נגיעה בשווי שוק, סכום דיבידנד, התאמת סימנים שרת↔לקוח) ולא מול ה-API החי.</t>
+          <t>שבע בורסות אומתו חי מול ה-API: WMT ו-RIVN (דולר), ESLT.TA (נסחרת בשקל, מדווחת בדולר), DLEKG.TA (שקל), DHER.DE (יורו), ולאחר הפריסה SHEL.L · BP.L · ULVR.L (לונדון, פנס). בקריאה אחת אחרי הפריסה: SHEL.L £32.62 · BP.L £5.32 · ULVR.L £50.27 · WMT $114.96 · DHER.DE €37.88 · DLEKG.TA ₪83.51 — כל אחת עם המטבע הנכון שלה. יוהנסבורג (ZAc) מכוסה ביחידה בלבד, אין מניה לבדוק. בנוסף 40 טענות יחידה: רגישות אותיות, שדות ריקים, אי-נגיעה בשווי שוק, סכום דיבידנד, התאמת סימנים שרת↔לקוח.</t>
         </is>
       </c>
     </row>
@@ -4363,7 +4363,7 @@
       <c r="A130" s="24" t="n"/>
       <c r="B130" s="25" t="inlineStr">
         <is>
-          <t>48  —  חיים בייצור או ב-OTA</t>
+          <t>56  —  חיים בייצור או ב-OTA</t>
         </is>
       </c>
     </row>
@@ -4371,7 +4371,7 @@
       <c r="A131" s="24" t="n"/>
       <c r="B131" s="25" t="inlineStr">
         <is>
-          <t>8  —  מוכנים מקומית, ממתינים ל-push (100-107)</t>
+          <t>0  —  ממתינים ל-push: הכל נפרס (commit 91ee6d3)</t>
         </is>
       </c>
     </row>
@@ -4387,7 +4387,7 @@
       <c r="A133" s="24" t="n"/>
       <c r="B133" s="25" t="inlineStr">
         <is>
-          <t>5  —  בורסות שאומתו חי · 2 נוספות (לונדון, יוהנסבורג) ביחידה בלבד</t>
+          <t>8  —  בורסות שאומתו חי (NYSE · TASE · XETRA · LSE) · JSE ביחידה בלבד</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Privacy page cache fix
</commit_message>
<xml_diff>
--- a/BuddhaVest_Progress.xlsx
+++ b/BuddhaVest_Progress.xlsx
@@ -187,7 +187,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="44">
+  <cellXfs count="51">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -303,6 +303,27 @@
     </xf>
     <xf numFmtId="0" fontId="10" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -669,7 +690,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F135"/>
+  <dimension ref="A1:F139"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -690,7 +711,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Last updated: 2026-07-25  |  Session 8</t>
+          <t>Last updated: 2026-08-03  |  Session 9</t>
         </is>
       </c>
     </row>
@@ -4250,136 +4271,233 @@
       </c>
     </row>
     <row r="120">
-      <c r="A120" s="10" t="inlineStr">
+      <c r="A120" s="44" t="inlineStr">
+        <is>
+          <t>110</t>
+        </is>
+      </c>
+      <c r="B120" s="45" t="inlineStr">
+        <is>
+          <t>עמוד הפרטיות הוגש מהמטמון</t>
+        </is>
+      </c>
+      <c r="C120" s="44" t="inlineStr">
+        <is>
+          <t>Backend / Legal / Bug Fix</t>
+        </is>
+      </c>
+      <c r="D120" s="46" t="inlineStr">
+        <is>
+          <t>⏳ ממתין ל-push</t>
+        </is>
+      </c>
+      <c r="E120" s="47" t="inlineStr">
+        <is>
+          <t>main.py</t>
+        </is>
+      </c>
+      <c r="F120" s="47" t="inlineStr">
+        <is>
+          <t>המידלוור שמונע מטמון החריג במפורש את /privacy, מתוך הנחה שדף משפטי סטטי כדאי לשמור. ההנחה היתה הפוכה. אומת חי: הכתובת הרגילה החזירה את הנוסח הישן ("the watchlist is never transmitted to our servers") בעוד שאותה כתובת עם פרמטר שאילתה חדש החזירה את המתוקן — כלומר הקוד תקין והתשובה נתקעה במטמון. גוגל משווה את הדף להצהרת Data Safety, כך שעותק ישן היה יוצר סתירה מולם. החריג הוסר; כל נתיב מקבל no-store.</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="48" t="inlineStr">
+        <is>
+          <t>111</t>
+        </is>
+      </c>
+      <c r="B121" s="49" t="inlineStr">
+        <is>
+          <t>טופס Data Safety מולא</t>
+        </is>
+      </c>
+      <c r="C121" s="48" t="inlineStr">
+        <is>
+          <t>Store / Legal</t>
+        </is>
+      </c>
+      <c r="D121" s="50" t="inlineStr">
+        <is>
+          <t>✅ הושלם</t>
+        </is>
+      </c>
+      <c r="E121" s="42" t="inlineStr">
+        <is>
+          <t>data-safety-answers.html</t>
+        </is>
+      </c>
+      <c r="F121" s="42" t="inlineStr">
+        <is>
+          <t>5 סוגי נתונים הוצהרו: אינטראקציות באפליקציה · היסטוריית חיפוש · תוכן שנוצר על ידי משתמשים · גלישה באינטרנט · מזהה המכשיר. כולם נאספים, אף אחד לא משותף, אף אחד לא זמני, מטרה יחידה פונקציונליות. לא הוצהרו: מידע אישי, פיננסי, מיקום, בריאות, אנשי קשר, קראש-לוגים — כל אחד אומת מול המניפסט ומול 19 התלויות. יומן המחקר לא הוצהר כי buddhavest_journal אף פעם לא מופיע בתוך fetch.</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="48" t="inlineStr">
+        <is>
+          <t>112</t>
+        </is>
+      </c>
+      <c r="B122" s="49" t="inlineStr">
+        <is>
+          <t>צ׳קליסט טפסי Play Console</t>
+        </is>
+      </c>
+      <c r="C122" s="48" t="inlineStr">
+        <is>
+          <t>Store</t>
+        </is>
+      </c>
+      <c r="D122" s="50" t="inlineStr">
+        <is>
+          <t>✅ הושלם</t>
+        </is>
+      </c>
+      <c r="E122" s="42" t="inlineStr">
+        <is>
+          <t>play-console-checklist.html</t>
+        </is>
+      </c>
+      <c r="F122" s="42" t="inlineStr">
+        <is>
+          <t>תשובות לכל סעיפי App content שנותרו: גישה לאפליקציה, מודעות, דירוג תוכן, קהל יעד, תכונות פיננסיות, אפליקציית חדשות, בריאות, ממשלה, הרשאות רגישות. שתי ההצהרות הרגישות באפליקציה מסוג זה — "תכונות פיננסיות" ו"אפליקציית חדשות" — מנומקות בנפרד.</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="44" t="inlineStr">
+        <is>
+          <t>113</t>
+        </is>
+      </c>
+      <c r="B123" s="45" t="inlineStr">
+        <is>
+          <t>צילומי מסך לחנות</t>
+        </is>
+      </c>
+      <c r="C123" s="44" t="inlineStr">
+        <is>
+          <t>Store</t>
+        </is>
+      </c>
+      <c r="D123" s="46" t="inlineStr">
+        <is>
+          <t>🔜 לא התחיל</t>
+        </is>
+      </c>
+      <c r="E123" s="47" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F123" s="47" t="inlineStr">
+        <is>
+          <t>הפער היחיד שנותר בדף החנות. גוגל דורשת לפחות 2 צילומי טלפון, מומלץ 4-8. אייקון ו-feature graphic כבר קיימים במידות הנכונות (1024x1024 ו-1024x500). מדריך מוכן ב-מדריך-צילומי-מסך-לחנות.html.</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="10" t="inlineStr">
         <is>
           <t>Legend</t>
         </is>
       </c>
     </row>
-    <row r="121">
-      <c r="A121" s="6" t="inlineStr">
+    <row r="125">
+      <c r="A125" s="6" t="inlineStr">
         <is>
           <t>✅ Live</t>
         </is>
       </c>
-      <c r="B121" s="7" t="inlineStr">
+      <c r="B125" s="7" t="inlineStr">
         <is>
           <t>פרוס ופעיל ב-Render — נראה לכל המשתמשים</t>
         </is>
       </c>
-      <c r="C121" s="6" t="inlineStr"/>
-      <c r="D121" s="8" t="inlineStr"/>
-      <c r="E121" s="9" t="inlineStr"/>
-      <c r="F121" s="9" t="inlineStr"/>
-    </row>
-    <row r="122">
-      <c r="A122" s="6" t="inlineStr">
+      <c r="C125" s="6" t="inlineStr"/>
+      <c r="D125" s="8" t="inlineStr"/>
+      <c r="E125" s="9" t="inlineStr"/>
+      <c r="F125" s="9" t="inlineStr"/>
+    </row>
+    <row r="126">
+      <c r="A126" s="6" t="inlineStr">
         <is>
           <t>✅ In APK</t>
         </is>
       </c>
-      <c r="B122" s="7" t="inlineStr">
+      <c r="B126" s="7" t="inlineStr">
         <is>
           <t>כלול ב-APK המותקן — נראה לכל המשתמשים</t>
         </is>
       </c>
-      <c r="C122" s="6" t="inlineStr"/>
-      <c r="D122" s="8" t="inlineStr"/>
-      <c r="E122" s="9" t="inlineStr"/>
-      <c r="F122" s="9" t="inlineStr"/>
-    </row>
-    <row r="123">
-      <c r="A123" s="6" t="inlineStr">
+      <c r="C126" s="6" t="inlineStr"/>
+      <c r="D126" s="8" t="inlineStr"/>
+      <c r="E126" s="9" t="inlineStr"/>
+      <c r="F126" s="9" t="inlineStr"/>
+    </row>
+    <row r="127">
+      <c r="A127" s="6" t="inlineStr">
         <is>
           <t>⏳ Next APK</t>
         </is>
       </c>
-      <c r="B123" s="7" t="inlineStr">
+      <c r="B127" s="7" t="inlineStr">
         <is>
           <t>הקוד מוזג — דורש build ו-APK חדש</t>
         </is>
       </c>
-      <c r="C123" s="6" t="inlineStr"/>
-      <c r="D123" s="8" t="inlineStr"/>
-      <c r="E123" s="9" t="inlineStr"/>
-      <c r="F123" s="9" t="inlineStr"/>
-    </row>
-    <row r="124">
-      <c r="A124" s="6" t="inlineStr">
+      <c r="C127" s="6" t="inlineStr"/>
+      <c r="D127" s="8" t="inlineStr"/>
+      <c r="E127" s="9" t="inlineStr"/>
+      <c r="F127" s="9" t="inlineStr"/>
+    </row>
+    <row r="128">
+      <c r="A128" s="6" t="inlineStr">
         <is>
           <t>✅ Live (OTA)</t>
         </is>
       </c>
-      <c r="B124" s="7" t="inlineStr">
+      <c r="B128" s="7" t="inlineStr">
         <is>
           <t>שינוי JS — מועבר אוטומטית בהפעלה הבאה</t>
         </is>
       </c>
-      <c r="C124" s="6" t="inlineStr"/>
-      <c r="D124" s="8" t="inlineStr"/>
-      <c r="E124" s="9" t="inlineStr"/>
-      <c r="F124" s="9" t="inlineStr"/>
-    </row>
-    <row r="125">
-      <c r="A125" s="21" t="inlineStr">
+      <c r="C128" s="6" t="inlineStr"/>
+      <c r="D128" s="8" t="inlineStr"/>
+      <c r="E128" s="9" t="inlineStr"/>
+      <c r="F128" s="9" t="inlineStr"/>
+    </row>
+    <row r="129">
+      <c r="A129" s="21" t="inlineStr">
         <is>
           <t>⏳ ממתין ל-push</t>
         </is>
       </c>
-      <c r="B125" s="22" t="inlineStr">
+      <c r="B129" s="22" t="inlineStr">
         <is>
           <t>הקוד מוכן מקומית — טרם נדחף/נפרס</t>
         </is>
       </c>
     </row>
-    <row r="126">
-      <c r="A126" s="21" t="inlineStr">
+    <row r="130">
+      <c r="A130" s="21" t="inlineStr">
         <is>
           <t>⏳ דורש build</t>
         </is>
       </c>
-      <c r="B126" s="22" t="inlineStr">
+      <c r="B130" s="22" t="inlineStr">
         <is>
           <t>שינוי נייטיב — OTA לא מספיק, צריך AAB/APK חדש</t>
         </is>
       </c>
     </row>
-    <row r="128">
-      <c r="A128" s="23" t="inlineStr">
+    <row r="131"/>
+    <row r="132">
+      <c r="A132" s="23" t="inlineStr">
         <is>
           <t>סיכום Session 6-8</t>
-        </is>
-      </c>
-    </row>
-    <row r="129">
-      <c r="A129" s="24" t="n"/>
-      <c r="B129" s="25" t="inlineStr">
-        <is>
-          <t>58  —  פריטים חדשים שנוספו (52-109)</t>
-        </is>
-      </c>
-    </row>
-    <row r="130">
-      <c r="A130" s="24" t="n"/>
-      <c r="B130" s="25" t="inlineStr">
-        <is>
-          <t>56  —  חיים בייצור או ב-OTA</t>
-        </is>
-      </c>
-    </row>
-    <row r="131">
-      <c r="A131" s="24" t="n"/>
-      <c r="B131" s="25" t="inlineStr">
-        <is>
-          <t>0  —  ממתינים ל-push: הכל נפרס (commit 91ee6d3)</t>
-        </is>
-      </c>
-    </row>
-    <row r="132">
-      <c r="A132" s="24" t="n"/>
-      <c r="B132" s="25" t="inlineStr">
-        <is>
-          <t>2  —  פתוחים: פריסת טאבלט אמיתית (99) · הגשה ל-Play (19)</t>
         </is>
       </c>
     </row>
@@ -4387,7 +4505,7 @@
       <c r="A133" s="24" t="n"/>
       <c r="B133" s="25" t="inlineStr">
         <is>
-          <t>8  —  בורסות שאומתו חי (NYSE · TASE · XETRA · LSE) · JSE ביחידה בלבד</t>
+          <t>58  —  פריטים חדשים שנוספו (52-109)</t>
         </is>
       </c>
     </row>
@@ -4395,12 +4513,44 @@
       <c r="A134" s="24" t="n"/>
       <c r="B134" s="25" t="inlineStr">
         <is>
+          <t>56  —  חיים בייצור או ב-OTA</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" s="24" t="n"/>
+      <c r="B135" s="25" t="inlineStr">
+        <is>
+          <t>0  —  ממתינים ל-push: הכל נפרס (commit 91ee6d3)</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" s="24" t="n"/>
+      <c r="B136" s="25" t="inlineStr">
+        <is>
+          <t>2  —  פתוחים: פריסת טאבלט אמיתית (99) · הגשה ל-Play (19)</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" s="24" t="n"/>
+      <c r="B137" s="25" t="inlineStr">
+        <is>
+          <t>8  —  בורסות שאומתו חי (NYSE · TASE · XETRA · LSE) · JSE ביחידה בלבד</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" s="24" t="n"/>
+      <c r="B138" s="25" t="inlineStr">
+        <is>
           <t>48  —  חבילות בדיקה התנהגותיות עוברות (48/48)</t>
         </is>
       </c>
     </row>
-    <row r="135">
-      <c r="B135" t="inlineStr">
+    <row r="139">
+      <c r="B139" t="inlineStr">
         <is>
           <t>18  —  ראוטים בשרת · 324 מפתחות i18n × 4 שפות</t>
         </is>

</xml_diff>

<commit_message>
Metric detail header shows which stock the number belongs to
</commit_message>
<xml_diff>
--- a/BuddhaVest_Progress.xlsx
+++ b/BuddhaVest_Progress.xlsx
@@ -3880,22 +3880,22 @@
       </c>
     </row>
     <row r="107">
-      <c r="A107" s="39" t="inlineStr">
+      <c r="A107" s="48" t="inlineStr">
         <is>
           <t>98</t>
         </is>
       </c>
-      <c r="B107" s="40" t="inlineStr">
+      <c r="B107" s="49" t="inlineStr">
         <is>
           <t>מחוון "טוען" — הבאנר נראה תקוע</t>
         </is>
       </c>
-      <c r="C107" s="39" t="inlineStr">
+      <c r="C107" s="48" t="inlineStr">
         <is>
           <t>Frontend / UX</t>
         </is>
       </c>
-      <c r="D107" s="41" t="inlineStr">
+      <c r="D107" s="50" t="inlineStr">
         <is>
           <t>✅ Live (OTA)</t>
         </is>
@@ -3951,22 +3951,22 @@
       </c>
     </row>
     <row r="110">
-      <c r="A110" s="39" t="inlineStr">
+      <c r="A110" s="48" t="inlineStr">
         <is>
           <t>100</t>
         </is>
       </c>
-      <c r="B110" s="40" t="inlineStr">
+      <c r="B110" s="49" t="inlineStr">
         <is>
           <t>לונדון: מחיר גבוה פי 100</t>
         </is>
       </c>
-      <c r="C110" s="39" t="inlineStr">
+      <c r="C110" s="48" t="inlineStr">
         <is>
           <t>Backend / Bug Fix</t>
         </is>
       </c>
-      <c r="D110" s="41" t="inlineStr">
+      <c r="D110" s="50" t="inlineStr">
         <is>
           <t>✅ Live</t>
         </is>
@@ -3983,22 +3983,22 @@
       </c>
     </row>
     <row r="111">
-      <c r="A111" s="39" t="inlineStr">
+      <c r="A111" s="48" t="inlineStr">
         <is>
           <t>101</t>
         </is>
       </c>
-      <c r="B111" s="40" t="inlineStr">
+      <c r="B111" s="49" t="inlineStr">
         <is>
           <t>טבלת יחידות משנה במקום מקרה פרטי</t>
         </is>
       </c>
-      <c r="C111" s="39" t="inlineStr">
+      <c r="C111" s="48" t="inlineStr">
         <is>
           <t>Backend / Architecture</t>
         </is>
       </c>
-      <c r="D111" s="41" t="inlineStr">
+      <c r="D111" s="50" t="inlineStr">
         <is>
           <t>✅ Live</t>
         </is>
@@ -4015,22 +4015,22 @@
       </c>
     </row>
     <row r="112">
-      <c r="A112" s="39" t="inlineStr">
+      <c r="A112" s="48" t="inlineStr">
         <is>
           <t>102</t>
         </is>
       </c>
-      <c r="B112" s="40" t="inlineStr">
+      <c r="B112" s="49" t="inlineStr">
         <is>
           <t>חלוקה רק לשדות של מחיר למניה</t>
         </is>
       </c>
-      <c r="C112" s="39" t="inlineStr">
+      <c r="C112" s="48" t="inlineStr">
         <is>
           <t>Backend / Accuracy</t>
         </is>
       </c>
-      <c r="D112" s="41" t="inlineStr">
+      <c r="D112" s="50" t="inlineStr">
         <is>
           <t>✅ Live</t>
         </is>
@@ -4047,22 +4047,22 @@
       </c>
     </row>
     <row r="113">
-      <c r="A113" s="39" t="inlineStr">
+      <c r="A113" s="48" t="inlineStr">
         <is>
           <t>103</t>
         </is>
       </c>
-      <c r="B113" s="40" t="inlineStr">
+      <c r="B113" s="49" t="inlineStr">
         <is>
           <t>מכפילים שנגזרים ממחיר — דיכוי מורחב</t>
         </is>
       </c>
-      <c r="C113" s="39" t="inlineStr">
+      <c r="C113" s="48" t="inlineStr">
         <is>
           <t>Backend / Accuracy</t>
         </is>
       </c>
-      <c r="D113" s="41" t="inlineStr">
+      <c r="D113" s="50" t="inlineStr">
         <is>
           <t>✅ Live</t>
         </is>
@@ -4079,22 +4079,22 @@
       </c>
     </row>
     <row r="114">
-      <c r="A114" s="39" t="inlineStr">
+      <c r="A114" s="48" t="inlineStr">
         <is>
           <t>104</t>
         </is>
       </c>
-      <c r="B114" s="40" t="inlineStr">
+      <c r="B114" s="49" t="inlineStr">
         <is>
           <t>/quotes — אותו כלל כמו /analyze</t>
         </is>
       </c>
-      <c r="C114" s="39" t="inlineStr">
+      <c r="C114" s="48" t="inlineStr">
         <is>
           <t>Backend / Bug Fix</t>
         </is>
       </c>
-      <c r="D114" s="41" t="inlineStr">
+      <c r="D114" s="50" t="inlineStr">
         <is>
           <t>✅ Live</t>
         </is>
@@ -4111,22 +4111,22 @@
       </c>
     </row>
     <row r="115">
-      <c r="A115" s="39" t="inlineStr">
+      <c r="A115" s="48" t="inlineStr">
         <is>
           <t>105</t>
         </is>
       </c>
-      <c r="B115" s="40" t="inlineStr">
+      <c r="B115" s="49" t="inlineStr">
         <is>
           <t>סכום הדיבידנד עצמו</t>
         </is>
       </c>
-      <c r="C115" s="39" t="inlineStr">
+      <c r="C115" s="48" t="inlineStr">
         <is>
           <t>Backend / Bug Fix</t>
         </is>
       </c>
-      <c r="D115" s="41" t="inlineStr">
+      <c r="D115" s="50" t="inlineStr">
         <is>
           <t>✅ Live</t>
         </is>
@@ -4143,22 +4143,22 @@
       </c>
     </row>
     <row r="116">
-      <c r="A116" s="39" t="inlineStr">
+      <c r="A116" s="48" t="inlineStr">
         <is>
           <t>106</t>
         </is>
       </c>
-      <c r="B116" s="40" t="inlineStr">
+      <c r="B116" s="49" t="inlineStr">
         <is>
           <t>סימני מטבע — מקור אמת אחד</t>
         </is>
       </c>
-      <c r="C116" s="39" t="inlineStr">
+      <c r="C116" s="48" t="inlineStr">
         <is>
           <t>Frontend / Architecture</t>
         </is>
       </c>
-      <c r="D116" s="41" t="inlineStr">
+      <c r="D116" s="50" t="inlineStr">
         <is>
           <t>✅ Live (OTA)</t>
         </is>
@@ -4175,22 +4175,22 @@
       </c>
     </row>
     <row r="117">
-      <c r="A117" s="39" t="inlineStr">
+      <c r="A117" s="48" t="inlineStr">
         <is>
           <t>107</t>
         </is>
       </c>
-      <c r="B117" s="40" t="inlineStr">
+      <c r="B117" s="49" t="inlineStr">
         <is>
           <t>isUsd — השורה המשנית</t>
         </is>
       </c>
-      <c r="C117" s="39" t="inlineStr">
+      <c r="C117" s="48" t="inlineStr">
         <is>
           <t>Frontend / Bug Fix</t>
         </is>
       </c>
-      <c r="D117" s="41" t="inlineStr">
+      <c r="D117" s="50" t="inlineStr">
         <is>
           <t>✅ Live (OTA)</t>
         </is>
@@ -4207,22 +4207,22 @@
       </c>
     </row>
     <row r="118">
-      <c r="A118" s="39" t="inlineStr">
+      <c r="A118" s="48" t="inlineStr">
         <is>
           <t>108</t>
         </is>
       </c>
-      <c r="B118" s="40" t="inlineStr">
+      <c r="B118" s="49" t="inlineStr">
         <is>
           <t>אימות חוצה-בורסות</t>
         </is>
       </c>
-      <c r="C118" s="39" t="inlineStr">
+      <c r="C118" s="48" t="inlineStr">
         <is>
           <t>QA</t>
         </is>
       </c>
-      <c r="D118" s="41" t="inlineStr">
+      <c r="D118" s="50" t="inlineStr">
         <is>
           <t>✅ הושלם</t>
         </is>
@@ -4239,22 +4239,22 @@
       </c>
     </row>
     <row r="119">
-      <c r="A119" s="39" t="inlineStr">
+      <c r="A119" s="48" t="inlineStr">
         <is>
           <t>109</t>
         </is>
       </c>
-      <c r="B119" s="40" t="inlineStr">
+      <c r="B119" s="49" t="inlineStr">
         <is>
           <t>תיקון רתמת הבדיקות עצמה</t>
         </is>
       </c>
-      <c r="C119" s="39" t="inlineStr">
+      <c r="C119" s="48" t="inlineStr">
         <is>
           <t>QA</t>
         </is>
       </c>
-      <c r="D119" s="41" t="inlineStr">
+      <c r="D119" s="50" t="inlineStr">
         <is>
           <t>✅ הושלם</t>
         </is>
@@ -4303,34 +4303,34 @@
       </c>
     </row>
     <row r="121">
-      <c r="A121" s="48" t="inlineStr">
+      <c r="A121" s="44" t="inlineStr">
         <is>
           <t>111</t>
         </is>
       </c>
-      <c r="B121" s="49" t="inlineStr">
+      <c r="B121" s="45" t="inlineStr">
         <is>
           <t>טופס Data Safety מולא</t>
         </is>
       </c>
-      <c r="C121" s="48" t="inlineStr">
+      <c r="C121" s="44" t="inlineStr">
         <is>
           <t>Store / Legal</t>
         </is>
       </c>
-      <c r="D121" s="50" t="inlineStr">
-        <is>
-          <t>✅ הושלם</t>
-        </is>
-      </c>
-      <c r="E121" s="42" t="inlineStr">
+      <c r="D121" s="46" t="inlineStr">
+        <is>
+          <t>⏳ טיוטה — לא הוגש</t>
+        </is>
+      </c>
+      <c r="E121" s="47" t="inlineStr">
         <is>
           <t>data-safety-answers.html</t>
         </is>
       </c>
-      <c r="F121" s="42" t="inlineStr">
-        <is>
-          <t>5 סוגי נתונים הוצהרו: אינטראקציות באפליקציה · היסטוריית חיפוש · תוכן שנוצר על ידי משתמשים · גלישה באינטרנט · מזהה המכשיר. כולם נאספים, אף אחד לא משותף, אף אחד לא זמני, מטרה יחידה פונקציונליות. לא הוצהרו: מידע אישי, פיננסי, מיקום, בריאות, אנשי קשר, קראש-לוגים — כל אחד אומת מול המניפסט ומול 19 התלויות. יומן המחקר לא הוצהר כי buddhavest_journal אף פעם לא מופיע בתוך fetch.</t>
+      <c r="F121" s="47" t="inlineStr">
+        <is>
+          <t>התשובות מולאו ונשמרו כטיוטה, אבל הטופס מעולם לא הוגש — לוח הבקרה של Play מציג עיגול ריק ליד "אבטחת נתונים". אומת ישירות בקונסולה: הטופס נפתח בשלב 1 מתוך 5 עם כפתור "שמירת טיוטה" פעיל, והתשובות של שלב 2 (כן לאיסוף, כן להצפנה) שמורות. צריך לעבור שלבים 3-4-5 וללחוץ שליחה במסך התצוגה המקדימה. 5 סוגי נתונים שהוצהרו: אינטראקציות · חיפוש · תוכן משתמש · גלישה · מזהה מכשיר.</t>
         </is>
       </c>
     </row>
@@ -4493,7 +4493,6 @@
         </is>
       </c>
     </row>
-    <row r="131"/>
     <row r="132">
       <c r="A132" s="23" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Share count from statements per date - same bug existed twice; every empty chart now reports why
</commit_message>
<xml_diff>
--- a/BuddhaVest_Progress.xlsx
+++ b/BuddhaVest_Progress.xlsx
@@ -187,7 +187,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="51">
+  <cellXfs count="54">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -323,6 +323,15 @@
       <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
@@ -690,7 +699,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F139"/>
+  <dimension ref="A1:F145"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -4271,285 +4280,478 @@
       </c>
     </row>
     <row r="120">
-      <c r="A120" s="44" t="inlineStr">
+      <c r="A120" s="51" t="inlineStr">
+        <is>
+          <t>114</t>
+        </is>
+      </c>
+      <c r="B120" s="52" t="inlineStr">
+        <is>
+          <t>AMD: אפס גרפים בכל המכפילים</t>
+        </is>
+      </c>
+      <c r="C120" s="51" t="inlineStr">
+        <is>
+          <t>Backend / Bug Fix</t>
+        </is>
+      </c>
+      <c r="D120" s="53" t="inlineStr">
+        <is>
+          <t>⏳ ממתין ל-push</t>
+        </is>
+      </c>
+      <c r="E120" s="47" t="inlineStr">
+        <is>
+          <t>main.py</t>
+        </is>
+      </c>
+      <c r="F120" s="47" t="inlineStr">
+        <is>
+          <t>החישוב ההיסטורי קרא את מספר המניות רק מ-info["sharesOutstanding"], ויאהו לא מחזירה את השדה הזה ל-AMD. שורה אחת — if not shares — הפילה את כל הענף, וכל המכפילים חזרו ריקים: P/B, P/S, EV/EBITDA ו-Forward P/E. אומת חי: /metric-history/AMD/price_to_book ו-/ev_to_ebitda שניהם quarterly:[] בעוד WMT מחזירה 43 נקודות. הנתונים היו קיימים כל הזמן — /financials/AMD מכיל Ordinary Shares Number 1,630,410,843 בכל דוח.</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="51" t="inlineStr">
+        <is>
+          <t>115</t>
+        </is>
+      </c>
+      <c r="B121" s="52" t="inlineStr">
+        <is>
+          <t>אותו באג במקום שני: רכישות חוזרות</t>
+        </is>
+      </c>
+      <c r="C121" s="51" t="inlineStr">
+        <is>
+          <t>Backend / Bug Fix</t>
+        </is>
+      </c>
+      <c r="D121" s="53" t="inlineStr">
+        <is>
+          <t>⏳ ממתין ל-push</t>
+        </is>
+      </c>
+      <c r="E121" s="47" t="inlineStr">
+        <is>
+          <t>main.py</t>
+        </is>
+      </c>
+      <c r="F121" s="47" t="inlineStr">
+        <is>
+          <t>ענף ה-buyback הכיל עותק שני של אותה שורה, כך שגם תשואת הרכישות החוזרות של AMD היתה ריקה. נמצא רק בגלל החיפוש היזום אחרי מופעים נוספים, לא מדיווח משתמש.</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="51" t="inlineStr">
+        <is>
+          <t>116</t>
+        </is>
+      </c>
+      <c r="B122" s="52" t="inlineStr">
+        <is>
+          <t>מקור אחד לספירת מניות</t>
+        </is>
+      </c>
+      <c r="C122" s="51" t="inlineStr">
+        <is>
+          <t>Backend / Architecture</t>
+        </is>
+      </c>
+      <c r="D122" s="53" t="inlineStr">
+        <is>
+          <t>⏳ ממתין ל-push</t>
+        </is>
+      </c>
+      <c r="E122" s="47" t="inlineStr">
+        <is>
+          <t>main.py</t>
+        </is>
+      </c>
+      <c r="F122" s="47" t="inlineStr">
+        <is>
+          <t>_shares_lookup ברמת המודול מחליף את שני העותקים: Ordinary Shares Number ← Share Issued ← Diluted Average Shares ← Basic Average Shares ← השדה ב-info. שני הענפים קוראים לאותה פונקציה, כך שהם לא יכולים להתפצל שוב. 18 בדיקות יחידה.</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="51" t="inlineStr">
+        <is>
+          <t>117</t>
+        </is>
+      </c>
+      <c r="B123" s="52" t="inlineStr">
+        <is>
+          <t>ספירת מניות לפי תאריך</t>
+        </is>
+      </c>
+      <c r="C123" s="51" t="inlineStr">
+        <is>
+          <t>Backend / Accuracy</t>
+        </is>
+      </c>
+      <c r="D123" s="53" t="inlineStr">
+        <is>
+          <t>⏳ ממתין ל-push</t>
+        </is>
+      </c>
+      <c r="E123" s="47" t="inlineStr">
+        <is>
+          <t>main.py</t>
+        </is>
+      </c>
+      <c r="F123" s="47" t="inlineStr">
+        <is>
+          <t>שיפור שנחשף תוך כדי: הקוד לקח ספירה נוכחית אחת והחיל אותה על חמש שנות מחירים. לכל חברה שרוכשת מניות בחזרה זה מעוות כל נקודת עבר. AMD: 1,616M ב-2023 מול 1,630M ב-2026. עכשיו כל נקודה מקבלת את הספירה שהיתה בתוקף באותו תאריך.</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="51" t="inlineStr">
+        <is>
+          <t>118</t>
+        </is>
+      </c>
+      <c r="B124" s="52" t="inlineStr">
+        <is>
+          <t>כשל שקט הופך לכשל מדווח</t>
+        </is>
+      </c>
+      <c r="C124" s="51" t="inlineStr">
+        <is>
+          <t>Backend / Observability</t>
+        </is>
+      </c>
+      <c r="D124" s="53" t="inlineStr">
+        <is>
+          <t>⏳ ממתין ל-push</t>
+        </is>
+      </c>
+      <c r="E124" s="47" t="inlineStr">
+        <is>
+          <t>main.py</t>
+        </is>
+      </c>
+      <c r="F124" s="47" t="inlineStr">
+        <is>
+          <t>כל 14 המקומות שמחזירים use_price מדווחים עכשיו empty_reason: no_share_count · no_price_history · no_repurchase_rows · no_eps_series · no_dividend_history · all_points_rejected · no_statement_rows · metric_not_tracked · exception. הבעיה המקורית היתה בלתי נראית כי האריח הראה ערך (מיאהו) בזמן שהגרף היה ריק — מסך ריק עם אריח מלא נראה כמו חוסר נתונים ולא כמו באג.</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="51" t="inlineStr">
+        <is>
+          <t>119</t>
+        </is>
+      </c>
+      <c r="B125" s="52" t="inlineStr">
+        <is>
+          <t>שם המניה במסך המדד</t>
+        </is>
+      </c>
+      <c r="C125" s="51" t="inlineStr">
+        <is>
+          <t>Frontend / UX</t>
+        </is>
+      </c>
+      <c r="D125" s="53" t="inlineStr">
+        <is>
+          <t>⏳ ממתין ל-push</t>
+        </is>
+      </c>
+      <c r="E125" s="47" t="inlineStr">
+        <is>
+          <t>MetricHistoryScreen.js, StockScreen.js, ETFCard.js</t>
+        </is>
+      </c>
+      <c r="F125" s="47" t="inlineStr">
+        <is>
+          <t>המסך הציג "EV/EBITDA · 103.36" בלי שום אינדיקציה לאיזו חברה המספר שייך. השם מופיע עכשיו מעל שם המדד. עודכנו כל 10 נקודות הכניסה — תשע מ-StockScreen ואחת מ-ETFCard.</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="44" t="inlineStr">
         <is>
           <t>110</t>
         </is>
       </c>
-      <c r="B120" s="45" t="inlineStr">
+      <c r="B126" s="45" t="inlineStr">
         <is>
           <t>עמוד הפרטיות הוגש מהמטמון</t>
         </is>
       </c>
-      <c r="C120" s="44" t="inlineStr">
+      <c r="C126" s="44" t="inlineStr">
         <is>
           <t>Backend / Legal / Bug Fix</t>
         </is>
       </c>
-      <c r="D120" s="46" t="inlineStr">
+      <c r="D126" s="46" t="inlineStr">
         <is>
           <t>⏳ ממתין ל-push</t>
         </is>
       </c>
-      <c r="E120" s="47" t="inlineStr">
+      <c r="E126" s="47" t="inlineStr">
         <is>
           <t>main.py</t>
         </is>
       </c>
-      <c r="F120" s="47" t="inlineStr">
+      <c r="F126" s="47" t="inlineStr">
         <is>
           <t>המידלוור שמונע מטמון החריג במפורש את /privacy, מתוך הנחה שדף משפטי סטטי כדאי לשמור. ההנחה היתה הפוכה. אומת חי: הכתובת הרגילה החזירה את הנוסח הישן ("the watchlist is never transmitted to our servers") בעוד שאותה כתובת עם פרמטר שאילתה חדש החזירה את המתוקן — כלומר הקוד תקין והתשובה נתקעה במטמון. גוגל משווה את הדף להצהרת Data Safety, כך שעותק ישן היה יוצר סתירה מולם. החריג הוסר; כל נתיב מקבל no-store.</t>
         </is>
       </c>
     </row>
-    <row r="121">
-      <c r="A121" s="44" t="inlineStr">
+    <row r="127">
+      <c r="A127" s="44" t="inlineStr">
         <is>
           <t>111</t>
         </is>
       </c>
-      <c r="B121" s="45" t="inlineStr">
+      <c r="B127" s="45" t="inlineStr">
         <is>
           <t>טופס Data Safety מולא</t>
         </is>
       </c>
-      <c r="C121" s="44" t="inlineStr">
+      <c r="C127" s="44" t="inlineStr">
         <is>
           <t>Store / Legal</t>
         </is>
       </c>
-      <c r="D121" s="46" t="inlineStr">
+      <c r="D127" s="46" t="inlineStr">
         <is>
           <t>⏳ טיוטה — לא הוגש</t>
         </is>
       </c>
-      <c r="E121" s="47" t="inlineStr">
+      <c r="E127" s="47" t="inlineStr">
         <is>
           <t>data-safety-answers.html</t>
         </is>
       </c>
-      <c r="F121" s="47" t="inlineStr">
+      <c r="F127" s="47" t="inlineStr">
         <is>
           <t>התשובות מולאו ונשמרו כטיוטה, אבל הטופס מעולם לא הוגש — לוח הבקרה של Play מציג עיגול ריק ליד "אבטחת נתונים". אומת ישירות בקונסולה: הטופס נפתח בשלב 1 מתוך 5 עם כפתור "שמירת טיוטה" פעיל, והתשובות של שלב 2 (כן לאיסוף, כן להצפנה) שמורות. צריך לעבור שלבים 3-4-5 וללחוץ שליחה במסך התצוגה המקדימה. 5 סוגי נתונים שהוצהרו: אינטראקציות · חיפוש · תוכן משתמש · גלישה · מזהה מכשיר.</t>
         </is>
       </c>
     </row>
-    <row r="122">
-      <c r="A122" s="48" t="inlineStr">
+    <row r="128">
+      <c r="A128" s="48" t="inlineStr">
         <is>
           <t>112</t>
         </is>
       </c>
-      <c r="B122" s="49" t="inlineStr">
+      <c r="B128" s="49" t="inlineStr">
         <is>
           <t>צ׳קליסט טפסי Play Console</t>
         </is>
       </c>
-      <c r="C122" s="48" t="inlineStr">
+      <c r="C128" s="48" t="inlineStr">
         <is>
           <t>Store</t>
         </is>
       </c>
-      <c r="D122" s="50" t="inlineStr">
+      <c r="D128" s="50" t="inlineStr">
         <is>
           <t>✅ הושלם</t>
         </is>
       </c>
-      <c r="E122" s="42" t="inlineStr">
+      <c r="E128" s="42" t="inlineStr">
         <is>
           <t>play-console-checklist.html</t>
         </is>
       </c>
-      <c r="F122" s="42" t="inlineStr">
+      <c r="F128" s="42" t="inlineStr">
         <is>
           <t>תשובות לכל סעיפי App content שנותרו: גישה לאפליקציה, מודעות, דירוג תוכן, קהל יעד, תכונות פיננסיות, אפליקציית חדשות, בריאות, ממשלה, הרשאות רגישות. שתי ההצהרות הרגישות באפליקציה מסוג זה — "תכונות פיננסיות" ו"אפליקציית חדשות" — מנומקות בנפרד.</t>
         </is>
       </c>
     </row>
-    <row r="123">
-      <c r="A123" s="44" t="inlineStr">
+    <row r="129">
+      <c r="A129" s="44" t="inlineStr">
         <is>
           <t>113</t>
         </is>
       </c>
-      <c r="B123" s="45" t="inlineStr">
+      <c r="B129" s="45" t="inlineStr">
         <is>
           <t>צילומי מסך לחנות</t>
         </is>
       </c>
-      <c r="C123" s="44" t="inlineStr">
+      <c r="C129" s="44" t="inlineStr">
         <is>
           <t>Store</t>
         </is>
       </c>
-      <c r="D123" s="46" t="inlineStr">
+      <c r="D129" s="46" t="inlineStr">
         <is>
           <t>🔜 לא התחיל</t>
         </is>
       </c>
-      <c r="E123" s="47" t="inlineStr">
+      <c r="E129" s="47" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="F123" s="47" t="inlineStr">
+      <c r="F129" s="47" t="inlineStr">
         <is>
           <t>הפער היחיד שנותר בדף החנות. גוגל דורשת לפחות 2 צילומי טלפון, מומלץ 4-8. אייקון ו-feature graphic כבר קיימים במידות הנכונות (1024x1024 ו-1024x500). מדריך מוכן ב-מדריך-צילומי-מסך-לחנות.html.</t>
         </is>
       </c>
     </row>
-    <row r="124">
-      <c r="A124" s="10" t="inlineStr">
+    <row r="130">
+      <c r="A130" s="10" t="inlineStr">
         <is>
           <t>Legend</t>
         </is>
       </c>
     </row>
-    <row r="125">
-      <c r="A125" s="6" t="inlineStr">
+    <row r="131">
+      <c r="A131" s="6" t="inlineStr">
         <is>
           <t>✅ Live</t>
         </is>
       </c>
-      <c r="B125" s="7" t="inlineStr">
+      <c r="B131" s="7" t="inlineStr">
         <is>
           <t>פרוס ופעיל ב-Render — נראה לכל המשתמשים</t>
         </is>
       </c>
-      <c r="C125" s="6" t="inlineStr"/>
-      <c r="D125" s="8" t="inlineStr"/>
-      <c r="E125" s="9" t="inlineStr"/>
-      <c r="F125" s="9" t="inlineStr"/>
-    </row>
-    <row r="126">
-      <c r="A126" s="6" t="inlineStr">
+      <c r="C131" s="6" t="inlineStr"/>
+      <c r="D131" s="8" t="inlineStr"/>
+      <c r="E131" s="9" t="inlineStr"/>
+      <c r="F131" s="9" t="inlineStr"/>
+    </row>
+    <row r="132">
+      <c r="A132" s="6" t="inlineStr">
         <is>
           <t>✅ In APK</t>
         </is>
       </c>
-      <c r="B126" s="7" t="inlineStr">
+      <c r="B132" s="7" t="inlineStr">
         <is>
           <t>כלול ב-APK המותקן — נראה לכל המשתמשים</t>
         </is>
       </c>
-      <c r="C126" s="6" t="inlineStr"/>
-      <c r="D126" s="8" t="inlineStr"/>
-      <c r="E126" s="9" t="inlineStr"/>
-      <c r="F126" s="9" t="inlineStr"/>
-    </row>
-    <row r="127">
-      <c r="A127" s="6" t="inlineStr">
+      <c r="C132" s="6" t="inlineStr"/>
+      <c r="D132" s="8" t="inlineStr"/>
+      <c r="E132" s="9" t="inlineStr"/>
+      <c r="F132" s="9" t="inlineStr"/>
+    </row>
+    <row r="133">
+      <c r="A133" s="6" t="inlineStr">
         <is>
           <t>⏳ Next APK</t>
         </is>
       </c>
-      <c r="B127" s="7" t="inlineStr">
+      <c r="B133" s="7" t="inlineStr">
         <is>
           <t>הקוד מוזג — דורש build ו-APK חדש</t>
         </is>
       </c>
-      <c r="C127" s="6" t="inlineStr"/>
-      <c r="D127" s="8" t="inlineStr"/>
-      <c r="E127" s="9" t="inlineStr"/>
-      <c r="F127" s="9" t="inlineStr"/>
-    </row>
-    <row r="128">
-      <c r="A128" s="6" t="inlineStr">
+      <c r="C133" s="6" t="inlineStr"/>
+      <c r="D133" s="8" t="inlineStr"/>
+      <c r="E133" s="9" t="inlineStr"/>
+      <c r="F133" s="9" t="inlineStr"/>
+    </row>
+    <row r="134">
+      <c r="A134" s="6" t="inlineStr">
         <is>
           <t>✅ Live (OTA)</t>
         </is>
       </c>
-      <c r="B128" s="7" t="inlineStr">
+      <c r="B134" s="7" t="inlineStr">
         <is>
           <t>שינוי JS — מועבר אוטומטית בהפעלה הבאה</t>
         </is>
       </c>
-      <c r="C128" s="6" t="inlineStr"/>
-      <c r="D128" s="8" t="inlineStr"/>
-      <c r="E128" s="9" t="inlineStr"/>
-      <c r="F128" s="9" t="inlineStr"/>
-    </row>
-    <row r="129">
-      <c r="A129" s="21" t="inlineStr">
+      <c r="C134" s="6" t="inlineStr"/>
+      <c r="D134" s="8" t="inlineStr"/>
+      <c r="E134" s="9" t="inlineStr"/>
+      <c r="F134" s="9" t="inlineStr"/>
+    </row>
+    <row r="135">
+      <c r="A135" s="21" t="inlineStr">
         <is>
           <t>⏳ ממתין ל-push</t>
         </is>
       </c>
-      <c r="B129" s="22" t="inlineStr">
+      <c r="B135" s="22" t="inlineStr">
         <is>
           <t>הקוד מוכן מקומית — טרם נדחף/נפרס</t>
         </is>
       </c>
     </row>
-    <row r="130">
-      <c r="A130" s="21" t="inlineStr">
+    <row r="136">
+      <c r="A136" s="21" t="inlineStr">
         <is>
           <t>⏳ דורש build</t>
         </is>
       </c>
-      <c r="B130" s="22" t="inlineStr">
+      <c r="B136" s="22" t="inlineStr">
         <is>
           <t>שינוי נייטיב — OTA לא מספיק, צריך AAB/APK חדש</t>
         </is>
       </c>
     </row>
-    <row r="132">
-      <c r="A132" s="23" t="inlineStr">
+    <row r="137"/>
+    <row r="138">
+      <c r="A138" s="23" t="inlineStr">
         <is>
           <t>סיכום Session 6-8</t>
         </is>
       </c>
     </row>
-    <row r="133">
-      <c r="A133" s="24" t="n"/>
-      <c r="B133" s="25" t="inlineStr">
+    <row r="139">
+      <c r="A139" s="24" t="n"/>
+      <c r="B139" s="25" t="inlineStr">
         <is>
           <t>58  —  פריטים חדשים שנוספו (52-109)</t>
         </is>
       </c>
     </row>
-    <row r="134">
-      <c r="A134" s="24" t="n"/>
-      <c r="B134" s="25" t="inlineStr">
+    <row r="140">
+      <c r="A140" s="24" t="n"/>
+      <c r="B140" s="25" t="inlineStr">
         <is>
           <t>56  —  חיים בייצור או ב-OTA</t>
         </is>
       </c>
     </row>
-    <row r="135">
-      <c r="A135" s="24" t="n"/>
-      <c r="B135" s="25" t="inlineStr">
+    <row r="141">
+      <c r="A141" s="24" t="n"/>
+      <c r="B141" s="25" t="inlineStr">
         <is>
           <t>0  —  ממתינים ל-push: הכל נפרס (commit 91ee6d3)</t>
         </is>
       </c>
     </row>
-    <row r="136">
-      <c r="A136" s="24" t="n"/>
-      <c r="B136" s="25" t="inlineStr">
+    <row r="142">
+      <c r="A142" s="24" t="n"/>
+      <c r="B142" s="25" t="inlineStr">
         <is>
           <t>2  —  פתוחים: פריסת טאבלט אמיתית (99) · הגשה ל-Play (19)</t>
         </is>
       </c>
     </row>
-    <row r="137">
-      <c r="A137" s="24" t="n"/>
-      <c r="B137" s="25" t="inlineStr">
+    <row r="143">
+      <c r="A143" s="24" t="n"/>
+      <c r="B143" s="25" t="inlineStr">
         <is>
           <t>8  —  בורסות שאומתו חי (NYSE · TASE · XETRA · LSE) · JSE ביחידה בלבד</t>
         </is>
       </c>
     </row>
-    <row r="138">
-      <c r="A138" s="24" t="n"/>
-      <c r="B138" s="25" t="inlineStr">
+    <row r="144">
+      <c r="A144" s="24" t="n"/>
+      <c r="B144" s="25" t="inlineStr">
         <is>
           <t>48  —  חבילות בדיקה התנהגותיות עוברות (48/48)</t>
         </is>
       </c>
     </row>
-    <row r="139">
-      <c r="B139" t="inlineStr">
+    <row r="145">
+      <c r="B145" t="inlineStr">
         <is>
           <t>18  —  ראוטים בשרת · 324 מפתחות i18n × 4 שפות</t>
         </is>

</xml_diff>